<commit_message>
[ Version 0.0.21.4 ] - drainage vent electronics tasks was done.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="105">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -122,6 +122,9 @@
     <t xml:space="preserve">DO for power mosfet 1. (Vent servo power mosfet 1)</t>
   </si>
   <si>
+    <t xml:space="preserve">V1</t>
+  </si>
+  <si>
     <t xml:space="preserve">OUT_VSPM2_PIN</t>
   </si>
   <si>
@@ -129,6 +132,9 @@
   </si>
   <si>
     <t xml:space="preserve">DO for power mosfet 2. (Vent servo power mosfet 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V2</t>
   </si>
   <si>
     <t xml:space="preserve">IN_ESO1_PIN</t>
@@ -339,7 +345,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -388,12 +394,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="16">
@@ -529,7 +529,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -538,7 +538,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -551,10 +551,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -594,19 +590,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1091,27 +1083,27 @@
       <c r="U1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
-      <c r="U2" s="6"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -1139,29 +1131,29 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="7"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -1188,14 +1180,14 @@
       <c r="N5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
       <c r="E6" s="5" t="s">
         <v>19</v>
       </c>
@@ -1212,14 +1204,14 @@
       <c r="N6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
       <c r="E7" s="5" t="s">
         <v>22</v>
       </c>
@@ -1236,14 +1228,14 @@
       <c r="N7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
       <c r="E8" s="5" t="s">
         <v>25</v>
       </c>
@@ -1260,14 +1252,14 @@
       <c r="N8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+      <c r="A9" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
       <c r="E9" s="5" t="s">
         <v>28</v>
       </c>
@@ -1284,14 +1276,14 @@
       <c r="N9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+      <c r="A10" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
       <c r="E10" s="5" t="s">
         <v>31</v>
       </c>
@@ -1306,22 +1298,25 @@
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
+      <c r="O10" s="0" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
+      <c r="A11" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
+      <c r="B11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
       <c r="E11" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F11" s="5"/>
       <c r="G11" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
@@ -1330,22 +1325,25 @@
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
+      <c r="O11" s="0" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+      <c r="A12" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
+      <c r="B12" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
       <c r="E12" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F12" s="5"/>
       <c r="G12" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
@@ -1354,22 +1352,25 @@
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
       <c r="N12" s="5"/>
+      <c r="O12" s="0" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="A13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
+      <c r="B13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
@@ -1378,22 +1379,25 @@
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
+      <c r="O13" s="0" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+      <c r="A14" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
+      <c r="B14" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
       <c r="E14" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
@@ -1402,22 +1406,25 @@
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
+      <c r="O14" s="0" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
+      <c r="B15" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
       <c r="E15" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
@@ -1426,6 +1433,9 @@
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
+      <c r="O15" s="0" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -1451,29 +1461,29 @@
       <c r="U16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
-      <c r="T17" s="7"/>
-      <c r="U17" s="7"/>
+      <c r="A17" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6"/>
+      <c r="T17" s="6"/>
+      <c r="U17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
@@ -1500,20 +1510,20 @@
       <c r="N18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="n">
+      <c r="A19" s="7" t="n">
         <v>1</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
@@ -1547,29 +1557,29 @@
       <c r="U20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
-      <c r="S21" s="7"/>
-      <c r="T21" s="7"/>
-      <c r="U21" s="7"/>
+      <c r="A21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
@@ -1596,20 +1606,20 @@
       <c r="N22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="7" t="n">
         <v>1</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F23" s="5"/>
       <c r="G23" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
@@ -1643,61 +1653,61 @@
       <c r="U24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="15"/>
-      <c r="S25" s="15"/>
-      <c r="T25" s="15"/>
-      <c r="U25" s="15"/>
+      <c r="A25" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14"/>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14"/>
+      <c r="O25" s="14"/>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="14"/>
+      <c r="R25" s="14"/>
+      <c r="S25" s="14"/>
+      <c r="T25" s="14"/>
+      <c r="U25" s="14"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="7"/>
-      <c r="S26" s="7"/>
-      <c r="T26" s="7"/>
-      <c r="U26" s="7"/>
+      <c r="A26" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
+      <c r="U26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -1707,7 +1717,7 @@
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1723,30 +1733,30 @@
       <c r="R27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="n">
+      <c r="A28" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B28" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>60</v>
+      <c r="B28" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>62</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
@@ -1757,20 +1767,20 @@
       <c r="R28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="n">
+      <c r="A29" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B29" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>64</v>
+      <c r="B29" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
@@ -1778,7 +1788,7 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -1789,20 +1799,20 @@
       <c r="R29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="n">
+      <c r="A30" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B30" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C30" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>67</v>
+      <c r="B30" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -1810,7 +1820,7 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
@@ -1821,20 +1831,20 @@
       <c r="R30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="n">
+      <c r="A31" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B31" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C31" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D31" s="16" t="s">
-        <v>67</v>
+      <c r="B31" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
@@ -1842,7 +1852,7 @@
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
@@ -1853,20 +1863,20 @@
       <c r="R31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="n">
+      <c r="A32" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B32" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D32" s="16" t="s">
-        <v>67</v>
+      <c r="B32" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
@@ -1874,7 +1884,7 @@
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
       <c r="K32" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
@@ -1885,30 +1895,30 @@
       <c r="R32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="n">
+      <c r="A33" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B33" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>74</v>
+      <c r="B33" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
       <c r="K33" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
@@ -1919,30 +1929,30 @@
       <c r="R33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="n">
+      <c r="A34" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B34" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="D34" s="16" t="s">
-        <v>78</v>
+      <c r="B34" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
       <c r="K34" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="L34" s="5"/>
       <c r="M34" s="5"/>
@@ -1953,30 +1963,30 @@
       <c r="R34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="n">
+      <c r="A35" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B35" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C35" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="D35" s="16" t="s">
-        <v>67</v>
+      <c r="B35" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
@@ -2010,29 +2020,29 @@
       <c r="U36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="7"/>
-      <c r="R37" s="7"/>
-      <c r="S37" s="7"/>
-      <c r="T37" s="7"/>
-      <c r="U37" s="7"/>
+      <c r="A37" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B37" s="6"/>
+      <c r="C37" s="6"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="6"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="6"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6"/>
+      <c r="R37" s="6"/>
+      <c r="S37" s="6"/>
+      <c r="T37" s="6"/>
+      <c r="U37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
@@ -2044,7 +2054,7 @@
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -2060,25 +2070,25 @@
       <c r="O38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="n">
+      <c r="A39" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B39" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="D39" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E39" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
+      <c r="B39" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F39" s="5"/>
+      <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
@@ -2089,25 +2099,25 @@
       <c r="O39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="8" t="n">
+      <c r="A40" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B40" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="C40" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="D40" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="E40" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
+      <c r="B40" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
@@ -2141,142 +2151,142 @@
       <c r="U41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7"/>
-      <c r="H42" s="7"/>
-      <c r="I42" s="7"/>
-      <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
-      <c r="L42" s="7"/>
-      <c r="M42" s="7"/>
-      <c r="N42" s="7"/>
-      <c r="O42" s="7"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="7"/>
-      <c r="R42" s="7"/>
-      <c r="S42" s="7"/>
-      <c r="T42" s="7"/>
-      <c r="U42" s="7"/>
+      <c r="A42" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" s="6"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6"/>
+      <c r="K42" s="6"/>
+      <c r="L42" s="6"/>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="6"/>
+      <c r="P42" s="6"/>
+      <c r="Q42" s="6"/>
+      <c r="R42" s="6"/>
+      <c r="S42" s="6"/>
+      <c r="T42" s="6"/>
+      <c r="U42" s="6"/>
     </row>
     <row r="43" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>4</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="H43" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
+      <c r="H43" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="8" t="n">
+      <c r="A44" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="18"/>
-      <c r="C44" s="8"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="7"/>
       <c r="D44" s="5" t="s">
         <v>22</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
-      <c r="H44" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="I44" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="J44" s="8" t="s">
+      <c r="H44" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="K44" s="8" t="s">
+      <c r="I44" s="7" t="s">
         <v>97</v>
       </c>
+      <c r="J44" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="K44" s="7" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="8" t="n">
+      <c r="A45" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B45" s="18"/>
-      <c r="C45" s="18"/>
+      <c r="B45" s="15"/>
+      <c r="C45" s="15"/>
       <c r="D45" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
-      <c r="H45" s="8" t="s">
+      <c r="H45" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="I45" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="J45" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="K45" s="8" t="s">
+      <c r="I45" s="7" t="s">
         <v>100</v>
       </c>
+      <c r="J45" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K45" s="7" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="8" t="n">
+      <c r="A46" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B46" s="19"/>
-      <c r="C46" s="8"/>
+      <c r="B46" s="16"/>
+      <c r="C46" s="7"/>
       <c r="D46" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="6"/>
-      <c r="K46" s="6"/>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="8" t="n">
+      <c r="A47" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="18"/>
       <c r="D47" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
-      <c r="H47" s="6"/>
+      <c r="H47" s="17"/>
       <c r="I47" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J47" s="5"/>
-      <c r="K47" s="6"/>
+      <c r="K47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8" t="n">
+      <c r="A48" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="8"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="7"/>
       <c r="D48" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
@@ -2284,37 +2294,37 @@
       <c r="J48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="8" t="n">
+      <c r="A49" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B49" s="19"/>
-      <c r="C49" s="19"/>
+      <c r="B49" s="16"/>
+      <c r="C49" s="16"/>
       <c r="D49" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="8" t="n">
+      <c r="A50" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="21"/>
-      <c r="C50" s="8"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="7"/>
       <c r="D50" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="8" t="n">
+      <c r="A51" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B51" s="21"/>
-      <c r="C51" s="21"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
       <c r="D51" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>

</xml_diff>

<commit_message>
[ Version 0.0.24.5 ] - drainage vent GPIOs was updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -77,124 +77,118 @@
     <t xml:space="preserve">PIN</t>
   </si>
   <si>
-    <t xml:space="preserve">5V_PIN</t>
+    <t xml:space="preserve">SECTION</t>
   </si>
   <si>
     <t xml:space="preserve">5V</t>
   </si>
   <si>
-    <t xml:space="preserve">Power 5V for ESP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3V_PIN</t>
+    <t xml:space="preserve">Power 5V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3V</t>
   </si>
   <si>
     <t xml:space="preserve">3.3V</t>
   </si>
   <si>
-    <t xml:space="preserve">Power 3.3V for end switches.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GND_PIN</t>
+    <t xml:space="preserve">Power 3.3V.</t>
   </si>
   <si>
     <t xml:space="preserve">GND</t>
   </si>
   <si>
-    <t xml:space="preserve">Power GND for ESP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_PWM_PIN</t>
+    <t xml:space="preserve">GND.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_PWM</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO13</t>
   </si>
   <si>
-    <t xml:space="preserve">PWM output for vent servos. Allways on.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_VSPM1_PIN</t>
+    <t xml:space="preserve">PWM output for drainage vent servos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_SPM1</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO32</t>
   </si>
   <si>
-    <t xml:space="preserve">DO for power mosfet 1. (Vent servo power mosfet 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_VSPM2_PIN</t>
+    <t xml:space="preserve">DO for drainage vent power mosfet V1 – servo power mosfet 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_SPM2</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO33</t>
   </si>
   <si>
-    <t xml:space="preserve">DO for power mosfet 2. (Vent servo power mosfet 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ESO1_PIN</t>
+    <t xml:space="preserve">DO for drainage vent power mosfet V2 - servo power mosfet 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESO1</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO35</t>
   </si>
   <si>
-    <t xml:space="preserve">DI (only) pin for end sensor switch. (End switch open 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ESO2_PIN</t>
+    <t xml:space="preserve">DI (only) for drainage vent V1 open position end switch - end switch open 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESO2</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO36</t>
   </si>
   <si>
-    <t xml:space="preserve">DI (only) pin for end sensor switch. (End switch open 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ESC1_PIN</t>
+    <t xml:space="preserve">DI (only) for drainage vent V2 open position end switch - end switch open 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESC1</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO34</t>
   </si>
   <si>
-    <t xml:space="preserve">DI (only) pin for end sensor switch. (End switch close 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ESC2_PIN</t>
+    <t xml:space="preserve">DI (only) for drainage vent V1 close position end switch - end switch close 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESC2</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO39</t>
   </si>
   <si>
-    <t xml:space="preserve">DI (only) pin for end sensor switch. (End switch close 2)</t>
+    <t xml:space="preserve">DI (only) for drainage vent V2 close position end switch - end switch close 2.</t>
   </si>
   <si>
     <t xml:space="preserve">ESP-IDF TIMERS</t>
   </si>
   <si>
-    <t xml:space="preserve">TIMER_0</t>
+    <t xml:space="preserve">SYS_DRAIN_VENT_PWM_TIME</t>
   </si>
   <si>
     <t xml:space="preserve">LEDC_TIMER_0</t>
   </si>
   <si>
-    <t xml:space="preserve">Vent servo PWM timer. Hardcoded.</t>
+    <t xml:space="preserve">Drainage vent servo PWM timer.</t>
   </si>
   <si>
     <t xml:space="preserve">ESP-IDF CHANNELS</t>
   </si>
   <si>
-    <t xml:space="preserve">OUT_VSPWM_CHANNEL</t>
+    <t xml:space="preserve">SYS_DRAIN_VENT_PWM_CHNL</t>
   </si>
   <si>
     <t xml:space="preserve">LEDC_CHANNEL_0</t>
   </si>
   <si>
-    <t xml:space="preserve">Vent servo PWM channel. (Vent servo PWM)</t>
+    <t xml:space="preserve">Drainage vent servo PWM channel.</t>
   </si>
   <si>
     <t xml:space="preserve">DRAINAGE VENT</t>
@@ -255,9 +249,6 @@
   </si>
   <si>
     <t xml:space="preserve">VENT_MOVE_DELAY_MS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
   </si>
   <si>
     <t xml:space="preserve">Milisecond for vent movement, after which CLOSE/OPEN switchies are checked.</t>
@@ -345,7 +336,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -395,8 +386,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -406,13 +402,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC80"/>
-        <bgColor rgb="FFFFE0B2"/>
+        <bgColor rgb="FFE1BEE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5D6A7"/>
-        <bgColor rgb="FFC8E6C9"/>
+        <bgColor rgb="FF99CCFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -429,38 +425,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCDD2"/>
-        <bgColor rgb="FFFFE0B2"/>
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBBDEFB"/>
-        <bgColor rgb="FFC8E6C9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE0B2"/>
-        <bgColor rgb="FFFFF59D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC8E6C9"/>
-        <bgColor rgb="FFBBDEFB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF59D"/>
-        <bgColor rgb="FFFFE0B2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCE93D8"/>
-        <bgColor rgb="FF9999FF"/>
+        <fgColor rgb="FFE1BEE7"/>
+        <bgColor rgb="FFCC99FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -529,7 +501,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -558,7 +530,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -566,35 +538,39 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -602,11 +578,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -622,7 +598,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFF5F5F5"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -639,12 +615,12 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFE0B2"/>
+      <rgbColor rgb="FFFFFFCC"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFBBDEFB"/>
+      <rgbColor rgb="FFE1BEE7"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -655,11 +631,11 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC8E6C9"/>
-      <rgbColor rgb="FFFFF59D"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFFCDD2"/>
-      <rgbColor rgb="FFCE93D8"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC80"/>
       <rgbColor rgb="FF2196F3"/>
       <rgbColor rgb="FF29B6F6"/>
@@ -1178,105 +1154,126 @@
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
+      <c r="O5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="8"/>
+      <c r="G6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="5"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
-      <c r="E7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="E7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="5" t="s">
+      <c r="B8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5" t="s">
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="5" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5" t="s">
+      <c r="F9" s="11"/>
+      <c r="G9" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+      <c r="A10" s="10" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -1284,158 +1281,158 @@
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5" t="s">
+      <c r="F10" s="11"/>
+      <c r="G10" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="0" t="s">
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+    </row>
+    <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>34</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5" t="s">
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+    </row>
+    <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="0" t="s">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="12" t="s">
+      <c r="F12" s="11"/>
+      <c r="G12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="5" t="s">
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="12"/>
+    </row>
+    <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5" t="s">
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="0" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="12" t="s">
+      <c r="F13" s="11"/>
+      <c r="G13" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="5" t="s">
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+    </row>
+    <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5" t="s">
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="0" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="13" t="s">
+      <c r="F14" s="11"/>
+      <c r="G14" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="5" t="s">
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="12"/>
+    </row>
+    <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5" t="s">
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="0" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="13" t="s">
+      <c r="F15" s="11"/>
+      <c r="G15" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="0" t="s">
-        <v>37</v>
-      </c>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -1462,7 +1459,7 @@
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1508,30 +1505,40 @@
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
+      <c r="O18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="P18" s="4"/>
+      <c r="Q18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="11"/>
+      <c r="O19" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
@@ -1558,7 +1565,7 @@
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1604,30 +1611,40 @@
       <c r="L22" s="4"/>
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
+      <c r="O22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="P22" s="4"/>
+      <c r="Q22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
@@ -1654,7 +1671,7 @@
     </row>
     <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -1679,7 +1696,7 @@
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1707,7 +1724,7 @@
         <v>15</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
@@ -1717,7 +1734,7 @@
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
@@ -1733,30 +1750,30 @@
       <c r="R27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="n">
+      <c r="A28" s="15" t="n">
         <v>1</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
@@ -1767,20 +1784,20 @@
       <c r="R28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="n">
+      <c r="A29" s="15" t="n">
         <v>2</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
@@ -1788,7 +1805,7 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -1799,20 +1816,20 @@
       <c r="R29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="15" t="n">
         <v>3</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -1820,7 +1837,7 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
@@ -1831,20 +1848,20 @@
       <c r="R30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="15" t="n">
         <v>4</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
@@ -1852,7 +1869,7 @@
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
@@ -1863,20 +1880,20 @@
       <c r="R31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="n">
+      <c r="A32" s="15" t="n">
         <v>5</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
@@ -1884,7 +1901,7 @@
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
       <c r="K32" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
@@ -1895,30 +1912,30 @@
       <c r="R32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="15" t="n">
         <v>6</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5" t="s">
-        <v>78</v>
+        <v>21</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
       <c r="K33" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
@@ -1929,30 +1946,30 @@
       <c r="R33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="n">
+      <c r="A34" s="15" t="n">
         <v>7</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
       <c r="K34" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="L34" s="5"/>
       <c r="M34" s="5"/>
@@ -1963,30 +1980,30 @@
       <c r="R34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="n">
+      <c r="A35" s="15" t="n">
         <v>8</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
@@ -2021,7 +2038,7 @@
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -2054,7 +2071,7 @@
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
@@ -2070,25 +2087,25 @@
       <c r="O38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="n">
+      <c r="A39" s="15" t="n">
         <v>1</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
@@ -2099,25 +2116,25 @@
       <c r="O39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="7" t="n">
+      <c r="A40" s="15" t="n">
         <v>2</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
@@ -2152,7 +2169,7 @@
     </row>
     <row r="42" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -2177,13 +2194,13 @@
     </row>
     <row r="43" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>4</v>
@@ -2191,102 +2208,102 @@
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="H43" s="4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
       <c r="K43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="15"/>
-      <c r="C44" s="7"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="15"/>
       <c r="D44" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
-      <c r="H44" s="7" t="s">
+      <c r="H44" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="I44" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="J44" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="K44" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="I44" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="J44" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="K44" s="7" t="s">
-        <v>99</v>
-      </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7" t="n">
+      <c r="A45" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
       <c r="D45" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
-      <c r="H45" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I45" s="7" t="s">
+      <c r="H45" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I45" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="J45" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="K45" s="15" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="17"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="5" t="s">
         <v>100</v>
-      </c>
-      <c r="J45" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="K45" s="7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="B46" s="16"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="5" t="s">
-        <v>103</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="18"/>
+      <c r="J46" s="18"/>
+      <c r="K46" s="18"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7" t="n">
+      <c r="A47" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B47" s="18"/>
-      <c r="C47" s="18"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="19"/>
       <c r="D47" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
-      <c r="H47" s="17"/>
+      <c r="H47" s="18"/>
       <c r="I47" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J47" s="5"/>
-      <c r="K47" s="17"/>
+      <c r="K47" s="18"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="7" t="n">
+      <c r="A48" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B48" s="18"/>
-      <c r="C48" s="7"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="15"/>
       <c r="D48" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
@@ -2294,37 +2311,37 @@
       <c r="J48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="n">
+      <c r="A49" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B49" s="16"/>
-      <c r="C49" s="16"/>
+      <c r="B49" s="17"/>
+      <c r="C49" s="17"/>
       <c r="D49" s="5" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="7" t="n">
+      <c r="A50" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="19"/>
-      <c r="C50" s="7"/>
+      <c r="B50" s="20"/>
+      <c r="C50" s="15"/>
       <c r="D50" s="5" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7" t="n">
+      <c r="A51" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B51" s="19"/>
-      <c r="C51" s="19"/>
+      <c r="B51" s="20"/>
+      <c r="C51" s="20"/>
       <c r="D51" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
@@ -2353,7 +2370,7 @@
       <c r="U52" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="113">
+  <mergeCells count="120">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -2361,9 +2378,11 @@
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:N5"/>
+    <mergeCell ref="O5:Q5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="G6:N6"/>
+    <mergeCell ref="O6:Q8"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="G7:N7"/>
@@ -2373,6 +2392,7 @@
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="G9:N9"/>
+    <mergeCell ref="O9:Q15"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="G10:N10"/>
@@ -2396,17 +2416,21 @@
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="G18:N18"/>
+    <mergeCell ref="O18:Q18"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="G19:N19"/>
+    <mergeCell ref="O19:Q19"/>
     <mergeCell ref="A20:U20"/>
     <mergeCell ref="A21:U21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="G22:N22"/>
+    <mergeCell ref="O22:Q22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="G23:N23"/>
+    <mergeCell ref="O23:Q23"/>
     <mergeCell ref="A24:U24"/>
     <mergeCell ref="A25:U25"/>
     <mergeCell ref="A26:U26"/>

</xml_diff>

<commit_message>
[ Version 0.0.24.6 ] - drainage vent folder structure was updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="125">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -29,88 +29,157 @@
     <t xml:space="preserve">FOLDER STRUCTURE</t>
   </si>
   <si>
-    <t xml:space="preserve">1 LAYER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 LAYER</t>
+    <t xml:space="preserve">LAYER 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAYER 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">smart_flowerpot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">esp32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drivers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">motion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drainage_vent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">include</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drainage_vent.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drainage_vent.c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CmakeLists.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roulette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">code_plan.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flower_vent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">build</t>
+  </si>
+  <si>
+    <t xml:space="preserve">…</t>
+  </si>
+  <si>
+    <t xml:space="preserve">main</t>
+  </si>
+  <si>
+    <t xml:space="preserve">motion_main.c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sdkconfig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">libraries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwm_generator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwm_generator.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwm_generator.c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRIVERs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32 GPIO PINOUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIN</t>
   </si>
   <si>
     <t xml:space="preserve">DESCRIPTION</t>
   </si>
   <si>
-    <t xml:space="preserve">Main file of smart_flowerpot project.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRIVERS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTION</t>
+    <t xml:space="preserve">SECTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power 5V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Power 3.3V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GND.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_DRAIN_VENT_PWM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWM output for drainage vent servos.</t>
   </si>
   <si>
     <t xml:space="preserve">DRAINAGE_VENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vent system of drainage.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIBRARIES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PWM_GENERATOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generate PWM signal. Main purpose is for Servo driving.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRIVERs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESP32 GPIO PINOUT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SECTION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power 5V.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.3V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Power 3.3V.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GND.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_DRAIN_VENT_PWM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PWM output for drainage vent servos.</t>
   </si>
   <si>
     <t xml:space="preserve">OUT_DRAIN_VENT_SPM1</t>
@@ -380,16 +449,16 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -501,7 +570,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -526,7 +595,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -554,7 +627,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -769,7 +842,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U8"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -854,42 +927,66 @@
         <v>3</v>
       </c>
       <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
+      <c r="E4" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="G4" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="L4" s="4"/>
       <c r="M4" s="4" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
+      <c r="O4" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
+      <c r="Q4" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
+      <c r="S4" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="T4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
+      <c r="C5" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="E5" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
+      <c r="G5" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="I5" s="5" t="s">
+        <v>16</v>
+      </c>
       <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
+      <c r="K5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="L5" s="5"/>
       <c r="M5" s="5" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
@@ -900,27 +997,21 @@
       <c r="T5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>6</v>
-      </c>
+      <c r="A6" s="5"/>
       <c r="B6" s="5"/>
-      <c r="C6" s="5" t="s">
-        <v>7</v>
-      </c>
+      <c r="C6" s="5"/>
       <c r="D6" s="5"/>
-      <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
+      <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
+      <c r="K6" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="L6" s="5"/>
-      <c r="M6" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="M6" s="5"/>
       <c r="N6" s="5"/>
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
@@ -930,13 +1021,9 @@
       <c r="T6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>10</v>
-      </c>
+      <c r="A7" s="5"/>
       <c r="B7" s="5"/>
-      <c r="C7" s="5" t="s">
-        <v>11</v>
-      </c>
+      <c r="C7" s="5"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
       <c r="F7" s="5"/>
@@ -944,11 +1031,11 @@
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
+      <c r="K7" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="L7" s="5"/>
-      <c r="M7" s="5" t="s">
-        <v>12</v>
-      </c>
+      <c r="M7" s="5"/>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
       <c r="P7" s="5"/>
@@ -957,31 +1044,283 @@
       <c r="S7" s="5"/>
       <c r="T7" s="5"/>
     </row>
-    <row r="8" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
+    <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+    </row>
+    <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+    </row>
+    <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+    </row>
+    <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="5"/>
+      <c r="T12" s="5"/>
+    </row>
+    <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+    </row>
+    <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="5"/>
+      <c r="Q14" s="5"/>
+      <c r="R14" s="5"/>
+      <c r="S14" s="5"/>
+      <c r="T14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="5"/>
+      <c r="I15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J15" s="6"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="5"/>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="5"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
+      <c r="S16" s="5"/>
+      <c r="T16" s="5"/>
+    </row>
+    <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="5"/>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="5"/>
+      <c r="S17" s="5"/>
+      <c r="T17" s="5"/>
+    </row>
+    <row r="18" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="98">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -991,29 +1330,95 @@
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:T4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="A5:B17"/>
+    <mergeCell ref="C5:D14"/>
+    <mergeCell ref="E5:F14"/>
+    <mergeCell ref="G5:H14"/>
+    <mergeCell ref="I5:J7"/>
     <mergeCell ref="K5:L5"/>
-    <mergeCell ref="M5:T5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="S5:T5"/>
     <mergeCell ref="K6:L6"/>
-    <mergeCell ref="M6:T6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="Q6:R6"/>
+    <mergeCell ref="S6:T6"/>
     <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:T7"/>
-    <mergeCell ref="A8:U8"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="Q7:R7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="Q8:R8"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="Q9:R9"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="O10:P10"/>
+    <mergeCell ref="Q10:R10"/>
+    <mergeCell ref="S10:T10"/>
+    <mergeCell ref="I11:J12"/>
+    <mergeCell ref="K11:L11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="Q11:R11"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="O12:P12"/>
+    <mergeCell ref="Q12:R12"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="K13:L13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="Q13:R13"/>
+    <mergeCell ref="S13:T13"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="K14:L14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="S14:T14"/>
+    <mergeCell ref="C15:D17"/>
+    <mergeCell ref="E15:F17"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="K15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="S16:T16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="S17:T17"/>
+    <mergeCell ref="A18:U18"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1035,7 +1440,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1083,7 +1488,7 @@
     </row>
     <row r="3" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1107,45 +1512,45 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="6"/>
-      <c r="O4" s="6"/>
-      <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
+      <c r="A4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="7"/>
     </row>
     <row r="5" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
@@ -1155,284 +1560,284 @@
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="A6" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
+      <c r="B6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
-      <c r="N7" s="8"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
+      <c r="B7" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="A8" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
-      <c r="N8" s="8"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
+      <c r="B8" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="12" t="s">
+      <c r="B9" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13"/>
+      <c r="Q11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+    </row>
+    <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-    </row>
-    <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-    </row>
-    <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="12"/>
-      <c r="P13" s="12"/>
-      <c r="Q13" s="12"/>
+      <c r="B13" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="12"/>
-      <c r="Q14" s="12"/>
+      <c r="B14" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="13"/>
     </row>
     <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="12"/>
-      <c r="P15" s="12"/>
-      <c r="Q15" s="12"/>
+      <c r="B15" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="12"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -1458,45 +1863,45 @@
       <c r="U16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="6"/>
-      <c r="T17" s="6"/>
-      <c r="U17" s="6"/>
+      <c r="A17" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
+      <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
@@ -1506,39 +1911,39 @@
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
       <c r="O18" s="4" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="13"/>
+      <c r="B19" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
@@ -1564,45 +1969,45 @@
       <c r="U20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="6"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="6"/>
-      <c r="T21" s="6"/>
-      <c r="U21" s="6"/>
+      <c r="A21" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
+      <c r="Q21" s="7"/>
+      <c r="R21" s="7"/>
+      <c r="S21" s="7"/>
+      <c r="T21" s="7"/>
+      <c r="U21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
       <c r="E22" s="4" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
@@ -1612,39 +2017,39 @@
       <c r="M22" s="4"/>
       <c r="N22" s="4"/>
       <c r="O22" s="4" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
+      <c r="B23" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="P23" s="14"/>
+      <c r="Q23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
@@ -1670,76 +2075,76 @@
       <c r="U24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="14"/>
-      <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
-      <c r="R25" s="14"/>
-      <c r="S25" s="14"/>
-      <c r="T25" s="14"/>
-      <c r="U25" s="14"/>
+      <c r="A25" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
+      <c r="O25" s="15"/>
+      <c r="P25" s="15"/>
+      <c r="Q25" s="15"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+      <c r="T25" s="15"/>
+      <c r="U25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
-      <c r="T26" s="6"/>
-      <c r="U26" s="6"/>
+      <c r="A26" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="7"/>
+      <c r="R26" s="7"/>
+      <c r="S26" s="7"/>
+      <c r="T26" s="7"/>
+      <c r="U26" s="7"/>
     </row>
     <row r="27" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
@@ -1750,30 +2155,30 @@
       <c r="R27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="n">
+      <c r="A28" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5" t="s">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
@@ -1784,20 +2189,20 @@
       <c r="R28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="n">
+      <c r="A29" s="16" t="n">
         <v>2</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>64</v>
+        <v>87</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
@@ -1805,7 +2210,7 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -1816,20 +2221,20 @@
       <c r="R29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="n">
+      <c r="A30" s="16" t="n">
         <v>3</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -1837,7 +2242,7 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
@@ -1848,20 +2253,20 @@
       <c r="R30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="n">
+      <c r="A31" s="16" t="n">
         <v>4</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
@@ -1869,7 +2274,7 @@
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5" t="s">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
@@ -1880,20 +2285,20 @@
       <c r="R31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="n">
+      <c r="A32" s="16" t="n">
         <v>5</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
@@ -1901,7 +2306,7 @@
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
       <c r="K32" s="5" t="s">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
@@ -1912,30 +2317,30 @@
       <c r="R32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="n">
+      <c r="A33" s="16" t="n">
         <v>6</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>74</v>
+        <v>97</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
       <c r="K33" s="5" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
@@ -1946,30 +2351,30 @@
       <c r="R33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="n">
+      <c r="A34" s="16" t="n">
         <v>7</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
       <c r="K34" s="5" t="s">
-        <v>80</v>
+        <v>103</v>
       </c>
       <c r="L34" s="5"/>
       <c r="M34" s="5"/>
@@ -1980,30 +2385,30 @@
       <c r="R34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="n">
+      <c r="A35" s="16" t="n">
         <v>8</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5" t="s">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
@@ -2037,46 +2442,46 @@
       <c r="U36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
-      <c r="R37" s="6"/>
-      <c r="S37" s="6"/>
-      <c r="T37" s="6"/>
-      <c r="U37" s="6"/>
+      <c r="A37" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
+      <c r="K37" s="7"/>
+      <c r="L37" s="7"/>
+      <c r="M37" s="7"/>
+      <c r="N37" s="7"/>
+      <c r="O37" s="7"/>
+      <c r="P37" s="7"/>
+      <c r="Q37" s="7"/>
+      <c r="R37" s="7"/>
+      <c r="S37" s="7"/>
+      <c r="T37" s="7"/>
+      <c r="U37" s="7"/>
     </row>
     <row r="38" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4" t="s">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
@@ -2087,25 +2492,25 @@
       <c r="O38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="n">
+      <c r="A39" s="16" t="n">
         <v>1</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>85</v>
+        <v>108</v>
       </c>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
@@ -2116,25 +2521,25 @@
       <c r="O39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="n">
+      <c r="A40" s="16" t="n">
         <v>2</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>87</v>
+        <v>110</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
@@ -2168,142 +2573,142 @@
       <c r="U41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="6"/>
-      <c r="Q42" s="6"/>
-      <c r="R42" s="6"/>
-      <c r="S42" s="6"/>
-      <c r="T42" s="6"/>
-      <c r="U42" s="6"/>
+      <c r="A42" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
+      <c r="J42" s="7"/>
+      <c r="K42" s="7"/>
+      <c r="L42" s="7"/>
+      <c r="M42" s="7"/>
+      <c r="N42" s="7"/>
+      <c r="O42" s="7"/>
+      <c r="P42" s="7"/>
+      <c r="Q42" s="7"/>
+      <c r="R42" s="7"/>
+      <c r="S42" s="7"/>
+      <c r="T42" s="7"/>
+      <c r="U42" s="7"/>
     </row>
     <row r="43" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>89</v>
+        <v>112</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>90</v>
+        <v>113</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>91</v>
+        <v>114</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="H43" s="4" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="I43" s="4"/>
       <c r="J43" s="4"/>
       <c r="K43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="n">
+      <c r="A44" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="16"/>
-      <c r="C44" s="15"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="16"/>
       <c r="D44" s="5" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="E44" s="5"/>
       <c r="F44" s="5"/>
-      <c r="H44" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="I44" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="J44" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="K44" s="15" t="s">
-        <v>96</v>
+      <c r="H44" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="I44" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="J44" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="K44" s="16" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="n">
+      <c r="A45" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
+      <c r="B45" s="17"/>
+      <c r="C45" s="17"/>
       <c r="D45" s="5" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
-      <c r="H45" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="I45" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="J45" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="K45" s="15" t="s">
-        <v>99</v>
+      <c r="H45" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="I45" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="J45" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="n">
+      <c r="A46" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B46" s="17"/>
-      <c r="C46" s="15"/>
+      <c r="B46" s="18"/>
+      <c r="C46" s="16"/>
       <c r="D46" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
-      <c r="H46" s="18"/>
-      <c r="I46" s="18"/>
-      <c r="J46" s="18"/>
-      <c r="K46" s="18"/>
+      <c r="H46" s="19"/>
+      <c r="I46" s="19"/>
+      <c r="J46" s="19"/>
+      <c r="K46" s="19"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="n">
+      <c r="A47" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B47" s="19"/>
-      <c r="C47" s="19"/>
+      <c r="B47" s="20"/>
+      <c r="C47" s="20"/>
       <c r="D47" s="5" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
-      <c r="H47" s="18"/>
+      <c r="H47" s="19"/>
       <c r="I47" s="5" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="J47" s="5"/>
-      <c r="K47" s="18"/>
+      <c r="K47" s="19"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="n">
+      <c r="A48" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B48" s="19"/>
-      <c r="C48" s="15"/>
+      <c r="B48" s="20"/>
+      <c r="C48" s="16"/>
       <c r="D48" s="5" t="s">
-        <v>98</v>
+        <v>121</v>
       </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
@@ -2311,37 +2716,37 @@
       <c r="J48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="n">
+      <c r="A49" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="17"/>
+      <c r="B49" s="18"/>
+      <c r="C49" s="18"/>
       <c r="D49" s="5" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15" t="n">
+      <c r="A50" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="15"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="16"/>
       <c r="D50" s="5" t="s">
-        <v>99</v>
+        <v>122</v>
       </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="n">
+      <c r="A51" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B51" s="20"/>
-      <c r="C51" s="20"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="21"/>
       <c r="D51" s="5" t="s">
-        <v>95</v>
+        <v>118</v>
       </c>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>

</xml_diff>

<commit_message>
[ Version 0.0.24.7 ] - drainage vent program was updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="153">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -263,97 +263,181 @@
     <t xml:space="preserve">DRAINAGE VENT</t>
   </si>
   <si>
-    <t xml:space="preserve">VARIABLES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TYPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRUCT</t>
+    <t xml:space="preserve">STRUCTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FILE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATRIBUTE TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATRIBUTE NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_timer_config_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vsrp_dataset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_mode_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">speed_mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration structure for LEDC TIMER.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_timer_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer_num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_timer_bit_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">duty_resolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uint32_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">freq_hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_clk_cfg_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">clk_cfg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_channel_config_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration structure for LEDC CHANNEL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_channel_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">channel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer_sel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ledc_intr_type_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">intr_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gpio_num</t>
+  </si>
+  <si>
+    <t xml:space="preserve">duty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pwm_generator_config_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">timer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration structure for PWM GENERATOR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">out_pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">drainage_vent_dataset_t</t>
   </si>
   <si>
     <t xml:space="preserve">esp_timer_handle_t</t>
   </si>
   <si>
-    <t xml:space="preserve">vscp_timer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vsrp_dataset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One shot timer for switch off MOSFETs after some time constant. (vent system cut power)</t>
+    <t xml:space="preserve">power_cut_off_timer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset structure which store drainage vent runtime properties.</t>
   </si>
   <si>
     <t xml:space="preserve">TickType_t</t>
   </si>
   <si>
-    <t xml:space="preserve">vsrs_tick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tick of OPEN/CLOSE start action. (vent system request start)</t>
+    <t xml:space="preserve">event_start_tick</t>
   </si>
   <si>
     <t xml:space="preserve">uint8_t</t>
   </si>
   <si>
-    <t xml:space="preserve">vsp_code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Code of current process. (vent system process)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vsv1_enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logical value if vent 1 is enable. (vent system vent 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vsv2_enabled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logical value if vent 2 is enable. (vent system vent 2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">macro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VENT_MOVE_DELAY_MS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milisecond for vent movement, after which CLOSE/OPEN switchies are checked.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">time_t</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timestamp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Timestamp of error happened time.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">err_code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error code, describes what is broken and why it is broken. (error code)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STRUCTs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FILE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vent_driver.h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Struct for holding entire VENT system runtime properties. (vent system runtime properties)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Error structure.</t>
+    <t xml:space="preserve">control_flags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIT STRUCTURES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STRUCTURE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATRIBUTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIZE [bytes]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BYTE NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAINAGE V2 ENABLE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAINAGE V1 ENABLE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROCESS CODE</t>
   </si>
   <si>
     <t xml:space="preserve">RJ45 CONNECTION</t>
@@ -405,7 +489,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -449,16 +533,24 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="14"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -570,7 +662,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -595,11 +687,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -611,10 +699,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -623,19 +707,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1233,10 +1317,10 @@
         <v>17</v>
       </c>
       <c r="H15" s="5"/>
-      <c r="I15" s="6" t="s">
+      <c r="I15" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J15" s="6"/>
+      <c r="J15" s="5"/>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
@@ -1435,7 +1519,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U52"/>
+  <dimension ref="A1:W63"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1512,29 +1596,29 @@
       <c r="U3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
-      <c r="R4" s="7"/>
-      <c r="S4" s="7"/>
-      <c r="T4" s="7"/>
-      <c r="U4" s="7"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -1566,278 +1650,278 @@
       <c r="Q5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9" t="s">
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9" t="s">
+      <c r="F6" s="8"/>
+      <c r="G6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="10" t="s">
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9" t="s">
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="8"/>
+      <c r="G7" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="10"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9" t="s">
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9" t="s">
+      <c r="F8" s="8"/>
+      <c r="G8" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12" t="s">
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12" t="s">
+      <c r="F9" s="10"/>
+      <c r="G9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="13" t="s">
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12" t="s">
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12" t="s">
+      <c r="F10" s="10"/>
+      <c r="G10" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="13"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="13"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="n">
+      <c r="A11" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12" t="s">
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12" t="s">
+      <c r="F11" s="10"/>
+      <c r="G11" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="12"/>
-      <c r="M11" s="12"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="13"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
+      <c r="A12" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12" t="s">
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12" t="s">
+      <c r="F12" s="10"/>
+      <c r="G12" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="12"/>
-      <c r="M12" s="12"/>
-      <c r="N12" s="12"/>
-      <c r="O12" s="13"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="13"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
+      <c r="A13" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12" t="s">
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12" t="s">
+      <c r="F13" s="10"/>
+      <c r="G13" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="12"/>
-      <c r="N13" s="12"/>
-      <c r="O13" s="13"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="13"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
+      <c r="A14" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12" t="s">
+      <c r="F14" s="10"/>
+      <c r="G14" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
-      <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="13"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12" t="s">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12" t="s">
+      <c r="F15" s="10"/>
+      <c r="G15" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="12"/>
-      <c r="M15" s="12"/>
-      <c r="N15" s="12"/>
-      <c r="O15" s="13"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="13"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2"/>
@@ -1863,29 +1947,29 @@
       <c r="U16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-      <c r="S17" s="7"/>
-      <c r="T17" s="7"/>
-      <c r="U17" s="7"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="6"/>
+      <c r="S17" s="6"/>
+      <c r="T17" s="6"/>
+      <c r="U17" s="6"/>
     </row>
     <row r="18" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
@@ -1917,33 +2001,33 @@
       <c r="Q18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
+      <c r="A19" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12" t="s">
+      <c r="F19" s="10"/>
+      <c r="G19" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="12"/>
-      <c r="N19" s="12"/>
-      <c r="O19" s="14" t="s">
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="14"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2"/>
@@ -1969,29 +2053,29 @@
       <c r="U20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
-      <c r="S21" s="7"/>
-      <c r="T21" s="7"/>
-      <c r="U21" s="7"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="6"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="6"/>
+      <c r="U21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
@@ -2023,33 +2107,33 @@
       <c r="Q22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12" t="s">
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12" t="s">
+      <c r="F23" s="10"/>
+      <c r="G23" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="H23" s="12"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
-      <c r="L23" s="12"/>
-      <c r="M23" s="12"/>
-      <c r="N23" s="12"/>
-      <c r="O23" s="14" t="s">
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
@@ -2075,66 +2159,66 @@
       <c r="U24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="15"/>
-      <c r="S25" s="15"/>
-      <c r="T25" s="15"/>
-      <c r="U25" s="15"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="11"/>
+      <c r="O25" s="11"/>
+      <c r="P25" s="11"/>
+      <c r="Q25" s="11"/>
+      <c r="R25" s="11"/>
+      <c r="S25" s="11"/>
+      <c r="T25" s="11"/>
+      <c r="U25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
-      <c r="M26" s="7"/>
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="7"/>
-      <c r="S26" s="7"/>
-      <c r="T26" s="7"/>
-      <c r="U26" s="7"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
+      <c r="U26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" s="4"/>
       <c r="E27" s="4" t="s">
-        <v>37</v>
+        <v>81</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -2144,73 +2228,75 @@
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4" t="s">
-        <v>39</v>
+        <v>83</v>
       </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
+      <c r="N27" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="O27" s="4"/>
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
+      <c r="S27" s="4"/>
+      <c r="T27" s="4"/>
+      <c r="U27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="n">
+      <c r="A28" s="12" t="n">
         <v>1</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
       <c r="H28" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
       <c r="K28" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
-      <c r="N28" s="5"/>
+      <c r="N28" s="5" t="s">
+        <v>89</v>
+      </c>
       <c r="O28" s="5"/>
       <c r="P28" s="5"/>
       <c r="Q28" s="5"/>
       <c r="R28" s="5"/>
+      <c r="S28" s="5"/>
+      <c r="T28" s="5"/>
+      <c r="U28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>88</v>
-      </c>
+      <c r="A29" s="12"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
+      <c r="H29" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
       <c r="K29" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -2219,30 +2305,25 @@
       <c r="P29" s="5"/>
       <c r="Q29" s="5"/>
       <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
+      <c r="U29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>91</v>
-      </c>
+      <c r="A30" s="12"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
+      <c r="H30" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
@@ -2251,30 +2332,25 @@
       <c r="P30" s="5"/>
       <c r="Q30" s="5"/>
       <c r="R30" s="5"/>
+      <c r="S30" s="5"/>
+      <c r="T30" s="5"/>
+      <c r="U30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>93</v>
-      </c>
+      <c r="A31" s="12"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
+      <c r="H31" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
       <c r="K31" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
@@ -2283,30 +2359,25 @@
       <c r="P31" s="5"/>
       <c r="Q31" s="5"/>
       <c r="R31" s="5"/>
+      <c r="S31" s="5"/>
+      <c r="T31" s="5"/>
+      <c r="U31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>95</v>
-      </c>
+      <c r="A32" s="12"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
+      <c r="H32" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
       <c r="K32" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
@@ -2315,66 +2386,58 @@
       <c r="P32" s="5"/>
       <c r="Q32" s="5"/>
       <c r="R32" s="5"/>
+      <c r="S32" s="5"/>
+      <c r="T32" s="5"/>
+      <c r="U32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="16" t="n">
-        <v>6</v>
+      <c r="A33" s="12" t="n">
+        <v>2</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="E33" s="5" t="s">
         <v>98</v>
       </c>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
       <c r="H33" s="5" t="s">
-        <v>43</v>
+        <v>87</v>
       </c>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
       <c r="K33" s="5" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
-      <c r="N33" s="5"/>
+      <c r="N33" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="O33" s="5"/>
       <c r="P33" s="5"/>
       <c r="Q33" s="5"/>
       <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>101</v>
-      </c>
+      <c r="A34" s="12"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
       <c r="H34" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
       <c r="K34" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="L34" s="5"/>
       <c r="M34" s="5"/>
@@ -2383,32 +2446,25 @@
       <c r="P34" s="5"/>
       <c r="Q34" s="5"/>
       <c r="R34" s="5"/>
+      <c r="S34" s="5"/>
+      <c r="T34" s="5"/>
+      <c r="U34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="E35" s="5" t="s">
-        <v>104</v>
-      </c>
+      <c r="A35" s="12"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
       <c r="H35" s="5" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
       <c r="K35" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
@@ -2417,341 +2473,535 @@
       <c r="P35" s="5"/>
       <c r="Q35" s="5"/>
       <c r="R35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-      <c r="R36" s="2"/>
-      <c r="S36" s="2"/>
-      <c r="T36" s="2"/>
-      <c r="U36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="s">
+      <c r="S35" s="5"/>
+      <c r="T35" s="5"/>
+      <c r="U35" s="5"/>
+    </row>
+    <row r="36" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="L36" s="5"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
+      <c r="P36" s="5"/>
+      <c r="Q36" s="5"/>
+      <c r="R36" s="5"/>
+      <c r="S36" s="5"/>
+      <c r="T36" s="5"/>
+      <c r="U36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="7"/>
-      <c r="R37" s="7"/>
-      <c r="S37" s="7"/>
-      <c r="T37" s="7"/>
-      <c r="U37" s="7"/>
-    </row>
-    <row r="38" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4" t="s">
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+      <c r="S37" s="5"/>
+      <c r="T37" s="5"/>
+      <c r="U37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I38" s="4"/>
-      <c r="J38" s="4"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="4"/>
-      <c r="M38" s="4"/>
-      <c r="N38" s="4"/>
-      <c r="O38" s="4"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
+      <c r="Q38" s="5"/>
+      <c r="R38" s="5"/>
+      <c r="S38" s="5"/>
+      <c r="T38" s="5"/>
+      <c r="U38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D39" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>108</v>
-      </c>
+      <c r="A39" s="12"/>
+      <c r="B39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
+      <c r="K39" s="5" t="s">
+        <v>108</v>
+      </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
       <c r="N39" s="5"/>
       <c r="O39" s="5"/>
+      <c r="P39" s="5"/>
+      <c r="Q39" s="5"/>
+      <c r="R39" s="5"/>
+      <c r="S39" s="5"/>
+      <c r="T39" s="5"/>
+      <c r="U39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16" t="n">
-        <v>2</v>
+      <c r="A40" s="12" t="n">
+        <v>3</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>102</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
       <c r="E40" s="5" t="s">
-        <v>102</v>
+        <v>31</v>
       </c>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
+      <c r="K40" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
-      <c r="N40" s="5"/>
+      <c r="N40" s="5" t="s">
+        <v>111</v>
+      </c>
       <c r="O40" s="5"/>
-    </row>
-    <row r="41" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
-      <c r="P41" s="2"/>
-      <c r="Q41" s="2"/>
-      <c r="R41" s="2"/>
-      <c r="S41" s="2"/>
-      <c r="T41" s="2"/>
-      <c r="U41" s="2"/>
-    </row>
-    <row r="42" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7"/>
-      <c r="H42" s="7"/>
-      <c r="I42" s="7"/>
-      <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
-      <c r="L42" s="7"/>
-      <c r="M42" s="7"/>
-      <c r="N42" s="7"/>
-      <c r="O42" s="7"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="7"/>
-      <c r="R42" s="7"/>
-      <c r="S42" s="7"/>
-      <c r="T42" s="7"/>
-      <c r="U42" s="7"/>
-    </row>
-    <row r="43" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="P40" s="5"/>
+      <c r="Q40" s="5"/>
+      <c r="R40" s="5"/>
+      <c r="S40" s="5"/>
+      <c r="T40" s="5"/>
+      <c r="U40" s="5"/>
+    </row>
+    <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="L41" s="5"/>
+      <c r="M41" s="5"/>
+      <c r="N41" s="5"/>
+      <c r="O41" s="5"/>
+      <c r="P41" s="5"/>
+      <c r="Q41" s="5"/>
+      <c r="R41" s="5"/>
+      <c r="S41" s="5"/>
+      <c r="T41" s="5"/>
+      <c r="U41" s="5"/>
+    </row>
+    <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12"/>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="L42" s="5"/>
+      <c r="M42" s="5"/>
+      <c r="N42" s="5"/>
+      <c r="O42" s="5"/>
+      <c r="P42" s="5"/>
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
+      <c r="S42" s="5"/>
+      <c r="T42" s="5"/>
+      <c r="U42" s="5"/>
+    </row>
+    <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12"/>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="L43" s="5"/>
+      <c r="M43" s="5"/>
+      <c r="N43" s="5"/>
+      <c r="O43" s="5"/>
+      <c r="P43" s="5"/>
+      <c r="Q43" s="5"/>
+      <c r="R43" s="5"/>
+      <c r="S43" s="5"/>
+      <c r="T43" s="5"/>
+      <c r="U43" s="5"/>
+    </row>
+    <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E43" s="4"/>
-      <c r="F43" s="4"/>
-      <c r="H43" s="4" t="s">
+      <c r="I44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K44" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-    </row>
-    <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="B44" s="17"/>
-      <c r="C44" s="16"/>
-      <c r="D44" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="H44" s="16" t="s">
+      <c r="L44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="N44" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="I44" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="J44" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="K44" s="16" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="5" t="s">
-        <v>116</v>
-      </c>
+      <c r="O44" s="5"/>
+      <c r="P44" s="5"/>
+      <c r="Q44" s="5"/>
+      <c r="R44" s="5"/>
+      <c r="S44" s="5"/>
+      <c r="T44" s="5"/>
+      <c r="U44" s="5"/>
+    </row>
+    <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12"/>
+      <c r="B45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
-      <c r="H45" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="I45" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="J45" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="K45" s="16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B46" s="18"/>
-      <c r="C46" s="16"/>
-      <c r="D46" s="5" t="s">
-        <v>123</v>
-      </c>
+      <c r="G45" s="5"/>
+      <c r="H45" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K45" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="L45" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M45" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="N45" s="5"/>
+      <c r="O45" s="5"/>
+      <c r="P45" s="5"/>
+      <c r="Q45" s="5"/>
+      <c r="R45" s="5"/>
+      <c r="S45" s="5"/>
+      <c r="T45" s="5"/>
+      <c r="U45" s="5"/>
+    </row>
+    <row r="46" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="12"/>
+      <c r="B46" s="5"/>
+      <c r="C46" s="5"/>
+      <c r="D46" s="5"/>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19"/>
-      <c r="J46" s="19"/>
-      <c r="K46" s="19"/>
-    </row>
-    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="5" t="s">
+      <c r="G46" s="5"/>
+      <c r="H46" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J46" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K46" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L46" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="M46" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="N46" s="5"/>
+      <c r="O46" s="5"/>
+      <c r="P46" s="5"/>
+      <c r="Q46" s="5"/>
+      <c r="R46" s="5"/>
+      <c r="S46" s="5"/>
+      <c r="T46" s="5"/>
+      <c r="U46" s="5"/>
+    </row>
+    <row r="47" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="2"/>
+      <c r="M47" s="2"/>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
+      <c r="P47" s="2"/>
+      <c r="Q47" s="2"/>
+      <c r="R47" s="2"/>
+      <c r="S47" s="2"/>
+      <c r="T47" s="2"/>
+      <c r="U47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6"/>
+      <c r="K48" s="6"/>
+      <c r="L48" s="6"/>
+      <c r="M48" s="6"/>
+      <c r="N48" s="6"/>
+      <c r="O48" s="6"/>
+      <c r="P48" s="6"/>
+      <c r="Q48" s="6"/>
+      <c r="R48" s="6"/>
+      <c r="S48" s="6"/>
+      <c r="T48" s="6"/>
+      <c r="U48" s="6"/>
+      <c r="V48" s="6"/>
+      <c r="W48" s="6"/>
+    </row>
+    <row r="49" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="J47" s="5"/>
-      <c r="K47" s="19"/>
-    </row>
-    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="16"/>
-      <c r="D48" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
-    </row>
-    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="B49" s="18"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-    </row>
-    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="16" t="n">
-        <v>7</v>
-      </c>
-      <c r="B50" s="21"/>
-      <c r="C50" s="16"/>
-      <c r="D50" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-    </row>
-    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="B51" s="21"/>
-      <c r="C51" s="21"/>
-      <c r="D51" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-    </row>
-    <row r="52" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="O49" s="4"/>
+      <c r="P49" s="4"/>
+      <c r="Q49" s="4"/>
+      <c r="R49" s="4"/>
+      <c r="S49" s="4"/>
+      <c r="T49" s="4"/>
+      <c r="U49" s="4"/>
+      <c r="V49" s="4"/>
+      <c r="W49" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+      <c r="H50" s="4"/>
+      <c r="I50" s="4"/>
+      <c r="J50" s="4"/>
+      <c r="K50" s="4"/>
+      <c r="L50" s="4"/>
+      <c r="M50" s="4"/>
+      <c r="N50" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="O50" s="13"/>
+      <c r="P50" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q50" s="13"/>
+      <c r="R50" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="S50" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="T50" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="U50" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="V50" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="W50" s="13" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="G51" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="K51" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="O51" s="5"/>
+      <c r="P51" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q51" s="5"/>
+      <c r="R51" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="S51" s="5"/>
+      <c r="T51" s="5"/>
+      <c r="U51" s="5"/>
+      <c r="V51" s="5"/>
+      <c r="W51" s="5"/>
+    </row>
+    <row r="52" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -2774,8 +3024,210 @@
       <c r="T52" s="2"/>
       <c r="U52" s="2"/>
     </row>
+    <row r="53" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="6"/>
+      <c r="N53" s="6"/>
+      <c r="O53" s="6"/>
+      <c r="P53" s="6"/>
+      <c r="Q53" s="6"/>
+      <c r="R53" s="6"/>
+      <c r="S53" s="6"/>
+      <c r="T53" s="6"/>
+      <c r="U53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="H54" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B55" s="15"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E55" s="5"/>
+      <c r="F55" s="5"/>
+      <c r="H55" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="I55" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="J55" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="K55" s="12" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="H56" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="I56" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="J56" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="K56" s="12" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B57" s="16"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="H57" s="17"/>
+      <c r="I57" s="17"/>
+      <c r="J57" s="17"/>
+      <c r="K57" s="17"/>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E58" s="5"/>
+      <c r="F58" s="5"/>
+      <c r="H58" s="17"/>
+      <c r="I58" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="J58" s="5"/>
+      <c r="K58" s="17"/>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B59" s="18"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E59" s="5"/>
+      <c r="F59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="5"/>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B61" s="19"/>
+      <c r="C61" s="12"/>
+      <c r="D61" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B62" s="19"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
+      <c r="L63" s="2"/>
+      <c r="M63" s="2"/>
+      <c r="N63" s="2"/>
+      <c r="O63" s="2"/>
+      <c r="P63" s="2"/>
+      <c r="Q63" s="2"/>
+      <c r="R63" s="2"/>
+      <c r="S63" s="2"/>
+      <c r="T63" s="2"/>
+      <c r="U63" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="120">
+  <mergeCells count="153">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -2842,60 +3294,93 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="E27:G27"/>
     <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:R27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="H28:J32"/>
-    <mergeCell ref="K28:R28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="K29:R29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="K30:R30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="K31:R31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="K32:R32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="N27:U27"/>
+    <mergeCell ref="A28:A32"/>
+    <mergeCell ref="B28:D32"/>
+    <mergeCell ref="E28:G39"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="N28:U32"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="K29:M29"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="A33:A39"/>
+    <mergeCell ref="B33:D39"/>
     <mergeCell ref="H33:J33"/>
-    <mergeCell ref="K33:R33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="N33:U39"/>
     <mergeCell ref="H34:J34"/>
-    <mergeCell ref="K34:R34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="K34:M34"/>
     <mergeCell ref="H35:J35"/>
-    <mergeCell ref="K35:R35"/>
-    <mergeCell ref="A36:U36"/>
-    <mergeCell ref="A37:U37"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="H38:O38"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="H39:O39"/>
-    <mergeCell ref="B40:D40"/>
-    <mergeCell ref="E40:G40"/>
-    <mergeCell ref="H40:O40"/>
-    <mergeCell ref="A41:U41"/>
-    <mergeCell ref="A42:U42"/>
-    <mergeCell ref="D43:F43"/>
-    <mergeCell ref="H43:K43"/>
-    <mergeCell ref="D44:F44"/>
-    <mergeCell ref="D45:F45"/>
-    <mergeCell ref="D46:F46"/>
-    <mergeCell ref="D47:F47"/>
-    <mergeCell ref="I47:J48"/>
-    <mergeCell ref="D48:F48"/>
-    <mergeCell ref="D49:F49"/>
-    <mergeCell ref="D50:F50"/>
-    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="A40:A43"/>
+    <mergeCell ref="B40:D43"/>
+    <mergeCell ref="E40:G43"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="N40:U43"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="K43:M43"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B44:D46"/>
+    <mergeCell ref="E44:G46"/>
+    <mergeCell ref="H44:J44"/>
+    <mergeCell ref="K44:M44"/>
+    <mergeCell ref="N44:U46"/>
+    <mergeCell ref="H45:J45"/>
+    <mergeCell ref="K45:M45"/>
+    <mergeCell ref="H46:J46"/>
+    <mergeCell ref="K46:M46"/>
+    <mergeCell ref="A47:U47"/>
+    <mergeCell ref="A48:W48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="B49:D50"/>
+    <mergeCell ref="E49:G50"/>
+    <mergeCell ref="H49:J50"/>
+    <mergeCell ref="K49:M50"/>
+    <mergeCell ref="N49:O49"/>
+    <mergeCell ref="P49:V49"/>
+    <mergeCell ref="N50:O50"/>
+    <mergeCell ref="P50:Q50"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="H51:J51"/>
+    <mergeCell ref="K51:M51"/>
+    <mergeCell ref="N51:O51"/>
+    <mergeCell ref="P51:Q51"/>
+    <mergeCell ref="R51:W51"/>
     <mergeCell ref="A52:U52"/>
+    <mergeCell ref="A53:U53"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="H54:K54"/>
+    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="D56:F56"/>
+    <mergeCell ref="D57:F57"/>
+    <mergeCell ref="D58:F58"/>
+    <mergeCell ref="I58:J59"/>
+    <mergeCell ref="D59:F59"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="A63:U63"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.24.8 ] - drainage vent program was finished.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -212,25 +212,25 @@
     <t xml:space="preserve">IN_DRAIN_VENT_ESO2</t>
   </si>
   <si>
+    <t xml:space="preserve">GPIO39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI (only) for drainage vent V2 open position end switch - end switch open 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI (only) for drainage vent V1 close position end switch - end switch close 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_DRAIN_VENT_ESC2</t>
+  </si>
+  <si>
     <t xml:space="preserve">GPIO36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI (only) for drainage vent V2 open position end switch - end switch open 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_DRAIN_VENT_ESC1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI (only) for drainage vent V1 close position end switch - end switch close 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_DRAIN_VENT_ESC2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO39</t>
   </si>
   <si>
     <t xml:space="preserve">DI (only) for drainage vent V2 close position end switch - end switch close 2.</t>
@@ -489,7 +489,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -546,11 +546,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -662,7 +657,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -716,10 +711,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2952,22 +2943,22 @@
       <c r="A51" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B51" s="14" t="s">
+      <c r="B51" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="14" t="s">
+      <c r="C51" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D51" s="14" t="s">
+      <c r="D51" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="E51" s="14" t="s">
+      <c r="E51" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="F51" s="14" t="s">
+      <c r="F51" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="G51" s="14" t="s">
+      <c r="G51" s="5" t="s">
         <v>85</v>
       </c>
       <c r="H51" s="5" t="n">
@@ -3075,7 +3066,7 @@
       <c r="A55" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B55" s="15"/>
+      <c r="B55" s="14"/>
       <c r="C55" s="12"/>
       <c r="D55" s="5" t="s">
         <v>45</v>
@@ -3099,8 +3090,8 @@
       <c r="A56" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B56" s="15"/>
-      <c r="C56" s="15"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="14"/>
       <c r="D56" s="5" t="s">
         <v>144</v>
       </c>
@@ -3123,41 +3114,41 @@
       <c r="A57" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B57" s="16"/>
+      <c r="B57" s="15"/>
       <c r="C57" s="12"/>
       <c r="D57" s="5" t="s">
         <v>151</v>
       </c>
       <c r="E57" s="5"/>
       <c r="F57" s="5"/>
-      <c r="H57" s="17"/>
-      <c r="I57" s="17"/>
-      <c r="J57" s="17"/>
-      <c r="K57" s="17"/>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
+      <c r="J57" s="16"/>
+      <c r="K57" s="16"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B58" s="18"/>
-      <c r="C58" s="18"/>
+      <c r="B58" s="17"/>
+      <c r="C58" s="17"/>
       <c r="D58" s="5" t="s">
         <v>145</v>
       </c>
       <c r="E58" s="5"/>
       <c r="F58" s="5"/>
-      <c r="H58" s="17"/>
+      <c r="H58" s="16"/>
       <c r="I58" s="5" t="s">
         <v>152</v>
       </c>
       <c r="J58" s="5"/>
-      <c r="K58" s="17"/>
+      <c r="K58" s="16"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B59" s="18"/>
+      <c r="B59" s="17"/>
       <c r="C59" s="12"/>
       <c r="D59" s="5" t="s">
         <v>149</v>
@@ -3171,8 +3162,8 @@
       <c r="A60" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B60" s="16"/>
-      <c r="C60" s="16"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
       <c r="D60" s="5" t="s">
         <v>147</v>
       </c>
@@ -3183,7 +3174,7 @@
       <c r="A61" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B61" s="19"/>
+      <c r="B61" s="18"/>
       <c r="C61" s="12"/>
       <c r="D61" s="5" t="s">
         <v>150</v>
@@ -3195,8 +3186,8 @@
       <c r="A62" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B62" s="19"/>
-      <c r="C62" s="19"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
       <c r="D62" s="5" t="s">
         <v>146</v>
       </c>

</xml_diff>

<commit_message>
[ Version 0.0.24.9 ] - roulette temporary GPIOs was added to Excel.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="185">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -146,15 +146,15 @@
     <t xml:space="preserve">SECTION</t>
   </si>
   <si>
+    <t xml:space="preserve">NOTE</t>
+  </si>
+  <si>
     <t xml:space="preserve">5V</t>
   </si>
   <si>
     <t xml:space="preserve">Power 5V.</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
     <t xml:space="preserve">3V</t>
   </si>
   <si>
@@ -234,6 +234,102 @@
   </si>
   <si>
     <t xml:space="preserve">DI (only) for drainage vent V2 close position end switch - end switch close 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_EN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver enable pin – enable 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEMPORARY!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_EN2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R2 motor driver enable pin – enable 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR1_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 1 – direction 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR1_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 2 – direction 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR2_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R2 motor driver direction bit 1 – direction 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR2_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R2 motor driver direction bit 2 – direction 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESO1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 open position end switches – end switch open 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESO2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R2 open position end switches – end switch open 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESC1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R1 close position end switches – end switch close 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R2 close position end switches – end switch close 2.</t>
   </si>
   <si>
     <t xml:space="preserve">ESP-IDF TIMERS</t>
@@ -548,7 +644,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -558,7 +654,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC80"/>
-        <bgColor rgb="FFE1BEE7"/>
+        <bgColor rgb="FFF8BBD0"/>
       </patternFill>
     </fill>
     <fill>
@@ -588,7 +684,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE1BEE7"/>
-        <bgColor rgb="FFCC99FF"/>
+        <bgColor rgb="FFF8BBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8BBD0"/>
+        <bgColor rgb="FFE1BEE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -657,7 +759,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -694,11 +796,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -714,11 +836,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -726,11 +848,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -782,7 +904,7 @@
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFF8BBD0"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC80"/>
       <rgbColor rgb="FF2196F3"/>
@@ -1510,7 +1632,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W63"/>
+  <dimension ref="A1:W73"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1639,22 +1761,28 @@
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
+      <c r="R5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
@@ -1663,11 +1791,13 @@
       <c r="L6" s="8"/>
       <c r="M6" s="8"/>
       <c r="N6" s="8"/>
-      <c r="O6" s="8" t="s">
-        <v>43</v>
-      </c>
+      <c r="O6" s="8"/>
       <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
@@ -1695,6 +1825,10 @@
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+      <c r="U7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="n">
@@ -1722,825 +1856,895 @@
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10" t="s">
+      <c r="F9" s="11"/>
+      <c r="G9" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10" t="s">
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="n">
+      <c r="A10" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10" t="s">
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10" t="s">
+      <c r="F10" s="11"/>
+      <c r="G10" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="n">
+      <c r="A11" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10" t="s">
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10" t="s">
+      <c r="F11" s="11"/>
+      <c r="G11" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="n">
+      <c r="A12" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10" t="s">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10" t="s">
+      <c r="F12" s="11"/>
+      <c r="G12" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="n">
+      <c r="A13" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10" t="s">
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10" t="s">
+      <c r="F13" s="11"/>
+      <c r="G13" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="10"/>
-      <c r="Q13" s="10"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="11"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="n">
+      <c r="A14" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10" t="s">
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10" t="s">
+      <c r="F14" s="11"/>
+      <c r="G14" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="n">
+      <c r="A15" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10" t="s">
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10" t="s">
+      <c r="F15" s="11"/>
+      <c r="G15" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-    </row>
-    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="12"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="12"/>
+      <c r="U15" s="12"/>
+    </row>
+    <row r="16" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="6"/>
-      <c r="T17" s="6"/>
-      <c r="U17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="S16" s="15"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+    </row>
+    <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+      <c r="M17" s="14"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="14"/>
+      <c r="P17" s="14"/>
+      <c r="Q17" s="14"/>
+      <c r="R17" s="15"/>
+      <c r="S17" s="15"/>
+      <c r="T17" s="15"/>
+      <c r="U17" s="15"/>
+    </row>
+    <row r="18" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
+      <c r="N18" s="14"/>
+      <c r="O18" s="14"/>
+      <c r="P18" s="14"/>
+      <c r="Q18" s="14"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="15"/>
+      <c r="T18" s="15"/>
+      <c r="U18" s="15"/>
+    </row>
+    <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
+      <c r="J19" s="14"/>
+      <c r="K19" s="14"/>
+      <c r="L19" s="14"/>
+      <c r="M19" s="14"/>
+      <c r="N19" s="14"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="15"/>
+      <c r="S19" s="15"/>
+      <c r="T19" s="15"/>
+      <c r="U19" s="15"/>
+    </row>
+    <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="H20" s="14"/>
+      <c r="I20" s="14"/>
+      <c r="J20" s="14"/>
+      <c r="K20" s="14"/>
+      <c r="L20" s="14"/>
+      <c r="M20" s="14"/>
+      <c r="N20" s="14"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="15"/>
+      <c r="S20" s="15"/>
+      <c r="T20" s="15"/>
+      <c r="U20" s="15"/>
+    </row>
+    <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H21" s="14"/>
+      <c r="I21" s="14"/>
+      <c r="J21" s="14"/>
+      <c r="K21" s="14"/>
+      <c r="L21" s="14"/>
+      <c r="M21" s="14"/>
+      <c r="N21" s="14"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="15"/>
+      <c r="S21" s="15"/>
+      <c r="T21" s="15"/>
+      <c r="U21" s="15"/>
+    </row>
+    <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="H22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="14"/>
+      <c r="Q22" s="14"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="15"/>
+      <c r="T22" s="15"/>
+      <c r="U22" s="15"/>
+    </row>
+    <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="H23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="14"/>
+      <c r="L23" s="14"/>
+      <c r="M23" s="14"/>
+      <c r="N23" s="14"/>
+      <c r="O23" s="14"/>
+      <c r="P23" s="14"/>
+      <c r="Q23" s="14"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="15"/>
+      <c r="T23" s="15"/>
+      <c r="U23" s="15"/>
+    </row>
+    <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
+      <c r="M24" s="14"/>
+      <c r="N24" s="14"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="14"/>
+      <c r="R24" s="15"/>
+      <c r="S24" s="15"/>
+      <c r="T24" s="15"/>
+      <c r="U24" s="15"/>
+    </row>
+    <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+      <c r="L25" s="14"/>
+      <c r="M25" s="14"/>
+      <c r="N25" s="14"/>
+      <c r="O25" s="14"/>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="14"/>
+      <c r="R25" s="15"/>
+      <c r="S25" s="15"/>
+      <c r="T25" s="15"/>
+      <c r="U25" s="15"/>
+    </row>
+    <row r="26" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
+      <c r="R26" s="2"/>
+      <c r="S26" s="2"/>
+      <c r="T26" s="2"/>
+      <c r="U26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6"/>
+      <c r="R27" s="6"/>
+      <c r="S27" s="6"/>
+      <c r="T27" s="6"/>
+      <c r="U27" s="6"/>
+    </row>
+    <row r="28" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B28" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4" t="s">
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4" t="s">
+      <c r="F28" s="4"/>
+      <c r="G28" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4" t="s">
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="n">
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
+    </row>
+    <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="10" t="s">
+      <c r="B29" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
+      <c r="L29" s="11"/>
+      <c r="M29" s="11"/>
+      <c r="N29" s="11"/>
+      <c r="O29" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
-      <c r="T20" s="2"/>
-      <c r="U20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="6"/>
-      <c r="P21" s="6"/>
-      <c r="Q21" s="6"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="6"/>
-      <c r="T21" s="6"/>
-      <c r="U21" s="6"/>
-    </row>
-    <row r="22" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="P29" s="11"/>
+      <c r="Q29" s="11"/>
+    </row>
+    <row r="30" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="2"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
+      <c r="T30" s="2"/>
+      <c r="U30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4" t="s">
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4" t="s">
+      <c r="F32" s="4"/>
+      <c r="G32" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4" t="s">
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4"/>
+      <c r="O32" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9" t="n">
+      <c r="P32" s="4"/>
+      <c r="Q32" s="4"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
-      <c r="O23" s="10" t="s">
+      <c r="B33" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+      <c r="J33" s="11"/>
+      <c r="K33" s="11"/>
+      <c r="L33" s="11"/>
+      <c r="M33" s="11"/>
+      <c r="N33" s="11"/>
+      <c r="O33" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="P23" s="10"/>
-      <c r="Q23" s="10"/>
-    </row>
-    <row r="24" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
-      <c r="R25" s="11"/>
-      <c r="S25" s="11"/>
-      <c r="T25" s="11"/>
-      <c r="U25" s="11"/>
-    </row>
-    <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="6"/>
-      <c r="P26" s="6"/>
-      <c r="Q26" s="6"/>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
-      <c r="T26" s="6"/>
-      <c r="U26" s="6"/>
-    </row>
-    <row r="27" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="P33" s="11"/>
+      <c r="Q33" s="11"/>
+    </row>
+    <row r="34" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
+      <c r="O34" s="2"/>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="2"/>
+      <c r="R34" s="2"/>
+      <c r="S34" s="2"/>
+      <c r="T34" s="2"/>
+      <c r="U34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
+      <c r="O35" s="16"/>
+      <c r="P35" s="16"/>
+      <c r="Q35" s="16"/>
+      <c r="R35" s="16"/>
+      <c r="S35" s="16"/>
+      <c r="T35" s="16"/>
+      <c r="U35" s="16"/>
+    </row>
+    <row r="36" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" s="6"/>
+      <c r="C36" s="6"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="6"/>
+      <c r="N36" s="6"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6"/>
+      <c r="R36" s="6"/>
+      <c r="S36" s="6"/>
+      <c r="T36" s="6"/>
+      <c r="U36" s="6"/>
+    </row>
+    <row r="37" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B37" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4" t="s">
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="L37" s="4"/>
+      <c r="M37" s="4"/>
+      <c r="N37" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="O27" s="4"/>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-      <c r="R27" s="4"/>
-      <c r="S27" s="4"/>
-      <c r="T27" s="4"/>
-      <c r="U27" s="4"/>
-    </row>
-    <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="n">
+      <c r="O37" s="4"/>
+      <c r="P37" s="4"/>
+      <c r="Q37" s="4"/>
+      <c r="R37" s="4"/>
+      <c r="S37" s="4"/>
+      <c r="T37" s="4"/>
+      <c r="U37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
-      <c r="U28" s="5"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-    </row>
-    <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
-      <c r="S30" s="5"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
-    </row>
-    <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5"/>
-      <c r="R31" s="5"/>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
-      <c r="U31" s="5"/>
-    </row>
-    <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="12"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5"/>
-      <c r="R32" s="5"/>
-      <c r="S32" s="5"/>
-      <c r="T32" s="5"/>
-      <c r="U32" s="5"/>
-    </row>
-    <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
-      <c r="S33" s="5"/>
-      <c r="T33" s="5"/>
-      <c r="U33" s="5"/>
-    </row>
-    <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="5"/>
-      <c r="O34" s="5"/>
-      <c r="P34" s="5"/>
-      <c r="Q34" s="5"/>
-      <c r="R34" s="5"/>
-      <c r="S34" s="5"/>
-      <c r="T34" s="5"/>
-      <c r="U34" s="5"/>
-    </row>
-    <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="5"/>
-      <c r="O35" s="5"/>
-      <c r="P35" s="5"/>
-      <c r="Q35" s="5"/>
-      <c r="R35" s="5"/>
-      <c r="S35" s="5"/>
-      <c r="T35" s="5"/>
-      <c r="U35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="5"/>
-      <c r="O36" s="5"/>
-      <c r="P36" s="5"/>
-      <c r="Q36" s="5"/>
-      <c r="R36" s="5"/>
-      <c r="S36" s="5"/>
-      <c r="T36" s="5"/>
-      <c r="U36" s="5"/>
-    </row>
-    <row r="37" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="L37" s="5"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="5"/>
-      <c r="O37" s="5"/>
-      <c r="P37" s="5"/>
-      <c r="Q37" s="5"/>
-      <c r="R37" s="5"/>
-      <c r="S37" s="5"/>
-      <c r="T37" s="5"/>
-      <c r="U37" s="5"/>
-    </row>
-    <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
+      <c r="B38" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>118</v>
+      </c>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
-      <c r="N38" s="5"/>
+      <c r="N38" s="5" t="s">
+        <v>121</v>
+      </c>
       <c r="O38" s="5"/>
       <c r="P38" s="5"/>
       <c r="Q38" s="5"/>
@@ -2550,7 +2754,7 @@
       <c r="U38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12"/>
+      <c r="A39" s="17"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -2558,12 +2762,12 @@
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
       <c r="K39" s="5" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -2577,32 +2781,24 @@
       <c r="U39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>109</v>
-      </c>
+      <c r="A40" s="17"/>
+      <c r="B40" s="5"/>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
-      <c r="E40" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="E40" s="5"/>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
-      <c r="N40" s="5" t="s">
-        <v>111</v>
-      </c>
+      <c r="N40" s="5"/>
       <c r="O40" s="5"/>
       <c r="P40" s="5"/>
       <c r="Q40" s="5"/>
@@ -2612,7 +2808,7 @@
       <c r="U40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12"/>
+      <c r="A41" s="17"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -2620,12 +2816,12 @@
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>100</v>
+        <v>126</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5" t="s">
-        <v>101</v>
+        <v>127</v>
       </c>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
@@ -2639,7 +2835,7 @@
       <c r="U41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12"/>
+      <c r="A42" s="17"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
@@ -2647,12 +2843,12 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5" t="s">
-        <v>94</v>
+        <v>128</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5" t="s">
-        <v>95</v>
+        <v>129</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
@@ -2666,24 +2862,30 @@
       <c r="U42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12"/>
-      <c r="B43" s="5"/>
+      <c r="A43" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>130</v>
+      </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
-      <c r="N43" s="5"/>
+      <c r="N43" s="5" t="s">
+        <v>131</v>
+      </c>
       <c r="O43" s="5"/>
       <c r="P43" s="5"/>
       <c r="Q43" s="5"/>
@@ -2693,44 +2895,24 @@
       <c r="U43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="A44" s="17"/>
+      <c r="B44" s="5"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="I44" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J44" s="5" t="s">
-        <v>85</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
       <c r="K44" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="L44" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="M44" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="N44" s="5" t="s">
-        <v>116</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="L44" s="5"/>
+      <c r="M44" s="5"/>
+      <c r="N44" s="5"/>
       <c r="O44" s="5"/>
       <c r="P44" s="5"/>
       <c r="Q44" s="5"/>
@@ -2740,7 +2922,7 @@
       <c r="U44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="12"/>
+      <c r="A45" s="17"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
@@ -2748,23 +2930,15 @@
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
       <c r="H45" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="I45" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J45" s="5" t="s">
-        <v>85</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
       <c r="K45" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="L45" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="M45" s="5" t="s">
-        <v>85</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="L45" s="5"/>
+      <c r="M45" s="5"/>
       <c r="N45" s="5"/>
       <c r="O45" s="5"/>
       <c r="P45" s="5"/>
@@ -2775,7 +2949,7 @@
       <c r="U45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="12"/>
+      <c r="A46" s="17"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
@@ -2783,23 +2957,15 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="I46" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J46" s="5" t="s">
-        <v>85</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
       <c r="K46" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="L46" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="M46" s="5" t="s">
-        <v>85</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="L46" s="5"/>
+      <c r="M46" s="5"/>
       <c r="N46" s="5"/>
       <c r="O46" s="5"/>
       <c r="P46" s="5"/>
@@ -2809,416 +2975,730 @@
       <c r="T46" s="5"/>
       <c r="U46" s="5"/>
     </row>
-    <row r="47" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
-      <c r="N47" s="2"/>
-      <c r="O47" s="2"/>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="R47" s="2"/>
-      <c r="S47" s="2"/>
-      <c r="T47" s="2"/>
-      <c r="U47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="6"/>
-      <c r="N48" s="6"/>
-      <c r="O48" s="6"/>
-      <c r="P48" s="6"/>
-      <c r="Q48" s="6"/>
-      <c r="R48" s="6"/>
-      <c r="S48" s="6"/>
-      <c r="T48" s="6"/>
-      <c r="U48" s="6"/>
-      <c r="V48" s="6"/>
-      <c r="W48" s="6"/>
-    </row>
-    <row r="49" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B49" s="4" t="s">
+    <row r="47" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="17"/>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
+      <c r="E47" s="5"/>
+      <c r="F47" s="5"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="L47" s="5"/>
+      <c r="M47" s="5"/>
+      <c r="N47" s="5"/>
+      <c r="O47" s="5"/>
+      <c r="P47" s="5"/>
+      <c r="Q47" s="5"/>
+      <c r="R47" s="5"/>
+      <c r="S47" s="5"/>
+      <c r="T47" s="5"/>
+      <c r="U47" s="5"/>
+    </row>
+    <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="17"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="L48" s="5"/>
+      <c r="M48" s="5"/>
+      <c r="N48" s="5"/>
+      <c r="O48" s="5"/>
+      <c r="P48" s="5"/>
+      <c r="Q48" s="5"/>
+      <c r="R48" s="5"/>
+      <c r="S48" s="5"/>
+      <c r="T48" s="5"/>
+      <c r="U48" s="5"/>
+    </row>
+    <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="17"/>
+      <c r="B49" s="5"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="L49" s="5"/>
+      <c r="M49" s="5"/>
+      <c r="N49" s="5"/>
+      <c r="O49" s="5"/>
+      <c r="P49" s="5"/>
+      <c r="Q49" s="5"/>
+      <c r="R49" s="5"/>
+      <c r="S49" s="5"/>
+      <c r="T49" s="5"/>
+      <c r="U49" s="5"/>
+    </row>
+    <row r="50" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
+      <c r="E50" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F50" s="5"/>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="I49" s="4"/>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="L49" s="4"/>
-      <c r="M49" s="4"/>
-      <c r="N49" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="O49" s="4"/>
-      <c r="P49" s="4"/>
-      <c r="Q49" s="4"/>
-      <c r="R49" s="4"/>
-      <c r="S49" s="4"/>
-      <c r="T49" s="4"/>
-      <c r="U49" s="4"/>
-      <c r="V49" s="4"/>
-      <c r="W49" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-      <c r="L50" s="4"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="O50" s="13"/>
-      <c r="P50" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="Q50" s="13"/>
-      <c r="R50" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="S50" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="T50" s="13" t="s">
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+      <c r="N50" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="O50" s="5"/>
+      <c r="P50" s="5"/>
+      <c r="Q50" s="5"/>
+      <c r="R50" s="5"/>
+      <c r="S50" s="5"/>
+      <c r="T50" s="5"/>
+      <c r="U50" s="5"/>
+    </row>
+    <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="17"/>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="U50" s="13" t="s">
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5" t="s">
         <v>133</v>
-      </c>
-      <c r="V50" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="W50" s="13" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="D51" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E51" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="H51" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I51" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="J51" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="K51" s="5" t="n">
-        <v>1</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
-      <c r="N51" s="5" t="s">
-        <v>136</v>
-      </c>
+      <c r="N51" s="5"/>
       <c r="O51" s="5"/>
-      <c r="P51" s="5" t="s">
-        <v>137</v>
-      </c>
+      <c r="P51" s="5"/>
       <c r="Q51" s="5"/>
-      <c r="R51" s="5" t="s">
-        <v>138</v>
-      </c>
+      <c r="R51" s="5"/>
       <c r="S51" s="5"/>
       <c r="T51" s="5"/>
       <c r="U51" s="5"/>
-      <c r="V51" s="5"/>
-      <c r="W51" s="5"/>
-    </row>
-    <row r="52" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
-      <c r="N52" s="2"/>
-      <c r="O52" s="2"/>
-      <c r="P52" s="2"/>
-      <c r="Q52" s="2"/>
-      <c r="R52" s="2"/>
-      <c r="S52" s="2"/>
-      <c r="T52" s="2"/>
-      <c r="U52" s="2"/>
-    </row>
-    <row r="53" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="B53" s="6"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6"/>
-      <c r="I53" s="6"/>
-      <c r="J53" s="6"/>
-      <c r="K53" s="6"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="6"/>
-      <c r="N53" s="6"/>
-      <c r="O53" s="6"/>
-      <c r="P53" s="6"/>
-      <c r="Q53" s="6"/>
-      <c r="R53" s="6"/>
-      <c r="S53" s="6"/>
-      <c r="T53" s="6"/>
-      <c r="U53" s="6"/>
-    </row>
-    <row r="54" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="H54" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I54" s="4"/>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="17"/>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
+      <c r="Q52" s="5"/>
+      <c r="R52" s="5"/>
+      <c r="S52" s="5"/>
+      <c r="T52" s="5"/>
+      <c r="U52" s="5"/>
+    </row>
+    <row r="53" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="17"/>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="5"/>
+      <c r="H53" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="L53" s="5"/>
+      <c r="M53" s="5"/>
+      <c r="N53" s="5"/>
+      <c r="O53" s="5"/>
+      <c r="P53" s="5"/>
+      <c r="Q53" s="5"/>
+      <c r="R53" s="5"/>
+      <c r="S53" s="5"/>
+      <c r="T53" s="5"/>
+      <c r="U53" s="5"/>
+    </row>
+    <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F54" s="5"/>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I54" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J54" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K54" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="L54" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="M54" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="N54" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="O54" s="5"/>
+      <c r="P54" s="5"/>
+      <c r="Q54" s="5"/>
+      <c r="R54" s="5"/>
+      <c r="S54" s="5"/>
+      <c r="T54" s="5"/>
+      <c r="U54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B55" s="14"/>
-      <c r="C55" s="12"/>
-      <c r="D55" s="5" t="s">
-        <v>45</v>
-      </c>
+      <c r="A55" s="17"/>
+      <c r="B55" s="5"/>
+      <c r="C55" s="5"/>
+      <c r="D55" s="5"/>
       <c r="E55" s="5"/>
       <c r="F55" s="5"/>
-      <c r="H55" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="I55" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="J55" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="K55" s="12" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="5" t="s">
-        <v>144</v>
-      </c>
+      <c r="G55" s="5"/>
+      <c r="H55" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K55" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="L55" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="M55" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="N55" s="5"/>
+      <c r="O55" s="5"/>
+      <c r="P55" s="5"/>
+      <c r="Q55" s="5"/>
+      <c r="R55" s="5"/>
+      <c r="S55" s="5"/>
+      <c r="T55" s="5"/>
+      <c r="U55" s="5"/>
+    </row>
+    <row r="56" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="17"/>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
       <c r="E56" s="5"/>
       <c r="F56" s="5"/>
-      <c r="H56" s="12" t="s">
+      <c r="G56" s="5"/>
+      <c r="H56" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K56" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="L56" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="M56" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="N56" s="5"/>
+      <c r="O56" s="5"/>
+      <c r="P56" s="5"/>
+      <c r="Q56" s="5"/>
+      <c r="R56" s="5"/>
+      <c r="S56" s="5"/>
+      <c r="T56" s="5"/>
+      <c r="U56" s="5"/>
+    </row>
+    <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
+      <c r="L57" s="2"/>
+      <c r="M57" s="2"/>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" s="2"/>
+      <c r="Q57" s="2"/>
+      <c r="R57" s="2"/>
+      <c r="S57" s="2"/>
+      <c r="T57" s="2"/>
+      <c r="U57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
+      <c r="L58" s="6"/>
+      <c r="M58" s="6"/>
+      <c r="N58" s="6"/>
+      <c r="O58" s="6"/>
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="6"/>
+      <c r="T58" s="6"/>
+      <c r="U58" s="6"/>
+      <c r="V58" s="6"/>
+      <c r="W58" s="6"/>
+    </row>
+    <row r="59" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="I59" s="4"/>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="O59" s="4"/>
+      <c r="P59" s="4"/>
+      <c r="Q59" s="4"/>
+      <c r="R59" s="4"/>
+      <c r="S59" s="4"/>
+      <c r="T59" s="4"/>
+      <c r="U59" s="4"/>
+      <c r="V59" s="4"/>
+      <c r="W59" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+      <c r="H60" s="4"/>
+      <c r="I60" s="4"/>
+      <c r="J60" s="4"/>
+      <c r="K60" s="4"/>
+      <c r="L60" s="4"/>
+      <c r="M60" s="4"/>
+      <c r="N60" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="O60" s="18"/>
+      <c r="P60" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q60" s="18"/>
+      <c r="R60" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="S60" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="T60" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="U60" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="V60" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="W60" s="18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="F61" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="G61" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="H61" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I61" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J61" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="K61" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L61" s="5"/>
+      <c r="M61" s="5"/>
+      <c r="N61" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="O61" s="5"/>
+      <c r="P61" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q61" s="5"/>
+      <c r="R61" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="S61" s="5"/>
+      <c r="T61" s="5"/>
+      <c r="U61" s="5"/>
+      <c r="V61" s="5"/>
+      <c r="W61" s="5"/>
+    </row>
+    <row r="62" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+      <c r="I62" s="2"/>
+      <c r="J62" s="2"/>
+      <c r="K62" s="2"/>
+      <c r="L62" s="2"/>
+      <c r="M62" s="2"/>
+      <c r="N62" s="2"/>
+      <c r="O62" s="2"/>
+      <c r="P62" s="2"/>
+      <c r="Q62" s="2"/>
+      <c r="R62" s="2"/>
+      <c r="S62" s="2"/>
+      <c r="T62" s="2"/>
+      <c r="U62" s="2"/>
+    </row>
+    <row r="63" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B63" s="6"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
+      <c r="G63" s="6"/>
+      <c r="H63" s="6"/>
+      <c r="I63" s="6"/>
+      <c r="J63" s="6"/>
+      <c r="K63" s="6"/>
+      <c r="L63" s="6"/>
+      <c r="M63" s="6"/>
+      <c r="N63" s="6"/>
+      <c r="O63" s="6"/>
+      <c r="P63" s="6"/>
+      <c r="Q63" s="6"/>
+      <c r="R63" s="6"/>
+      <c r="S63" s="6"/>
+      <c r="T63" s="6"/>
+      <c r="U63" s="6"/>
+    </row>
+    <row r="64" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="H64" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+    </row>
+    <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B65" s="19"/>
+      <c r="C65" s="17"/>
+      <c r="D65" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="I56" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="J56" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="K56" s="12" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12" t="n">
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="H65" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="I65" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="J65" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="K65" s="17" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="E66" s="5"/>
+      <c r="F66" s="5"/>
+      <c r="H66" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="I66" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="J66" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="K66" s="17" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B57" s="15"/>
-      <c r="C57" s="12"/>
-      <c r="D57" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="E57" s="5"/>
-      <c r="F57" s="5"/>
-      <c r="H57" s="16"/>
-      <c r="I57" s="16"/>
-      <c r="J57" s="16"/>
-      <c r="K57" s="16"/>
-    </row>
-    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="12" t="n">
+      <c r="B67" s="20"/>
+      <c r="C67" s="17"/>
+      <c r="D67" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="H67" s="21"/>
+      <c r="I67" s="21"/>
+      <c r="J67" s="21"/>
+      <c r="K67" s="21"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="E58" s="5"/>
-      <c r="F58" s="5"/>
-      <c r="H58" s="16"/>
-      <c r="I58" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="J58" s="5"/>
-      <c r="K58" s="16"/>
-    </row>
-    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12" t="n">
+      <c r="B68" s="22"/>
+      <c r="C68" s="22"/>
+      <c r="D68" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="H68" s="21"/>
+      <c r="I68" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="J68" s="5"/>
+      <c r="K68" s="21"/>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
-    </row>
-    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="12" t="n">
+      <c r="B69" s="22"/>
+      <c r="C69" s="17"/>
+      <c r="D69" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
+      <c r="I69" s="5"/>
+      <c r="J69" s="5"/>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-    </row>
-    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="12" t="n">
+      <c r="B70" s="20"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="B61" s="18"/>
-      <c r="C61" s="12"/>
-      <c r="D61" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="E61" s="5"/>
-      <c r="F61" s="5"/>
-    </row>
-    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="12" t="n">
+      <c r="B71" s="23"/>
+      <c r="C71" s="17"/>
+      <c r="D71" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B62" s="18"/>
-      <c r="C62" s="18"/>
-      <c r="D62" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-    </row>
-    <row r="63" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
-      <c r="H63" s="2"/>
-      <c r="I63" s="2"/>
-      <c r="J63" s="2"/>
-      <c r="K63" s="2"/>
-      <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
-      <c r="P63" s="2"/>
-      <c r="Q63" s="2"/>
-      <c r="R63" s="2"/>
-      <c r="S63" s="2"/>
-      <c r="T63" s="2"/>
-      <c r="U63" s="2"/>
+      <c r="B72" s="23"/>
+      <c r="C72" s="23"/>
+      <c r="D72" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E72" s="5"/>
+      <c r="F72" s="5"/>
+    </row>
+    <row r="73" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
+      <c r="G73" s="2"/>
+      <c r="H73" s="2"/>
+      <c r="I73" s="2"/>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
+      <c r="L73" s="2"/>
+      <c r="M73" s="2"/>
+      <c r="N73" s="2"/>
+      <c r="O73" s="2"/>
+      <c r="P73" s="2"/>
+      <c r="Q73" s="2"/>
+      <c r="R73" s="2"/>
+      <c r="S73" s="2"/>
+      <c r="T73" s="2"/>
+      <c r="U73" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="153">
+  <mergeCells count="188">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -3227,10 +3707,12 @@
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="G5:N5"/>
     <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="R5:U5"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="G6:N6"/>
     <mergeCell ref="O6:Q8"/>
+    <mergeCell ref="R6:U8"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="G7:N7"/>
@@ -3241,6 +3723,7 @@
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="G9:N9"/>
     <mergeCell ref="O9:Q15"/>
+    <mergeCell ref="R9:U15"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="G10:N10"/>
@@ -3259,119 +3742,151 @@
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="G15:N15"/>
-    <mergeCell ref="A16:U16"/>
-    <mergeCell ref="A17:U17"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:N16"/>
+    <mergeCell ref="O16:Q25"/>
+    <mergeCell ref="R16:U25"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:N17"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="G18:N18"/>
-    <mergeCell ref="O18:Q18"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="G19:N19"/>
-    <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="A20:U20"/>
-    <mergeCell ref="A21:U21"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="G20:N20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="G21:N21"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="G22:N22"/>
-    <mergeCell ref="O22:Q22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="G23:N23"/>
-    <mergeCell ref="O23:Q23"/>
-    <mergeCell ref="A24:U24"/>
-    <mergeCell ref="A25:U25"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:N24"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="G25:N25"/>
     <mergeCell ref="A26:U26"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="N27:U27"/>
-    <mergeCell ref="A28:A32"/>
-    <mergeCell ref="B28:D32"/>
-    <mergeCell ref="E28:G39"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="K28:M28"/>
-    <mergeCell ref="N28:U32"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="K29:M29"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="K30:M30"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="K31:M31"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="A33:A39"/>
-    <mergeCell ref="B33:D39"/>
-    <mergeCell ref="H33:J33"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="N33:U39"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="K34:M34"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="K35:M35"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="A27:U27"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="G28:N28"/>
+    <mergeCell ref="O28:Q28"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="G29:N29"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="A30:U30"/>
+    <mergeCell ref="A31:U31"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="G32:N32"/>
+    <mergeCell ref="O32:Q32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="G33:N33"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="A34:U34"/>
+    <mergeCell ref="A35:U35"/>
+    <mergeCell ref="A36:U36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E37:G37"/>
     <mergeCell ref="H37:J37"/>
     <mergeCell ref="K37:M37"/>
+    <mergeCell ref="N37:U37"/>
+    <mergeCell ref="A38:A42"/>
+    <mergeCell ref="B38:D42"/>
+    <mergeCell ref="E38:G49"/>
     <mergeCell ref="H38:J38"/>
     <mergeCell ref="K38:M38"/>
+    <mergeCell ref="N38:U42"/>
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="K39:M39"/>
-    <mergeCell ref="A40:A43"/>
-    <mergeCell ref="B40:D43"/>
-    <mergeCell ref="E40:G43"/>
     <mergeCell ref="H40:J40"/>
     <mergeCell ref="K40:M40"/>
-    <mergeCell ref="N40:U43"/>
     <mergeCell ref="H41:J41"/>
     <mergeCell ref="K41:M41"/>
     <mergeCell ref="H42:J42"/>
     <mergeCell ref="K42:M42"/>
+    <mergeCell ref="A43:A49"/>
+    <mergeCell ref="B43:D49"/>
     <mergeCell ref="H43:J43"/>
     <mergeCell ref="K43:M43"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B44:D46"/>
-    <mergeCell ref="E44:G46"/>
+    <mergeCell ref="N43:U49"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="K44:M44"/>
-    <mergeCell ref="N44:U46"/>
     <mergeCell ref="H45:J45"/>
     <mergeCell ref="K45:M45"/>
     <mergeCell ref="H46:J46"/>
     <mergeCell ref="K46:M46"/>
-    <mergeCell ref="A47:U47"/>
-    <mergeCell ref="A48:W48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="B49:D50"/>
-    <mergeCell ref="E49:G50"/>
-    <mergeCell ref="H49:J50"/>
-    <mergeCell ref="K49:M50"/>
-    <mergeCell ref="N49:O49"/>
-    <mergeCell ref="P49:V49"/>
-    <mergeCell ref="N50:O50"/>
-    <mergeCell ref="P50:Q50"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="H47:J47"/>
+    <mergeCell ref="K47:M47"/>
+    <mergeCell ref="H48:J48"/>
+    <mergeCell ref="K48:M48"/>
+    <mergeCell ref="H49:J49"/>
+    <mergeCell ref="K49:M49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="B50:D53"/>
+    <mergeCell ref="E50:G53"/>
+    <mergeCell ref="H50:J50"/>
+    <mergeCell ref="K50:M50"/>
+    <mergeCell ref="N50:U53"/>
     <mergeCell ref="H51:J51"/>
     <mergeCell ref="K51:M51"/>
-    <mergeCell ref="N51:O51"/>
-    <mergeCell ref="P51:Q51"/>
-    <mergeCell ref="R51:W51"/>
-    <mergeCell ref="A52:U52"/>
-    <mergeCell ref="A53:U53"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="H54:K54"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="D56:F56"/>
-    <mergeCell ref="D57:F57"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="I58:J59"/>
-    <mergeCell ref="D59:F59"/>
-    <mergeCell ref="D60:F60"/>
-    <mergeCell ref="D61:F61"/>
-    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="H52:J52"/>
+    <mergeCell ref="K52:M52"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="K53:M53"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:D56"/>
+    <mergeCell ref="E54:G56"/>
+    <mergeCell ref="H54:J54"/>
+    <mergeCell ref="K54:M54"/>
+    <mergeCell ref="N54:U56"/>
+    <mergeCell ref="H55:J55"/>
+    <mergeCell ref="K55:M55"/>
+    <mergeCell ref="H56:J56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="A57:U57"/>
+    <mergeCell ref="A58:W58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="B59:D60"/>
+    <mergeCell ref="E59:G60"/>
+    <mergeCell ref="H59:J60"/>
+    <mergeCell ref="K59:M60"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="P59:V59"/>
+    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="P60:Q60"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="K61:M61"/>
+    <mergeCell ref="N61:O61"/>
+    <mergeCell ref="P61:Q61"/>
+    <mergeCell ref="R61:W61"/>
+    <mergeCell ref="A62:U62"/>
     <mergeCell ref="A63:U63"/>
+    <mergeCell ref="D64:F64"/>
+    <mergeCell ref="H64:K64"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="D67:F67"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="I68:J69"/>
+    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="D70:F70"/>
+    <mergeCell ref="D71:F71"/>
+    <mergeCell ref="D72:F72"/>
+    <mergeCell ref="A73:U73"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.25 ] - roulette driver schematic was added.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -759,7 +759,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -796,7 +796,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -808,10 +808,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -820,15 +816,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1889,10 +1877,10 @@
       </c>
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
-      <c r="U9" s="12"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="n">
@@ -1920,10 +1908,10 @@
       <c r="O10" s="11"/>
       <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
-      <c r="U10" s="12"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="n">
@@ -1951,10 +1939,10 @@
       <c r="O11" s="11"/>
       <c r="P11" s="11"/>
       <c r="Q11" s="11"/>
-      <c r="R11" s="12"/>
-      <c r="S11" s="12"/>
-      <c r="T11" s="12"/>
-      <c r="U11" s="12"/>
+      <c r="R11" s="10"/>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="n">
@@ -1982,10 +1970,10 @@
       <c r="O12" s="11"/>
       <c r="P12" s="11"/>
       <c r="Q12" s="11"/>
-      <c r="R12" s="12"/>
-      <c r="S12" s="12"/>
-      <c r="T12" s="12"/>
-      <c r="U12" s="12"/>
+      <c r="R12" s="10"/>
+      <c r="S12" s="10"/>
+      <c r="T12" s="10"/>
+      <c r="U12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="n">
@@ -2013,10 +2001,10 @@
       <c r="O13" s="11"/>
       <c r="P13" s="11"/>
       <c r="Q13" s="11"/>
-      <c r="R13" s="12"/>
-      <c r="S13" s="12"/>
-      <c r="T13" s="12"/>
-      <c r="U13" s="12"/>
+      <c r="R13" s="10"/>
+      <c r="S13" s="10"/>
+      <c r="T13" s="10"/>
+      <c r="U13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="n">
@@ -2044,10 +2032,10 @@
       <c r="O14" s="11"/>
       <c r="P14" s="11"/>
       <c r="Q14" s="11"/>
-      <c r="R14" s="12"/>
-      <c r="S14" s="12"/>
-      <c r="T14" s="12"/>
-      <c r="U14" s="12"/>
+      <c r="R14" s="10"/>
+      <c r="S14" s="10"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="n">
@@ -2075,324 +2063,324 @@
       <c r="O15" s="11"/>
       <c r="P15" s="11"/>
       <c r="Q15" s="11"/>
-      <c r="R15" s="12"/>
-      <c r="S15" s="12"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="12"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="n">
+      <c r="A16" s="12" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14" t="s">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14" t="s">
+      <c r="F16" s="13"/>
+      <c r="G16" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="H16" s="14"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14" t="s">
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="13"/>
+      <c r="N16" s="13"/>
+      <c r="O16" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="14"/>
-      <c r="R16" s="15" t="s">
+      <c r="P16" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="R16" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15"/>
-      <c r="U16" s="15"/>
+      <c r="S16" s="13"/>
+      <c r="T16" s="13"/>
+      <c r="U16" s="13"/>
     </row>
     <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14" t="s">
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14" t="s">
+      <c r="F17" s="13"/>
+      <c r="G17" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
-      <c r="Q17" s="14"/>
-      <c r="R17" s="15"/>
-      <c r="S17" s="15"/>
-      <c r="T17" s="15"/>
-      <c r="U17" s="15"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="S17" s="13"/>
+      <c r="T17" s="13"/>
+      <c r="U17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="n">
+      <c r="A18" s="12" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14" t="s">
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14" t="s">
+      <c r="F18" s="13"/>
+      <c r="G18" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="15"/>
-      <c r="T18" s="15"/>
-      <c r="U18" s="15"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="13"/>
+      <c r="U18" s="13"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14" t="s">
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14" t="s">
+      <c r="F19" s="13"/>
+      <c r="G19" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="14"/>
-      <c r="I19" s="14"/>
-      <c r="J19" s="14"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
-      <c r="M19" s="14"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="14"/>
-      <c r="P19" s="14"/>
-      <c r="Q19" s="14"/>
-      <c r="R19" s="15"/>
-      <c r="S19" s="15"/>
-      <c r="T19" s="15"/>
-      <c r="U19" s="15"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="13"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="13"/>
+      <c r="U19" s="13"/>
     </row>
     <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="n">
+      <c r="A20" s="12" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14" t="s">
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14" t="s">
+      <c r="F20" s="13"/>
+      <c r="G20" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="14"/>
-      <c r="R20" s="15"/>
-      <c r="S20" s="15"/>
-      <c r="T20" s="15"/>
-      <c r="U20" s="15"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
+      <c r="R20" s="13"/>
+      <c r="S20" s="13"/>
+      <c r="T20" s="13"/>
+      <c r="U20" s="13"/>
     </row>
     <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14" t="s">
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14" t="s">
+      <c r="F21" s="13"/>
+      <c r="G21" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="14"/>
-      <c r="P21" s="14"/>
-      <c r="Q21" s="14"/>
-      <c r="R21" s="15"/>
-      <c r="S21" s="15"/>
-      <c r="T21" s="15"/>
-      <c r="U21" s="15"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="13"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="13"/>
     </row>
     <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="n">
+      <c r="A22" s="12" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14" t="s">
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14" t="s">
+      <c r="F22" s="13"/>
+      <c r="G22" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
-      <c r="Q22" s="14"/>
-      <c r="R22" s="15"/>
-      <c r="S22" s="15"/>
-      <c r="T22" s="15"/>
-      <c r="U22" s="15"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="13"/>
+      <c r="R22" s="13"/>
+      <c r="S22" s="13"/>
+      <c r="T22" s="13"/>
+      <c r="U22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14" t="s">
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14" t="s">
+      <c r="F23" s="13"/>
+      <c r="G23" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-      <c r="M23" s="14"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="14"/>
-      <c r="P23" s="14"/>
-      <c r="Q23" s="14"/>
-      <c r="R23" s="15"/>
-      <c r="S23" s="15"/>
-      <c r="T23" s="15"/>
-      <c r="U23" s="15"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="13"/>
+      <c r="R23" s="13"/>
+      <c r="S23" s="13"/>
+      <c r="T23" s="13"/>
+      <c r="U23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="n">
+      <c r="A24" s="12" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14" t="s">
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="14" t="s">
+      <c r="F24" s="13"/>
+      <c r="G24" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
-      <c r="R24" s="15"/>
-      <c r="S24" s="15"/>
-      <c r="T24" s="15"/>
-      <c r="U24" s="15"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="13"/>
+      <c r="R24" s="13"/>
+      <c r="S24" s="13"/>
+      <c r="T24" s="13"/>
+      <c r="U24" s="13"/>
     </row>
     <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14" t="s">
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="14"/>
-      <c r="G25" s="14" t="s">
+      <c r="F25" s="13"/>
+      <c r="G25" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="H25" s="14"/>
-      <c r="I25" s="14"/>
-      <c r="J25" s="14"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="14"/>
-      <c r="P25" s="14"/>
-      <c r="Q25" s="14"/>
-      <c r="R25" s="15"/>
-      <c r="S25" s="15"/>
-      <c r="T25" s="15"/>
-      <c r="U25" s="15"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
+      <c r="O25" s="13"/>
+      <c r="P25" s="13"/>
+      <c r="Q25" s="13"/>
+      <c r="R25" s="13"/>
+      <c r="S25" s="13"/>
+      <c r="T25" s="13"/>
+      <c r="U25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2"/>
@@ -2630,29 +2618,29 @@
       <c r="U34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="16"/>
-      <c r="Q35" s="16"/>
-      <c r="R35" s="16"/>
-      <c r="S35" s="16"/>
-      <c r="T35" s="16"/>
-      <c r="U35" s="16"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="14"/>
+      <c r="M35" s="14"/>
+      <c r="N35" s="14"/>
+      <c r="O35" s="14"/>
+      <c r="P35" s="14"/>
+      <c r="Q35" s="14"/>
+      <c r="R35" s="14"/>
+      <c r="S35" s="14"/>
+      <c r="T35" s="14"/>
+      <c r="U35" s="14"/>
     </row>
     <row r="36" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
@@ -2715,7 +2703,7 @@
       <c r="U37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="17" t="n">
+      <c r="A38" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B38" s="5" t="s">
@@ -2754,7 +2742,7 @@
       <c r="U38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="17"/>
+      <c r="A39" s="9"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
@@ -2781,7 +2769,7 @@
       <c r="U39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="17"/>
+      <c r="A40" s="9"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
@@ -2808,7 +2796,7 @@
       <c r="U40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17"/>
+      <c r="A41" s="9"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -2835,7 +2823,7 @@
       <c r="U41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17"/>
+      <c r="A42" s="9"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
@@ -2862,7 +2850,7 @@
       <c r="U42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17" t="n">
+      <c r="A43" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B43" s="5" t="s">
@@ -2895,7 +2883,7 @@
       <c r="U43" s="5"/>
     </row>
     <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17"/>
+      <c r="A44" s="9"/>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
@@ -2922,7 +2910,7 @@
       <c r="U44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="17"/>
+      <c r="A45" s="9"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
@@ -2949,7 +2937,7 @@
       <c r="U45" s="5"/>
     </row>
     <row r="46" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="17"/>
+      <c r="A46" s="9"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
@@ -2976,7 +2964,7 @@
       <c r="U46" s="5"/>
     </row>
     <row r="47" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="17"/>
+      <c r="A47" s="9"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
@@ -3003,7 +2991,7 @@
       <c r="U47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="17"/>
+      <c r="A48" s="9"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
@@ -3030,7 +3018,7 @@
       <c r="U48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="17"/>
+      <c r="A49" s="9"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
@@ -3057,7 +3045,7 @@
       <c r="U49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="17" t="n">
+      <c r="A50" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B50" s="5" t="s">
@@ -3092,7 +3080,7 @@
       <c r="U50" s="5"/>
     </row>
     <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="17"/>
+      <c r="A51" s="9"/>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
@@ -3119,7 +3107,7 @@
       <c r="U51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="17"/>
+      <c r="A52" s="9"/>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
@@ -3146,7 +3134,7 @@
       <c r="U52" s="5"/>
     </row>
     <row r="53" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="17"/>
+      <c r="A53" s="9"/>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
       <c r="D53" s="5"/>
@@ -3173,7 +3161,7 @@
       <c r="U53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="17" t="n">
+      <c r="A54" s="9" t="n">
         <v>4</v>
       </c>
       <c r="B54" s="5" t="s">
@@ -3220,7 +3208,7 @@
       <c r="U54" s="5"/>
     </row>
     <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="17"/>
+      <c r="A55" s="9"/>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
@@ -3255,7 +3243,7 @@
       <c r="U55" s="5"/>
     </row>
     <row r="56" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="17"/>
+      <c r="A56" s="9"/>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
@@ -3392,35 +3380,35 @@
       <c r="K60" s="4"/>
       <c r="L60" s="4"/>
       <c r="M60" s="4"/>
-      <c r="N60" s="18" t="s">
+      <c r="N60" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="O60" s="18"/>
-      <c r="P60" s="18" t="s">
+      <c r="O60" s="15"/>
+      <c r="P60" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="Q60" s="18"/>
-      <c r="R60" s="18" t="s">
+      <c r="Q60" s="15"/>
+      <c r="R60" s="15" t="s">
         <v>162</v>
       </c>
-      <c r="S60" s="18" t="s">
+      <c r="S60" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="T60" s="18" t="s">
+      <c r="T60" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="U60" s="18" t="s">
+      <c r="U60" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="V60" s="18" t="s">
+      <c r="V60" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="W60" s="18" t="s">
+      <c r="W60" s="15" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="17" t="n">
+      <c r="A61" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B61" s="5" t="s">
@@ -3543,93 +3531,93 @@
       <c r="K64" s="4"/>
     </row>
     <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="17" t="n">
+      <c r="A65" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B65" s="19"/>
-      <c r="C65" s="17"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="9"/>
       <c r="D65" s="5" t="s">
         <v>45</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
-      <c r="H65" s="17" t="s">
+      <c r="H65" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="I65" s="17" t="s">
+      <c r="I65" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="J65" s="17" t="s">
+      <c r="J65" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="K65" s="17" t="s">
+      <c r="K65" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="17" t="n">
+      <c r="A66" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B66" s="19"/>
-      <c r="C66" s="19"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="16"/>
       <c r="D66" s="5" t="s">
         <v>176</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
-      <c r="H66" s="17" t="s">
+      <c r="H66" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="I66" s="17" t="s">
+      <c r="I66" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="J66" s="17" t="s">
+      <c r="J66" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="K66" s="17" t="s">
+      <c r="K66" s="9" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="17" t="n">
+      <c r="A67" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B67" s="20"/>
-      <c r="C67" s="17"/>
+      <c r="B67" s="17"/>
+      <c r="C67" s="9"/>
       <c r="D67" s="5" t="s">
         <v>183</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
-      <c r="H67" s="21"/>
-      <c r="I67" s="21"/>
-      <c r="J67" s="21"/>
-      <c r="K67" s="21"/>
+      <c r="H67" s="18"/>
+      <c r="I67" s="18"/>
+      <c r="J67" s="18"/>
+      <c r="K67" s="18"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="17" t="n">
+      <c r="A68" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B68" s="22"/>
-      <c r="C68" s="22"/>
+      <c r="B68" s="19"/>
+      <c r="C68" s="19"/>
       <c r="D68" s="5" t="s">
         <v>177</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
-      <c r="H68" s="21"/>
+      <c r="H68" s="18"/>
       <c r="I68" s="5" t="s">
         <v>184</v>
       </c>
       <c r="J68" s="5"/>
-      <c r="K68" s="21"/>
+      <c r="K68" s="18"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="17" t="n">
+      <c r="A69" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B69" s="22"/>
-      <c r="C69" s="17"/>
+      <c r="B69" s="19"/>
+      <c r="C69" s="9"/>
       <c r="D69" s="5" t="s">
         <v>181</v>
       </c>
@@ -3639,11 +3627,11 @@
       <c r="J69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="17" t="n">
+      <c r="A70" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B70" s="20"/>
-      <c r="C70" s="20"/>
+      <c r="B70" s="17"/>
+      <c r="C70" s="17"/>
       <c r="D70" s="5" t="s">
         <v>179</v>
       </c>
@@ -3651,11 +3639,11 @@
       <c r="F70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="17" t="n">
+      <c r="A71" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B71" s="23"/>
-      <c r="C71" s="17"/>
+      <c r="B71" s="20"/>
+      <c r="C71" s="9"/>
       <c r="D71" s="5" t="s">
         <v>182</v>
       </c>
@@ -3663,11 +3651,11 @@
       <c r="F71" s="5"/>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="17" t="n">
+      <c r="A72" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B72" s="23"/>
-      <c r="C72" s="23"/>
+      <c r="B72" s="20"/>
+      <c r="C72" s="20"/>
       <c r="D72" s="5" t="s">
         <v>178</v>
       </c>

</xml_diff>

<commit_message>
[ Version 0.0.25.1 ] - excel GPIOs was updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="178">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -239,7 +239,7 @@
     <t xml:space="preserve">OUT_ROULETTE_EN1</t>
   </si>
   <si>
-    <t xml:space="preserve">GPIO21</t>
+    <t xml:space="preserve">GPIO16</t>
   </si>
   <si>
     <t xml:space="preserve">DO for roulette R1 motor driver enable pin – enable 1.</t>
@@ -248,85 +248,64 @@
     <t xml:space="preserve">ROULETTE</t>
   </si>
   <si>
-    <t xml:space="preserve">TEMPORARY!</t>
-  </si>
-  <si>
     <t xml:space="preserve">OUT_ROULETTE_EN2</t>
   </si>
   <si>
+    <t xml:space="preserve">GPIO17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R2 motor driver enable pin – enable 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 1 – direction 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT_ROULETTE_DIR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 2 – direction 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESO1</t>
+  </si>
+  <si>
     <t xml:space="preserve">GPIO22</t>
   </si>
   <si>
-    <t xml:space="preserve">DO for roulette R2 motor driver enable pin – enable 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_DIR1_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 1 – direction 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_DIR1_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R1 motor driver direction bit 2 – direction 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_DIR2_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R2 motor driver direction bit 1 – direction 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OUT_ROULETTE_DIR2_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R2 motor driver direction bit 2 – direction 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_ESO1</t>
+    <t xml:space="preserve">DI for roulette R1 open position end switches – end switch open 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESO2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPIO25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DI for roulette R2 open position end switches – end switch open 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESC1</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO23</t>
   </si>
   <si>
-    <t xml:space="preserve">DI for roulette R1 open position end switches – end switch open 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_ESO2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R2 open position end switches – end switch open 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_ESC1</t>
+    <t xml:space="preserve">DI for roulette R1 close position end switches – end switch close 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN_ROULETTE_ESC2</t>
   </si>
   <si>
     <t xml:space="preserve">GPIO26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R1 close position end switches – end switch close 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_ESC2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO27</t>
   </si>
   <si>
     <t xml:space="preserve">DI for roulette R2 close position end switches – end switch close 2.</t>
@@ -1620,7 +1599,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W73"/>
+  <dimension ref="A1:W71"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2096,9 +2075,7 @@
       </c>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="13" t="s">
-        <v>75</v>
-      </c>
+      <c r="R16" s="13"/>
       <c r="S16" s="13"/>
       <c r="T16" s="13"/>
       <c r="U16" s="13"/>
@@ -2108,16 +2085,16 @@
         <v>12</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H17" s="13"/>
       <c r="I17" s="13"/>
@@ -2139,16 +2116,16 @@
         <v>13</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F18" s="13"/>
       <c r="G18" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
@@ -2170,16 +2147,16 @@
         <v>14</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F19" s="13"/>
       <c r="G19" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H19" s="13"/>
       <c r="I19" s="13"/>
@@ -2201,16 +2178,16 @@
         <v>15</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F20" s="13"/>
       <c r="G20" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
@@ -2232,16 +2209,16 @@
         <v>16</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
       <c r="E21" s="13" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H21" s="13"/>
       <c r="I21" s="13"/>
@@ -2263,16 +2240,16 @@
         <v>17</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H22" s="13"/>
       <c r="I22" s="13"/>
@@ -2294,16 +2271,16 @@
         <v>18</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H23" s="13"/>
       <c r="I23" s="13"/>
@@ -2320,419 +2297,411 @@
       <c r="T23" s="13"/>
       <c r="U23" s="13"/>
     </row>
-    <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="13" t="s">
+    <row r="24" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2"/>
+      <c r="T24" s="2"/>
+      <c r="U24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6"/>
+      <c r="K25" s="6"/>
+      <c r="L25" s="6"/>
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6"/>
+      <c r="R25" s="6"/>
+      <c r="S25" s="6"/>
+      <c r="T25" s="6"/>
+      <c r="U25" s="6"/>
+    </row>
+    <row r="26" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P26" s="4"/>
+      <c r="Q26" s="4"/>
+    </row>
+    <row r="27" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13" t="s">
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13" t="s">
+      <c r="F27" s="11"/>
+      <c r="G27" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="13"/>
-      <c r="R24" s="13"/>
-      <c r="S24" s="13"/>
-      <c r="T24" s="13"/>
-      <c r="U24" s="13"/>
-    </row>
-    <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="13" t="s">
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="11"/>
+      <c r="M27" s="11"/>
+      <c r="N27" s="11"/>
+      <c r="O27" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="P27" s="11"/>
+      <c r="Q27" s="11"/>
+    </row>
+    <row r="28" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
+      <c r="O28" s="2"/>
+      <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
+      <c r="S28" s="2"/>
+      <c r="T28" s="2"/>
+      <c r="U28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13" t="s">
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+      <c r="R29" s="6"/>
+      <c r="S29" s="6"/>
+      <c r="T29" s="6"/>
+      <c r="U29" s="6"/>
+    </row>
+    <row r="30" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="4"/>
+      <c r="O30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P30" s="4"/>
+      <c r="Q30" s="4"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="H25" s="13"/>
-      <c r="I25" s="13"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="13"/>
-      <c r="M25" s="13"/>
-      <c r="N25" s="13"/>
-      <c r="O25" s="13"/>
-      <c r="P25" s="13"/>
-      <c r="Q25" s="13"/>
-      <c r="R25" s="13"/>
-      <c r="S25" s="13"/>
-      <c r="T25" s="13"/>
-      <c r="U25" s="13"/>
-    </row>
-    <row r="26" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="2"/>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2"/>
-      <c r="U26" s="2"/>
-    </row>
-    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
+      <c r="F31" s="11"/>
+      <c r="G31" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
-      <c r="M27" s="6"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="6"/>
-      <c r="P27" s="6"/>
-      <c r="Q27" s="6"/>
-      <c r="R27" s="6"/>
-      <c r="S27" s="6"/>
-      <c r="T27" s="6"/>
-      <c r="U27" s="6"/>
-    </row>
-    <row r="28" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+      <c r="J31" s="11"/>
+      <c r="K31" s="11"/>
+      <c r="L31" s="11"/>
+      <c r="M31" s="11"/>
+      <c r="N31" s="11"/>
+      <c r="O31" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="P31" s="11"/>
+      <c r="Q31" s="11"/>
+    </row>
+    <row r="32" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+      <c r="O32" s="2"/>
+      <c r="P32" s="2"/>
+      <c r="Q32" s="2"/>
+      <c r="R32" s="2"/>
+      <c r="S32" s="2"/>
+      <c r="T32" s="2"/>
+      <c r="U32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
+      <c r="O33" s="14"/>
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="14"/>
+      <c r="T33" s="14"/>
+      <c r="U33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="6"/>
+      <c r="L34" s="6"/>
+      <c r="M34" s="6"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="6"/>
+      <c r="P34" s="6"/>
+      <c r="Q34" s="6"/>
+      <c r="R34" s="6"/>
+      <c r="S34" s="6"/>
+      <c r="T34" s="6"/>
+      <c r="U34" s="6"/>
+    </row>
+    <row r="35" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B35" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4" t="s">
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-      <c r="M28" s="4"/>
-      <c r="N28" s="4"/>
-      <c r="O28" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="P28" s="4"/>
-      <c r="Q28" s="4"/>
-    </row>
-    <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="n">
+      <c r="O35" s="4"/>
+      <c r="P35" s="4"/>
+      <c r="Q35" s="4"/>
+      <c r="R35" s="4"/>
+      <c r="S35" s="4"/>
+      <c r="T35" s="4"/>
+      <c r="U35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B29" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
-      <c r="O29" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="P29" s="11"/>
-      <c r="Q29" s="11"/>
-    </row>
-    <row r="30" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-    </row>
-    <row r="31" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
-      <c r="Q31" s="6"/>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
-      <c r="T31" s="6"/>
-      <c r="U31" s="6"/>
-    </row>
-    <row r="32" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4"/>
-      <c r="O32" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>108</v>
-      </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11" t="s">
+      <c r="B36" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11" t="s">
+      <c r="C36" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="H33" s="11"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11"/>
-      <c r="O33" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="P33" s="11"/>
-      <c r="Q33" s="11"/>
-    </row>
-    <row r="34" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
-      <c r="P34" s="2"/>
-      <c r="Q34" s="2"/>
-      <c r="R34" s="2"/>
-      <c r="S34" s="2"/>
-      <c r="T34" s="2"/>
-      <c r="U34" s="2"/>
-    </row>
-    <row r="35" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="s">
+      <c r="D36" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="14"/>
-      <c r="K35" s="14"/>
-      <c r="L35" s="14"/>
-      <c r="M35" s="14"/>
-      <c r="N35" s="14"/>
-      <c r="O35" s="14"/>
-      <c r="P35" s="14"/>
-      <c r="Q35" s="14"/>
-      <c r="R35" s="14"/>
-      <c r="S35" s="14"/>
-      <c r="T35" s="14"/>
-      <c r="U35" s="14"/>
-    </row>
-    <row r="36" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="s">
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="6"/>
-      <c r="Q36" s="6"/>
-      <c r="R36" s="6"/>
-      <c r="S36" s="6"/>
-      <c r="T36" s="6"/>
-      <c r="U36" s="6"/>
-    </row>
-    <row r="37" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4" t="s">
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4" t="s">
+      <c r="L36" s="5"/>
+      <c r="M36" s="5"/>
+      <c r="N36" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4" t="s">
+      <c r="O36" s="5"/>
+      <c r="P36" s="5"/>
+      <c r="Q36" s="5"/>
+      <c r="R36" s="5"/>
+      <c r="S36" s="5"/>
+      <c r="T36" s="5"/>
+      <c r="U36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="9"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="L37" s="4"/>
-      <c r="M37" s="4"/>
-      <c r="N37" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="O37" s="4"/>
-      <c r="P37" s="4"/>
-      <c r="Q37" s="4"/>
-      <c r="R37" s="4"/>
-      <c r="S37" s="4"/>
-      <c r="T37" s="4"/>
-      <c r="U37" s="4"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+      <c r="S37" s="5"/>
+      <c r="T37" s="5"/>
+      <c r="U37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>118</v>
-      </c>
+      <c r="A38" s="9"/>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
-      <c r="N38" s="5" t="s">
-        <v>121</v>
-      </c>
+      <c r="N38" s="5"/>
       <c r="O38" s="5"/>
       <c r="P38" s="5"/>
       <c r="Q38" s="5"/>
@@ -2750,12 +2719,12 @@
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
       <c r="K39" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -2777,12 +2746,12 @@
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
@@ -2796,24 +2765,30 @@
       <c r="U40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9"/>
-      <c r="B41" s="5"/>
+      <c r="A41" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>123</v>
+      </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>126</v>
+        <v>112</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5" t="s">
-        <v>127</v>
+        <v>113</v>
       </c>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
-      <c r="N41" s="5"/>
+      <c r="N41" s="5" t="s">
+        <v>124</v>
+      </c>
       <c r="O41" s="5"/>
       <c r="P41" s="5"/>
       <c r="Q41" s="5"/>
@@ -2831,12 +2806,12 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
@@ -2850,30 +2825,24 @@
       <c r="U42" s="5"/>
     </row>
     <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>130</v>
-      </c>
+      <c r="A43" s="9"/>
+      <c r="B43" s="5"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
-      <c r="N43" s="5" t="s">
-        <v>131</v>
-      </c>
+      <c r="N43" s="5"/>
       <c r="O43" s="5"/>
       <c r="P43" s="5"/>
       <c r="Q43" s="5"/>
@@ -2891,12 +2860,12 @@
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="L44" s="5"/>
       <c r="M44" s="5"/>
@@ -2918,12 +2887,12 @@
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
       <c r="H45" s="5" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
@@ -2945,12 +2914,12 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
@@ -2972,12 +2941,12 @@
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
       <c r="H47" s="5" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
@@ -2991,24 +2960,32 @@
       <c r="U47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="9"/>
-      <c r="B48" s="5"/>
+      <c r="A48" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
+      <c r="E48" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
       <c r="H48" s="5" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
       <c r="K48" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
-      <c r="N48" s="5"/>
+      <c r="N48" s="5" t="s">
+        <v>136</v>
+      </c>
       <c r="O48" s="5"/>
       <c r="P48" s="5"/>
       <c r="Q48" s="5"/>
@@ -3026,12 +3003,12 @@
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
       <c r="H49" s="5" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="L49" s="5"/>
       <c r="M49" s="5"/>
@@ -3045,32 +3022,24 @@
       <c r="U49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>141</v>
-      </c>
+      <c r="A50" s="9"/>
+      <c r="B50" s="5"/>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
-      <c r="E50" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="E50" s="5"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="5" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
-      <c r="N50" s="5" t="s">
-        <v>143</v>
-      </c>
+      <c r="N50" s="5"/>
       <c r="O50" s="5"/>
       <c r="P50" s="5"/>
       <c r="Q50" s="5"/>
@@ -3088,12 +3057,12 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
       <c r="K51" s="5" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
@@ -3107,24 +3076,44 @@
       <c r="U51" s="5"/>
     </row>
     <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="9"/>
-      <c r="B52" s="5"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
+      <c r="A52" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
       <c r="H52" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
+        <v>139</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J52" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="K52" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="L52" s="5"/>
-      <c r="M52" s="5"/>
-      <c r="N52" s="5"/>
+        <v>140</v>
+      </c>
+      <c r="L52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="M52" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="N52" s="5" t="s">
+        <v>141</v>
+      </c>
       <c r="O52" s="5"/>
       <c r="P52" s="5"/>
       <c r="Q52" s="5"/>
@@ -3142,15 +3131,23 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
       <c r="H53" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
+        <v>142</v>
+      </c>
+      <c r="I53" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="K53" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="L53" s="5"/>
-      <c r="M53" s="5"/>
+        <v>143</v>
+      </c>
+      <c r="L53" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="M53" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="N53" s="5"/>
       <c r="O53" s="5"/>
       <c r="P53" s="5"/>
@@ -3161,44 +3158,32 @@
       <c r="U53" s="5"/>
     </row>
     <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E54" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="A54" s="9"/>
+      <c r="B54" s="5"/>
+      <c r="C54" s="5"/>
+      <c r="D54" s="5"/>
+      <c r="E54" s="5"/>
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
       <c r="H54" s="5" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="N54" s="5" t="s">
-        <v>148</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="N54" s="5"/>
       <c r="O54" s="5"/>
       <c r="P54" s="5"/>
       <c r="Q54" s="5"/>
@@ -3207,486 +3192,416 @@
       <c r="T54" s="5"/>
       <c r="U54" s="5"/>
     </row>
-    <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="9"/>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5" t="s">
+    <row r="55" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+      <c r="I55" s="2"/>
+      <c r="J55" s="2"/>
+      <c r="K55" s="2"/>
+      <c r="L55" s="2"/>
+      <c r="M55" s="2"/>
+      <c r="N55" s="2"/>
+      <c r="O55" s="2"/>
+      <c r="P55" s="2"/>
+      <c r="Q55" s="2"/>
+      <c r="R55" s="2"/>
+      <c r="S55" s="2"/>
+      <c r="T55" s="2"/>
+      <c r="U55" s="2"/>
+    </row>
+    <row r="56" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6"/>
+      <c r="K56" s="6"/>
+      <c r="L56" s="6"/>
+      <c r="M56" s="6"/>
+      <c r="N56" s="6"/>
+      <c r="O56" s="6"/>
+      <c r="P56" s="6"/>
+      <c r="Q56" s="6"/>
+      <c r="R56" s="6"/>
+      <c r="S56" s="6"/>
+      <c r="T56" s="6"/>
+      <c r="U56" s="6"/>
+      <c r="V56" s="6"/>
+      <c r="W56" s="6"/>
+    </row>
+    <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="I55" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="J55" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="K55" s="5" t="s">
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="L55" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="M55" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="N55" s="5"/>
-      <c r="O55" s="5"/>
-      <c r="P55" s="5"/>
-      <c r="Q55" s="5"/>
-      <c r="R55" s="5"/>
-      <c r="S55" s="5"/>
-      <c r="T55" s="5"/>
-      <c r="U55" s="5"/>
-    </row>
-    <row r="56" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="9"/>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="5" t="s">
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="I56" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="J56" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="K56" s="5" t="s">
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="4"/>
+      <c r="R57" s="4"/>
+      <c r="S57" s="4"/>
+      <c r="T57" s="4"/>
+      <c r="U57" s="4"/>
+      <c r="V57" s="4"/>
+      <c r="W57" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="L56" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="M56" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="N56" s="5"/>
-      <c r="O56" s="5"/>
-      <c r="P56" s="5"/>
-      <c r="Q56" s="5"/>
-      <c r="R56" s="5"/>
-      <c r="S56" s="5"/>
-      <c r="T56" s="5"/>
-      <c r="U56" s="5"/>
-    </row>
-    <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
-      <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="2"/>
-      <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" s="2"/>
-      <c r="Q57" s="2"/>
-      <c r="R57" s="2"/>
-      <c r="S57" s="2"/>
-      <c r="T57" s="2"/>
-      <c r="U57" s="2"/>
-    </row>
-    <row r="58" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="6" t="s">
+    </row>
+    <row r="58" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="B58" s="6"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="6"/>
-      <c r="E58" s="6"/>
-      <c r="F58" s="6"/>
-      <c r="G58" s="6"/>
-      <c r="H58" s="6"/>
-      <c r="I58" s="6"/>
-      <c r="J58" s="6"/>
-      <c r="K58" s="6"/>
-      <c r="L58" s="6"/>
-      <c r="M58" s="6"/>
-      <c r="N58" s="6"/>
-      <c r="O58" s="6"/>
-      <c r="P58" s="6"/>
-      <c r="Q58" s="6"/>
-      <c r="R58" s="6"/>
-      <c r="S58" s="6"/>
-      <c r="T58" s="6"/>
-      <c r="U58" s="6"/>
-      <c r="V58" s="6"/>
-      <c r="W58" s="6"/>
-    </row>
-    <row r="59" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B59" s="4" t="s">
+      <c r="O58" s="15"/>
+      <c r="P58" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4" t="s">
+      <c r="Q58" s="15"/>
+      <c r="R58" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4" t="s">
+      <c r="S58" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="I59" s="4"/>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4" t="s">
+      <c r="T58" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="L59" s="4"/>
-      <c r="M59" s="4"/>
-      <c r="N59" s="4" t="s">
+      <c r="U58" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="O59" s="4"/>
-      <c r="P59" s="4"/>
-      <c r="Q59" s="4"/>
-      <c r="R59" s="4"/>
-      <c r="S59" s="4"/>
-      <c r="T59" s="4"/>
-      <c r="U59" s="4"/>
-      <c r="V59" s="4"/>
-      <c r="W59" s="4" t="s">
+      <c r="V58" s="15" t="s">
         <v>159</v>
       </c>
+      <c r="W58" s="15" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H59" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I59" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J59" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K59" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L59" s="5"/>
+      <c r="M59" s="5"/>
+      <c r="N59" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="O59" s="5"/>
+      <c r="P59" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q59" s="5"/>
+      <c r="R59" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="S59" s="5"/>
+      <c r="T59" s="5"/>
+      <c r="U59" s="5"/>
+      <c r="V59" s="5"/>
+      <c r="W59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4"/>
-      <c r="B60" s="4"/>
-      <c r="C60" s="4"/>
-      <c r="D60" s="4"/>
-      <c r="E60" s="4"/>
-      <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
-      <c r="H60" s="4"/>
-      <c r="I60" s="4"/>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
-      <c r="L60" s="4"/>
-      <c r="M60" s="4"/>
-      <c r="N60" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="O60" s="15"/>
-      <c r="P60" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q60" s="15"/>
-      <c r="R60" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="S60" s="15" t="s">
-        <v>163</v>
-      </c>
-      <c r="T60" s="15" t="s">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="2"/>
+      <c r="H60" s="2"/>
+      <c r="I60" s="2"/>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
+      <c r="L60" s="2"/>
+      <c r="M60" s="2"/>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
+      <c r="P60" s="2"/>
+      <c r="Q60" s="2"/>
+      <c r="R60" s="2"/>
+      <c r="S60" s="2"/>
+      <c r="T60" s="2"/>
+      <c r="U60" s="2"/>
+    </row>
+    <row r="61" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="U60" s="15" t="s">
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
+      <c r="G61" s="6"/>
+      <c r="H61" s="6"/>
+      <c r="I61" s="6"/>
+      <c r="J61" s="6"/>
+      <c r="K61" s="6"/>
+      <c r="L61" s="6"/>
+      <c r="M61" s="6"/>
+      <c r="N61" s="6"/>
+      <c r="O61" s="6"/>
+      <c r="P61" s="6"/>
+      <c r="Q61" s="6"/>
+      <c r="R61" s="6"/>
+      <c r="S61" s="6"/>
+      <c r="T61" s="6"/>
+      <c r="U61" s="6"/>
+    </row>
+    <row r="62" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="V60" s="15" t="s">
+      <c r="B62" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="W60" s="15" t="s">
+      <c r="C62" s="4" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="9" t="n">
+      <c r="D62" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="H62" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+    </row>
+    <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B61" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="E61" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="F61" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="H61" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I61" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="J61" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="K61" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L61" s="5"/>
-      <c r="M61" s="5"/>
-      <c r="N61" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="O61" s="5"/>
-      <c r="P61" s="5" t="s">
+      <c r="B63" s="16"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="H63" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="Q61" s="5"/>
-      <c r="R61" s="5" t="s">
+      <c r="I63" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="S61" s="5"/>
-      <c r="T61" s="5"/>
-      <c r="U61" s="5"/>
-      <c r="V61" s="5"/>
-      <c r="W61" s="5"/>
-    </row>
-    <row r="62" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="2"/>
-      <c r="I62" s="2"/>
-      <c r="J62" s="2"/>
-      <c r="K62" s="2"/>
-      <c r="L62" s="2"/>
-      <c r="M62" s="2"/>
-      <c r="N62" s="2"/>
-      <c r="O62" s="2"/>
-      <c r="P62" s="2"/>
-      <c r="Q62" s="2"/>
-      <c r="R62" s="2"/>
-      <c r="S62" s="2"/>
-      <c r="T62" s="2"/>
-      <c r="U62" s="2"/>
-    </row>
-    <row r="63" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="6" t="s">
+      <c r="J63" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B63" s="6"/>
-      <c r="C63" s="6"/>
-      <c r="D63" s="6"/>
-      <c r="E63" s="6"/>
-      <c r="F63" s="6"/>
-      <c r="G63" s="6"/>
-      <c r="H63" s="6"/>
-      <c r="I63" s="6"/>
-      <c r="J63" s="6"/>
-      <c r="K63" s="6"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="6"/>
-      <c r="N63" s="6"/>
-      <c r="O63" s="6"/>
-      <c r="P63" s="6"/>
-      <c r="Q63" s="6"/>
-      <c r="R63" s="6"/>
-      <c r="S63" s="6"/>
-      <c r="T63" s="6"/>
-      <c r="U63" s="6"/>
-    </row>
-    <row r="64" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="s">
+      <c r="K63" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B64" s="4" t="s">
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="H64" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I64" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="C64" s="4" t="s">
+      <c r="J64" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="D64" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="H64" s="4" t="s">
+      <c r="K64" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-    </row>
-    <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B65" s="16"/>
+        <v>3</v>
+      </c>
+      <c r="B65" s="17"/>
       <c r="C65" s="9"/>
       <c r="D65" s="5" t="s">
-        <v>45</v>
+        <v>176</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
-      <c r="H65" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="I65" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="J65" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="K65" s="9" t="s">
-        <v>179</v>
-      </c>
+      <c r="H65" s="18"/>
+      <c r="I65" s="18"/>
+      <c r="J65" s="18"/>
+      <c r="K65" s="18"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B66" s="16"/>
-      <c r="C66" s="16"/>
+        <v>4</v>
+      </c>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
       <c r="D66" s="5" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
-      <c r="H66" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I66" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="J66" s="9" t="s">
-        <v>181</v>
-      </c>
-      <c r="K66" s="9" t="s">
-        <v>182</v>
-      </c>
+      <c r="H66" s="18"/>
+      <c r="I66" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="J66" s="5"/>
+      <c r="K66" s="18"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B67" s="17"/>
+        <v>5</v>
+      </c>
+      <c r="B67" s="19"/>
       <c r="C67" s="9"/>
       <c r="D67" s="5" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
-      <c r="H67" s="18"/>
-      <c r="I67" s="18"/>
-      <c r="J67" s="18"/>
-      <c r="K67" s="18"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B68" s="19"/>
-      <c r="C68" s="19"/>
+        <v>6</v>
+      </c>
+      <c r="B68" s="17"/>
+      <c r="C68" s="17"/>
       <c r="D68" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
-      <c r="H68" s="18"/>
-      <c r="I68" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="J68" s="5"/>
-      <c r="K68" s="18"/>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B69" s="19"/>
+        <v>7</v>
+      </c>
+      <c r="B69" s="20"/>
       <c r="C69" s="9"/>
       <c r="D69" s="5" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
-      <c r="I69" s="5"/>
-      <c r="J69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="B70" s="20"/>
+      <c r="C70" s="20"/>
       <c r="D70" s="5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
     </row>
-    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B71" s="20"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="E71" s="5"/>
-      <c r="F71" s="5"/>
-    </row>
-    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B72" s="20"/>
-      <c r="C72" s="20"/>
-      <c r="D72" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="E72" s="5"/>
-      <c r="F72" s="5"/>
-    </row>
-    <row r="73" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="2"/>
-      <c r="I73" s="2"/>
-      <c r="J73" s="2"/>
-      <c r="K73" s="2"/>
-      <c r="L73" s="2"/>
-      <c r="M73" s="2"/>
-      <c r="N73" s="2"/>
-      <c r="O73" s="2"/>
-      <c r="P73" s="2"/>
-      <c r="Q73" s="2"/>
-      <c r="R73" s="2"/>
-      <c r="S73" s="2"/>
-      <c r="T73" s="2"/>
-      <c r="U73" s="2"/>
+    <row r="71" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2"/>
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="E71" s="2"/>
+      <c r="F71" s="2"/>
+      <c r="G71" s="2"/>
+      <c r="H71" s="2"/>
+      <c r="I71" s="2"/>
+      <c r="J71" s="2"/>
+      <c r="K71" s="2"/>
+      <c r="L71" s="2"/>
+      <c r="M71" s="2"/>
+      <c r="N71" s="2"/>
+      <c r="O71" s="2"/>
+      <c r="P71" s="2"/>
+      <c r="Q71" s="2"/>
+      <c r="R71" s="2"/>
+      <c r="S71" s="2"/>
+      <c r="T71" s="2"/>
+      <c r="U71" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="188">
+  <mergeCells count="182">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -3733,8 +3648,8 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:N16"/>
-    <mergeCell ref="O16:Q25"/>
-    <mergeCell ref="R16:U25"/>
+    <mergeCell ref="O16:Q23"/>
+    <mergeCell ref="R16:U23"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:N17"/>
@@ -3756,59 +3671,57 @@
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="G23:N23"/>
-    <mergeCell ref="B24:D24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="G24:N24"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="G25:N25"/>
-    <mergeCell ref="A26:U26"/>
-    <mergeCell ref="A27:U27"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="G28:N28"/>
-    <mergeCell ref="O28:Q28"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="G29:N29"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="A30:U30"/>
-    <mergeCell ref="A31:U31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="G32:N32"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="G33:N33"/>
-    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="A25:U25"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G26:N26"/>
+    <mergeCell ref="O26:Q26"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:N27"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="A28:U28"/>
+    <mergeCell ref="A29:U29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="G30:N30"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="G31:N31"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="A32:U32"/>
+    <mergeCell ref="A33:U33"/>
     <mergeCell ref="A34:U34"/>
-    <mergeCell ref="A35:U35"/>
-    <mergeCell ref="A36:U36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="N35:U35"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="B36:D40"/>
+    <mergeCell ref="E36:G47"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="N36:U40"/>
     <mergeCell ref="H37:J37"/>
     <mergeCell ref="K37:M37"/>
-    <mergeCell ref="N37:U37"/>
-    <mergeCell ref="A38:A42"/>
-    <mergeCell ref="B38:D42"/>
-    <mergeCell ref="E38:G49"/>
     <mergeCell ref="H38:J38"/>
     <mergeCell ref="K38:M38"/>
-    <mergeCell ref="N38:U42"/>
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="H40:J40"/>
     <mergeCell ref="K40:M40"/>
+    <mergeCell ref="A41:A47"/>
+    <mergeCell ref="B41:D47"/>
     <mergeCell ref="H41:J41"/>
     <mergeCell ref="K41:M41"/>
+    <mergeCell ref="N41:U47"/>
     <mergeCell ref="H42:J42"/>
     <mergeCell ref="K42:M42"/>
-    <mergeCell ref="A43:A49"/>
-    <mergeCell ref="B43:D49"/>
     <mergeCell ref="H43:J43"/>
     <mergeCell ref="K43:M43"/>
-    <mergeCell ref="N43:U49"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="K44:M44"/>
     <mergeCell ref="H45:J45"/>
@@ -3817,64 +3730,60 @@
     <mergeCell ref="K46:M46"/>
     <mergeCell ref="H47:J47"/>
     <mergeCell ref="K47:M47"/>
+    <mergeCell ref="A48:A51"/>
+    <mergeCell ref="B48:D51"/>
+    <mergeCell ref="E48:G51"/>
     <mergeCell ref="H48:J48"/>
     <mergeCell ref="K48:M48"/>
+    <mergeCell ref="N48:U51"/>
     <mergeCell ref="H49:J49"/>
     <mergeCell ref="K49:M49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="B50:D53"/>
-    <mergeCell ref="E50:G53"/>
     <mergeCell ref="H50:J50"/>
     <mergeCell ref="K50:M50"/>
-    <mergeCell ref="N50:U53"/>
     <mergeCell ref="H51:J51"/>
     <mergeCell ref="K51:M51"/>
+    <mergeCell ref="A52:A54"/>
+    <mergeCell ref="B52:D54"/>
+    <mergeCell ref="E52:G54"/>
     <mergeCell ref="H52:J52"/>
     <mergeCell ref="K52:M52"/>
+    <mergeCell ref="N52:U54"/>
     <mergeCell ref="H53:J53"/>
     <mergeCell ref="K53:M53"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="B54:D56"/>
-    <mergeCell ref="E54:G56"/>
     <mergeCell ref="H54:J54"/>
     <mergeCell ref="K54:M54"/>
-    <mergeCell ref="N54:U56"/>
-    <mergeCell ref="H55:J55"/>
-    <mergeCell ref="K55:M55"/>
-    <mergeCell ref="H56:J56"/>
-    <mergeCell ref="K56:M56"/>
-    <mergeCell ref="A57:U57"/>
-    <mergeCell ref="A58:W58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="B59:D60"/>
-    <mergeCell ref="E59:G60"/>
-    <mergeCell ref="H59:J60"/>
-    <mergeCell ref="K59:M60"/>
+    <mergeCell ref="A55:U55"/>
+    <mergeCell ref="A56:W56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="B57:D58"/>
+    <mergeCell ref="E57:G58"/>
+    <mergeCell ref="H57:J58"/>
+    <mergeCell ref="K57:M58"/>
+    <mergeCell ref="N57:O57"/>
+    <mergeCell ref="P57:V57"/>
+    <mergeCell ref="N58:O58"/>
+    <mergeCell ref="P58:Q58"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="H59:J59"/>
+    <mergeCell ref="K59:M59"/>
     <mergeCell ref="N59:O59"/>
-    <mergeCell ref="P59:V59"/>
-    <mergeCell ref="N60:O60"/>
-    <mergeCell ref="P60:Q60"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="E61:G61"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="K61:M61"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="P61:Q61"/>
-    <mergeCell ref="R61:W61"/>
-    <mergeCell ref="A62:U62"/>
-    <mergeCell ref="A63:U63"/>
+    <mergeCell ref="P59:Q59"/>
+    <mergeCell ref="R59:W59"/>
+    <mergeCell ref="A60:U60"/>
+    <mergeCell ref="A61:U61"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="H62:K62"/>
+    <mergeCell ref="D63:F63"/>
     <mergeCell ref="D64:F64"/>
-    <mergeCell ref="H64:K64"/>
     <mergeCell ref="D65:F65"/>
     <mergeCell ref="D66:F66"/>
+    <mergeCell ref="I66:J67"/>
     <mergeCell ref="D67:F67"/>
     <mergeCell ref="D68:F68"/>
-    <mergeCell ref="I68:J69"/>
     <mergeCell ref="D69:F69"/>
     <mergeCell ref="D70:F70"/>
-    <mergeCell ref="D71:F71"/>
-    <mergeCell ref="D72:F72"/>
-    <mergeCell ref="A73:U73"/>
+    <mergeCell ref="A71:U71"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.26 ] - roulette docs was updated & file structure was init.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="187">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -555,6 +555,33 @@
   </si>
   <si>
     <t xml:space="preserve">CABLE INPUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roulette_dataset_t</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roulette.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dataset structure which store roulette runtime properties.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE R2 ENABLE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE R1 ENABLE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR M2 ENABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR M1 ENABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR DIR2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR DIR1</t>
   </si>
 </sst>
 </file>
@@ -564,7 +591,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -621,6 +648,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -738,7 +770,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -820,6 +852,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1599,7 +1635,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W71"/>
+  <dimension ref="A1:AC83"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3241,6 +3277,12 @@
       <c r="U56" s="6"/>
       <c r="V56" s="6"/>
       <c r="W56" s="6"/>
+      <c r="X56" s="6"/>
+      <c r="Y56" s="6"/>
+      <c r="Z56" s="6"/>
+      <c r="AA56" s="6"/>
+      <c r="AB56" s="6"/>
+      <c r="AC56" s="6"/>
     </row>
     <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
@@ -3277,9 +3319,15 @@
       <c r="T57" s="4"/>
       <c r="U57" s="4"/>
       <c r="V57" s="4"/>
-      <c r="W57" s="4" t="s">
+      <c r="W57" s="4"/>
+      <c r="X57" s="4"/>
+      <c r="Y57" s="4"/>
+      <c r="Z57" s="4"/>
+      <c r="AA57" s="4"/>
+      <c r="AB57" s="4" t="s">
         <v>152</v>
       </c>
+      <c r="AC57" s="4"/>
     </row>
     <row r="58" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4"/>
@@ -3306,21 +3354,27 @@
       <c r="R58" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="S58" s="15" t="s">
+      <c r="S58" s="15"/>
+      <c r="T58" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="T58" s="15" t="s">
+      <c r="U58" s="15"/>
+      <c r="V58" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="U58" s="15" t="s">
+      <c r="W58" s="15"/>
+      <c r="X58" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="V58" s="15" t="s">
+      <c r="Y58" s="15"/>
+      <c r="Z58" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="W58" s="15" t="s">
+      <c r="AA58" s="15"/>
+      <c r="AB58" s="15" t="s">
         <v>160</v>
       </c>
+      <c r="AC58" s="15"/>
     </row>
     <row r="59" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="n">
@@ -3374,6 +3428,12 @@
       <c r="U59" s="5"/>
       <c r="V59" s="5"/>
       <c r="W59" s="5"/>
+      <c r="X59" s="5"/>
+      <c r="Y59" s="5"/>
+      <c r="Z59" s="5"/>
+      <c r="AA59" s="5"/>
+      <c r="AB59" s="5"/>
+      <c r="AC59" s="5"/>
     </row>
     <row r="60" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="2"/>
@@ -3600,8 +3660,444 @@
       <c r="T71" s="2"/>
       <c r="U71" s="2"/>
     </row>
+    <row r="72" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="14"/>
+      <c r="C72" s="14"/>
+      <c r="D72" s="14"/>
+      <c r="E72" s="14"/>
+      <c r="F72" s="14"/>
+      <c r="G72" s="14"/>
+      <c r="H72" s="14"/>
+      <c r="I72" s="14"/>
+      <c r="J72" s="14"/>
+      <c r="K72" s="14"/>
+      <c r="L72" s="14"/>
+      <c r="M72" s="14"/>
+      <c r="N72" s="14"/>
+      <c r="O72" s="14"/>
+      <c r="P72" s="14"/>
+      <c r="Q72" s="14"/>
+      <c r="R72" s="14"/>
+      <c r="S72" s="14"/>
+      <c r="T72" s="14"/>
+      <c r="U72" s="14"/>
+    </row>
+    <row r="73" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B73" s="6"/>
+      <c r="C73" s="6"/>
+      <c r="D73" s="6"/>
+      <c r="E73" s="6"/>
+      <c r="F73" s="6"/>
+      <c r="G73" s="6"/>
+      <c r="H73" s="6"/>
+      <c r="I73" s="6"/>
+      <c r="J73" s="6"/>
+      <c r="K73" s="6"/>
+      <c r="L73" s="6"/>
+      <c r="M73" s="6"/>
+      <c r="N73" s="6"/>
+      <c r="O73" s="6"/>
+      <c r="P73" s="6"/>
+      <c r="Q73" s="6"/>
+      <c r="R73" s="6"/>
+      <c r="S73" s="6"/>
+      <c r="T73" s="6"/>
+      <c r="U73" s="6"/>
+    </row>
+    <row r="74" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+      <c r="H74" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="I74" s="4"/>
+      <c r="J74" s="4"/>
+      <c r="K74" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="L74" s="4"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="O74" s="4"/>
+      <c r="P74" s="4"/>
+      <c r="Q74" s="4"/>
+      <c r="R74" s="4"/>
+      <c r="S74" s="4"/>
+      <c r="T74" s="4"/>
+      <c r="U74" s="4"/>
+    </row>
+    <row r="75" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C75" s="5"/>
+      <c r="D75" s="5"/>
+      <c r="E75" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="F75" s="5"/>
+      <c r="G75" s="5"/>
+      <c r="H75" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="I75" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J75" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K75" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="L75" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="M75" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="N75" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="O75" s="5"/>
+      <c r="P75" s="5"/>
+      <c r="Q75" s="5"/>
+      <c r="R75" s="5"/>
+      <c r="S75" s="5"/>
+      <c r="T75" s="5"/>
+      <c r="U75" s="5"/>
+    </row>
+    <row r="76" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="9"/>
+      <c r="B76" s="5"/>
+      <c r="C76" s="5"/>
+      <c r="D76" s="5"/>
+      <c r="E76" s="5"/>
+      <c r="F76" s="5"/>
+      <c r="G76" s="5"/>
+      <c r="H76" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="I76" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J76" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K76" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="L76" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="M76" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="N76" s="5"/>
+      <c r="O76" s="5"/>
+      <c r="P76" s="5"/>
+      <c r="Q76" s="5"/>
+      <c r="R76" s="5"/>
+      <c r="S76" s="5"/>
+      <c r="T76" s="5"/>
+      <c r="U76" s="5"/>
+    </row>
+    <row r="77" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="9"/>
+      <c r="B77" s="5"/>
+      <c r="C77" s="5"/>
+      <c r="D77" s="5"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="5"/>
+      <c r="H77" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="I77" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J77" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K77" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="L77" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="M77" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="N77" s="5"/>
+      <c r="O77" s="5"/>
+      <c r="P77" s="5"/>
+      <c r="Q77" s="5"/>
+      <c r="R77" s="5"/>
+      <c r="S77" s="5"/>
+      <c r="T77" s="5"/>
+      <c r="U77" s="5"/>
+    </row>
+    <row r="78" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2"/>
+      <c r="B78" s="2"/>
+      <c r="C78" s="2"/>
+      <c r="D78" s="2"/>
+      <c r="E78" s="2"/>
+      <c r="F78" s="2"/>
+      <c r="G78" s="2"/>
+      <c r="H78" s="2"/>
+      <c r="I78" s="2"/>
+      <c r="J78" s="2"/>
+      <c r="K78" s="2"/>
+      <c r="L78" s="2"/>
+      <c r="M78" s="2"/>
+      <c r="N78" s="2"/>
+      <c r="O78" s="2"/>
+      <c r="P78" s="2"/>
+      <c r="Q78" s="2"/>
+      <c r="R78" s="2"/>
+      <c r="S78" s="2"/>
+      <c r="T78" s="2"/>
+      <c r="U78" s="2"/>
+    </row>
+    <row r="79" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="B79" s="6"/>
+      <c r="C79" s="6"/>
+      <c r="D79" s="6"/>
+      <c r="E79" s="6"/>
+      <c r="F79" s="6"/>
+      <c r="G79" s="6"/>
+      <c r="H79" s="6"/>
+      <c r="I79" s="6"/>
+      <c r="J79" s="6"/>
+      <c r="K79" s="6"/>
+      <c r="L79" s="6"/>
+      <c r="M79" s="6"/>
+      <c r="N79" s="6"/>
+      <c r="O79" s="6"/>
+      <c r="P79" s="6"/>
+      <c r="Q79" s="6"/>
+      <c r="R79" s="6"/>
+      <c r="S79" s="6"/>
+      <c r="T79" s="6"/>
+      <c r="U79" s="6"/>
+      <c r="V79" s="6"/>
+      <c r="W79" s="6"/>
+      <c r="X79" s="6"/>
+      <c r="Y79" s="6"/>
+      <c r="Z79" s="6"/>
+      <c r="AA79" s="6"/>
+      <c r="AB79" s="6"/>
+      <c r="AC79" s="6"/>
+    </row>
+    <row r="80" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F80" s="4"/>
+      <c r="G80" s="4"/>
+      <c r="H80" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="I80" s="4"/>
+      <c r="J80" s="4"/>
+      <c r="K80" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="L80" s="4"/>
+      <c r="M80" s="4"/>
+      <c r="N80" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="O80" s="4"/>
+      <c r="P80" s="4"/>
+      <c r="Q80" s="4"/>
+      <c r="R80" s="4"/>
+      <c r="S80" s="4"/>
+      <c r="T80" s="4"/>
+      <c r="U80" s="4"/>
+      <c r="V80" s="4"/>
+      <c r="W80" s="4"/>
+      <c r="X80" s="4"/>
+      <c r="Y80" s="4"/>
+      <c r="Z80" s="4"/>
+      <c r="AA80" s="4"/>
+      <c r="AB80" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="AC80" s="4"/>
+    </row>
+    <row r="81" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="4"/>
+      <c r="H81" s="4"/>
+      <c r="I81" s="4"/>
+      <c r="J81" s="4"/>
+      <c r="K81" s="4"/>
+      <c r="L81" s="4"/>
+      <c r="M81" s="4"/>
+      <c r="N81" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="O81" s="15"/>
+      <c r="P81" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q81" s="15"/>
+      <c r="R81" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="S81" s="15"/>
+      <c r="T81" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="U81" s="15"/>
+      <c r="V81" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="W81" s="15"/>
+      <c r="X81" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="Y81" s="15"/>
+      <c r="Z81" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="AA81" s="15"/>
+      <c r="AB81" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="AC81" s="15"/>
+    </row>
+    <row r="82" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B82" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="C82" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="D82" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F82" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I82" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="J82" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="K82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L82" s="5"/>
+      <c r="M82" s="5"/>
+      <c r="N82" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="O82" s="5"/>
+      <c r="P82" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="Q82" s="5"/>
+      <c r="R82" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="S82" s="5"/>
+      <c r="T82" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="U82" s="5"/>
+      <c r="V82" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="W82" s="5"/>
+      <c r="X82" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="Y82" s="5"/>
+      <c r="Z82" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="AA82" s="5"/>
+      <c r="AB82" s="5"/>
+      <c r="AC82" s="5"/>
+    </row>
+    <row r="83" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+      <c r="F83" s="2"/>
+      <c r="G83" s="2"/>
+      <c r="H83" s="2"/>
+      <c r="I83" s="2"/>
+      <c r="J83" s="2"/>
+      <c r="K83" s="2"/>
+      <c r="L83" s="2"/>
+      <c r="M83" s="2"/>
+      <c r="N83" s="2"/>
+      <c r="O83" s="2"/>
+      <c r="P83" s="2"/>
+      <c r="Q83" s="2"/>
+      <c r="R83" s="2"/>
+      <c r="S83" s="2"/>
+      <c r="T83" s="2"/>
+      <c r="U83" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="182">
+  <mergeCells count="236">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -3753,23 +4249,30 @@
     <mergeCell ref="H54:J54"/>
     <mergeCell ref="K54:M54"/>
     <mergeCell ref="A55:U55"/>
-    <mergeCell ref="A56:W56"/>
+    <mergeCell ref="A56:AC56"/>
     <mergeCell ref="A57:A58"/>
     <mergeCell ref="B57:D58"/>
     <mergeCell ref="E57:G58"/>
     <mergeCell ref="H57:J58"/>
     <mergeCell ref="K57:M58"/>
     <mergeCell ref="N57:O57"/>
-    <mergeCell ref="P57:V57"/>
+    <mergeCell ref="P57:AA57"/>
+    <mergeCell ref="AB57:AC57"/>
     <mergeCell ref="N58:O58"/>
     <mergeCell ref="P58:Q58"/>
+    <mergeCell ref="R58:S58"/>
+    <mergeCell ref="T58:U58"/>
+    <mergeCell ref="V58:W58"/>
+    <mergeCell ref="X58:Y58"/>
+    <mergeCell ref="Z58:AA58"/>
+    <mergeCell ref="AB58:AC58"/>
     <mergeCell ref="B59:D59"/>
     <mergeCell ref="E59:G59"/>
     <mergeCell ref="H59:J59"/>
     <mergeCell ref="K59:M59"/>
     <mergeCell ref="N59:O59"/>
     <mergeCell ref="P59:Q59"/>
-    <mergeCell ref="R59:W59"/>
+    <mergeCell ref="R59:AC59"/>
     <mergeCell ref="A60:U60"/>
     <mergeCell ref="A61:U61"/>
     <mergeCell ref="D62:F62"/>
@@ -3784,6 +4287,53 @@
     <mergeCell ref="D69:F69"/>
     <mergeCell ref="D70:F70"/>
     <mergeCell ref="A71:U71"/>
+    <mergeCell ref="A72:U72"/>
+    <mergeCell ref="A73:U73"/>
+    <mergeCell ref="B74:D74"/>
+    <mergeCell ref="E74:G74"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="K74:M74"/>
+    <mergeCell ref="N74:U74"/>
+    <mergeCell ref="A75:A77"/>
+    <mergeCell ref="B75:D77"/>
+    <mergeCell ref="E75:G77"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="K75:M75"/>
+    <mergeCell ref="N75:U77"/>
+    <mergeCell ref="H76:J76"/>
+    <mergeCell ref="K76:M76"/>
+    <mergeCell ref="H77:J77"/>
+    <mergeCell ref="K77:M77"/>
+    <mergeCell ref="A78:U78"/>
+    <mergeCell ref="A79:AC79"/>
+    <mergeCell ref="A80:A81"/>
+    <mergeCell ref="B80:D81"/>
+    <mergeCell ref="E80:G81"/>
+    <mergeCell ref="H80:J81"/>
+    <mergeCell ref="K80:M81"/>
+    <mergeCell ref="N80:O80"/>
+    <mergeCell ref="P80:AA80"/>
+    <mergeCell ref="AB80:AC80"/>
+    <mergeCell ref="N81:O81"/>
+    <mergeCell ref="P81:Q81"/>
+    <mergeCell ref="R81:S81"/>
+    <mergeCell ref="T81:U81"/>
+    <mergeCell ref="V81:W81"/>
+    <mergeCell ref="X81:Y81"/>
+    <mergeCell ref="Z81:AA81"/>
+    <mergeCell ref="AB81:AC81"/>
+    <mergeCell ref="B82:D82"/>
+    <mergeCell ref="E82:G82"/>
+    <mergeCell ref="H82:J82"/>
+    <mergeCell ref="K82:M82"/>
+    <mergeCell ref="N82:O82"/>
+    <mergeCell ref="P82:Q82"/>
+    <mergeCell ref="R82:S82"/>
+    <mergeCell ref="T82:U82"/>
+    <mergeCell ref="V82:W82"/>
+    <mergeCell ref="X82:Y82"/>
+    <mergeCell ref="Z82:AC82"/>
+    <mergeCell ref="A83:U83"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.26.2 ] - roulette header was updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -591,7 +591,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -648,11 +648,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -770,7 +765,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -852,10 +847,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4010,13 +4001,13 @@
       <c r="A82" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B82" s="21" t="s">
+      <c r="B82" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="C82" s="21" t="s">
+      <c r="C82" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D82" s="21" t="s">
+      <c r="D82" s="5" t="s">
         <v>110</v>
       </c>
       <c r="E82" s="5" t="s">

</xml_diff>

<commit_message>
[ Version 0.0.26.3 ] - some roulette code was written.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="183">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -570,18 +570,6 @@
   </si>
   <si>
     <t xml:space="preserve">ROULETTE R1 ENABLE </t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR M2 ENABLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR M1 ENABLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR DIR2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR DIR1</t>
   </si>
 </sst>
 </file>
@@ -4042,24 +4030,16 @@
       </c>
       <c r="Q82" s="5"/>
       <c r="R82" s="5" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
       <c r="S82" s="5"/>
-      <c r="T82" s="5" t="s">
-        <v>184</v>
-      </c>
+      <c r="T82" s="5"/>
       <c r="U82" s="5"/>
-      <c r="V82" s="5" t="s">
-        <v>185</v>
-      </c>
+      <c r="V82" s="5"/>
       <c r="W82" s="5"/>
-      <c r="X82" s="5" t="s">
-        <v>186</v>
-      </c>
+      <c r="X82" s="5"/>
       <c r="Y82" s="5"/>
-      <c r="Z82" s="5" t="s">
-        <v>163</v>
-      </c>
+      <c r="Z82" s="5"/>
       <c r="AA82" s="5"/>
       <c r="AB82" s="5"/>
       <c r="AC82" s="5"/>
@@ -4088,7 +4068,7 @@
       <c r="U83" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="236">
+  <mergeCells count="232">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -4319,11 +4299,7 @@
     <mergeCell ref="K82:M82"/>
     <mergeCell ref="N82:O82"/>
     <mergeCell ref="P82:Q82"/>
-    <mergeCell ref="R82:S82"/>
-    <mergeCell ref="T82:U82"/>
-    <mergeCell ref="V82:W82"/>
-    <mergeCell ref="X82:Y82"/>
-    <mergeCell ref="Z82:AC82"/>
+    <mergeCell ref="R82:AC82"/>
     <mergeCell ref="A83:U83"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
[ Version 0.0.28.6 ] - drainage vent TODOs was done.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="180">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -518,9 +518,6 @@
     <t xml:space="preserve">RJ45 CONNECTION</t>
   </si>
   <si>
-    <t xml:space="preserve">CABLE</t>
-  </si>
-  <si>
     <t xml:space="preserve">COLOR 1</t>
   </si>
   <si>
@@ -530,31 +527,25 @@
     <t xml:space="preserve">RJ45 socket schematics – BOTTOM VIEW</t>
   </si>
   <si>
-    <t xml:space="preserve">GND_1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GND_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5V_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5V_1</t>
+    <t xml:space="preserve">+10V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESO</t>
   </si>
   <si>
     <t xml:space="preserve">ESC</t>
   </si>
   <si>
-    <t xml:space="preserve">ESO</t>
+    <t xml:space="preserve">CABLE INPUT</t>
   </si>
   <si>
     <t xml:space="preserve">PWM</t>
   </si>
   <si>
-    <t xml:space="preserve">ESC button</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CABLE INPUT</t>
+    <t xml:space="preserve">+6V</t>
   </si>
   <si>
     <t xml:space="preserve">roulette_dataset_t</t>
@@ -579,7 +570,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -636,6 +627,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -753,7 +749,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -819,6 +815,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3470,151 +3470,124 @@
         <v>166</v>
       </c>
       <c r="C62" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="G62" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="D62" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="H62" s="4" t="s">
-        <v>168</v>
-      </c>
+      <c r="H62" s="4"/>
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
     </row>
     <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B63" s="16"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="5" t="s">
-        <v>45</v>
-      </c>
+      <c r="A63" s="16"/>
+      <c r="B63" s="9"/>
+      <c r="C63" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D63" s="5"/>
       <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="H63" s="9" t="s">
+      <c r="G63" s="17" t="s">
         <v>169</v>
       </c>
-      <c r="I63" s="9" t="s">
+      <c r="H63" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="I63" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="J63" s="17" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="16"/>
+      <c r="B64" s="16"/>
+      <c r="C64" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="J63" s="9" t="s">
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="G64" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="H64" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="I64" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="J64" s="17" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="18"/>
+      <c r="B65" s="9"/>
+      <c r="C65" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="D65" s="17"/>
+      <c r="E65" s="17"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="19"/>
+      <c r="I65" s="19"/>
+      <c r="J65" s="19"/>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="18"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="K63" s="9" t="s">
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="G66" s="19"/>
+      <c r="H66" s="5" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B64" s="16"/>
-      <c r="C64" s="16"/>
-      <c r="D64" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="E64" s="5"/>
-      <c r="F64" s="5"/>
-      <c r="H64" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I64" s="9" t="s">
+      <c r="I66" s="5"/>
+      <c r="J66" s="19"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="20"/>
+      <c r="B67" s="9"/>
+      <c r="C67" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="20"/>
+      <c r="B68" s="20"/>
+      <c r="C68" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="J64" s="9" t="s">
+      <c r="D68" s="17"/>
+      <c r="E68" s="17"/>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="21"/>
+      <c r="B69" s="9"/>
+      <c r="C69" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="K64" s="9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B65" s="17"/>
-      <c r="C65" s="9"/>
-      <c r="D65" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="E65" s="5"/>
-      <c r="F65" s="5"/>
-      <c r="H65" s="18"/>
-      <c r="I65" s="18"/>
-      <c r="J65" s="18"/>
-      <c r="K65" s="18"/>
-    </row>
-    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B66" s="19"/>
-      <c r="C66" s="19"/>
-      <c r="D66" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
-      <c r="H66" s="18"/>
-      <c r="I66" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="J66" s="5"/>
-      <c r="K66" s="18"/>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B67" s="19"/>
-      <c r="C67" s="9"/>
-      <c r="D67" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B68" s="17"/>
-      <c r="C68" s="17"/>
-      <c r="D68" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-    </row>
-    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B69" s="20"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="5" t="s">
-        <v>175</v>
-      </c>
+      <c r="D69" s="5"/>
       <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B70" s="20"/>
-      <c r="C70" s="20"/>
-      <c r="D70" s="5" t="s">
-        <v>171</v>
-      </c>
+      <c r="A70" s="21"/>
+      <c r="B70" s="21"/>
+      <c r="C70" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D70" s="5"/>
       <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
@@ -3729,12 +3702,12 @@
         <v>1</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
       <c r="E75" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
@@ -3757,7 +3730,7 @@
         <v>110</v>
       </c>
       <c r="N75" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="O75" s="5"/>
       <c r="P75" s="5"/>
@@ -3990,7 +3963,7 @@
         <v>1</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>110</v>
@@ -4022,11 +3995,11 @@
       <c r="L82" s="5"/>
       <c r="M82" s="5"/>
       <c r="N82" s="5" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="O82" s="5"/>
       <c r="P82" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="Q82" s="5"/>
       <c r="R82" s="5" t="s">
@@ -4246,17 +4219,17 @@
     <mergeCell ref="R59:AC59"/>
     <mergeCell ref="A60:U60"/>
     <mergeCell ref="A61:U61"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="H62:K62"/>
-    <mergeCell ref="D63:F63"/>
-    <mergeCell ref="D64:F64"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="D66:F66"/>
-    <mergeCell ref="I66:J67"/>
-    <mergeCell ref="D67:F67"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="D69:F69"/>
-    <mergeCell ref="D70:F70"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="G62:J62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="C64:E64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="C66:E66"/>
+    <mergeCell ref="H66:I67"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="C70:E70"/>
     <mergeCell ref="A71:U71"/>
     <mergeCell ref="A72:U72"/>
     <mergeCell ref="A73:U73"/>

</xml_diff>

<commit_message>
[ Version 0.0.28.7 ] - drainage vent RJ45 pinout was updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="180">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -518,6 +518,9 @@
     <t xml:space="preserve">RJ45 CONNECTION</t>
   </si>
   <si>
+    <t xml:space="preserve">CABLE</t>
+  </si>
+  <si>
     <t xml:space="preserve">COLOR 1</t>
   </si>
   <si>
@@ -530,22 +533,19 @@
     <t xml:space="preserve">+10V</t>
   </si>
   <si>
-    <t xml:space="preserve">?</t>
-  </si>
-  <si>
     <t xml:space="preserve">ESO</t>
   </si>
   <si>
     <t xml:space="preserve">ESC</t>
   </si>
   <si>
+    <t xml:space="preserve">+6V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWM</t>
+  </si>
+  <si>
     <t xml:space="preserve">CABLE INPUT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PWM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+6V</t>
   </si>
   <si>
     <t xml:space="preserve">roulette_dataset_t</t>
@@ -570,7 +570,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -627,11 +627,6 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -749,7 +744,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -815,10 +810,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3470,124 +3461,151 @@
         <v>166</v>
       </c>
       <c r="C62" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D62" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D62" s="4"/>
       <c r="E62" s="4"/>
-      <c r="G62" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="H62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="H62" s="4" t="s">
+        <v>168</v>
+      </c>
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
     </row>
     <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="16"/>
-      <c r="B63" s="9"/>
-      <c r="C63" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="D63" s="5"/>
+      <c r="A63" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B63" s="16"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="5" t="s">
+        <v>169</v>
+      </c>
       <c r="E63" s="5"/>
-      <c r="G63" s="17" t="s">
+      <c r="F63" s="5"/>
+      <c r="H63" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="I63" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="J63" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K63" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="H64" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="H63" s="17" t="s">
+      <c r="I64" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="I63" s="17" t="s">
+      <c r="J64" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="K64" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B65" s="17"/>
+      <c r="C65" s="9"/>
+      <c r="D65" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="J63" s="17" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="16"/>
-      <c r="B64" s="16"/>
-      <c r="C64" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
-      <c r="G64" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="H64" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="I64" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="J64" s="17" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="18"/>
-      <c r="B65" s="9"/>
-      <c r="C65" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="D65" s="17"/>
-      <c r="E65" s="17"/>
-      <c r="G65" s="19"/>
-      <c r="H65" s="19"/>
-      <c r="I65" s="19"/>
-      <c r="J65" s="19"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="5"/>
+      <c r="H65" s="18"/>
+      <c r="I65" s="18"/>
+      <c r="J65" s="18"/>
+      <c r="K65" s="18"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="18"/>
-      <c r="B66" s="18"/>
-      <c r="C66" s="5" t="s">
+      <c r="A66" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B66" s="17"/>
+      <c r="C66" s="17"/>
+      <c r="D66" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D66" s="5"/>
       <c r="E66" s="5"/>
-      <c r="G66" s="19"/>
-      <c r="H66" s="5" t="s">
+      <c r="F66" s="5"/>
+      <c r="H66" s="18"/>
+      <c r="I66" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="J66" s="5"/>
+      <c r="K66" s="18"/>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B67" s="19"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="I66" s="5"/>
-      <c r="J66" s="19"/>
-    </row>
-    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="20"/>
-      <c r="B67" s="9"/>
-      <c r="C67" s="5" t="s">
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5"/>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B68" s="19"/>
+      <c r="C68" s="19"/>
+      <c r="D68" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="20"/>
-      <c r="B68" s="20"/>
-      <c r="C68" s="17" t="s">
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B69" s="20"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="D68" s="17"/>
-      <c r="E68" s="17"/>
-    </row>
-    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="21"/>
-      <c r="B69" s="9"/>
-      <c r="C69" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D69" s="5"/>
       <c r="E69" s="5"/>
+      <c r="F69" s="5"/>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="21"/>
-      <c r="B70" s="21"/>
-      <c r="C70" s="5" t="s">
+      <c r="A70" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B70" s="20"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D70" s="5"/>
       <c r="E70" s="5"/>
+      <c r="F70" s="5"/>
     </row>
     <row r="71" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="2"/>
@@ -4219,17 +4237,17 @@
     <mergeCell ref="R59:AC59"/>
     <mergeCell ref="A60:U60"/>
     <mergeCell ref="A61:U61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="G62:J62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="C64:E64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="C66:E66"/>
-    <mergeCell ref="H66:I67"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="C70:E70"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="H62:K62"/>
+    <mergeCell ref="D63:F63"/>
+    <mergeCell ref="D64:F64"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="D66:F66"/>
+    <mergeCell ref="I66:J67"/>
+    <mergeCell ref="D67:F67"/>
+    <mergeCell ref="D68:F68"/>
+    <mergeCell ref="D69:F69"/>
+    <mergeCell ref="D70:F70"/>
     <mergeCell ref="A71:U71"/>
     <mergeCell ref="A72:U72"/>
     <mergeCell ref="A73:U73"/>

</xml_diff>

<commit_message>
[ Version 0.0.28.8 ] - drainage vent bit optimalization was done.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="181">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -83,12 +83,18 @@
     <t xml:space="preserve">drainage_vent.c</t>
   </si>
   <si>
-    <t xml:space="preserve">CmakeLists.txt</t>
+    <t xml:space="preserve">CMakeLists.txt</t>
   </si>
   <si>
     <t xml:space="preserve">roulette</t>
   </si>
   <si>
+    <t xml:space="preserve">roulette.h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roulette.c</t>
+  </si>
+  <si>
     <t xml:space="preserve">code_plan.md</t>
   </si>
   <si>
@@ -506,6 +512,9 @@
     <t xml:space="preserve">B0</t>
   </si>
   <si>
+    <t xml:space="preserve">SPARE</t>
+  </si>
+  <si>
     <t xml:space="preserve">DRAINAGE V2 ENABLE </t>
   </si>
   <si>
@@ -551,13 +560,7 @@
     <t xml:space="preserve">roulette_dataset_t</t>
   </si>
   <si>
-    <t xml:space="preserve">roulette.h</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dataset structure which store roulette runtime properties.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROULETTE R2 ENABLE </t>
   </si>
   <si>
     <t xml:space="preserve">ROULETTE R1 ENABLE </t>
@@ -1012,7 +1015,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1228,10 +1231,12 @@
       </c>
       <c r="J8" s="5"/>
       <c r="K8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
       <c r="P8" s="5"/>
@@ -1249,11 +1254,11 @@
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
@@ -1273,12 +1278,10 @@
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
-      <c r="I10" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="I10" s="5"/>
       <c r="J10" s="5"/>
       <c r="K10" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
@@ -1299,12 +1302,10 @@
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
-      <c r="I11" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="I11" s="5"/>
       <c r="J11" s="5"/>
       <c r="K11" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
@@ -1325,11 +1326,11 @@
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
+      <c r="I12" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="J12" s="5"/>
-      <c r="K12" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="K12" s="5"/>
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
       <c r="N12" s="5"/>
@@ -1350,10 +1351,12 @@
       <c r="G13" s="5"/>
       <c r="H13" s="5"/>
       <c r="I13" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
+      <c r="K13" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
@@ -1377,7 +1380,9 @@
         <v>28</v>
       </c>
       <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
+      <c r="K14" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
@@ -1391,23 +1396,17 @@
     <row r="15" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5"/>
       <c r="B15" s="5"/>
-      <c r="C15" s="5" t="s">
-        <v>29</v>
-      </c>
+      <c r="C15" s="5"/>
       <c r="D15" s="5"/>
-      <c r="E15" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="E15" s="5"/>
       <c r="F15" s="5"/>
-      <c r="G15" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="G15" s="5"/>
       <c r="H15" s="5"/>
-      <c r="I15" s="5" t="s">
-        <v>31</v>
-      </c>
+      <c r="I15" s="5"/>
       <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
+      <c r="K15" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
@@ -1425,11 +1424,11 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="5" t="s">
-        <v>32</v>
-      </c>
+      <c r="G16" s="5"/>
       <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
+      <c r="I16" s="5" t="s">
+        <v>20</v>
+      </c>
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
@@ -1449,11 +1448,11 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
-      <c r="G17" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="G17" s="5"/>
       <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
+      <c r="I17" s="5" t="s">
+        <v>30</v>
+      </c>
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
@@ -1466,31 +1465,109 @@
       <c r="S17" s="5"/>
       <c r="T17" s="5"/>
     </row>
-    <row r="18" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
-      <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
+    <row r="18" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="5"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="5"/>
+      <c r="S18" s="5"/>
+      <c r="T18" s="5"/>
+    </row>
+    <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="5"/>
+      <c r="Q19" s="5"/>
+      <c r="R19" s="5"/>
+      <c r="S19" s="5"/>
+      <c r="T19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="5"/>
+      <c r="T20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="98">
+  <mergeCells count="113">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -1504,10 +1581,10 @@
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="Q4:R4"/>
     <mergeCell ref="S4:T4"/>
-    <mergeCell ref="A5:B17"/>
-    <mergeCell ref="C5:D14"/>
-    <mergeCell ref="E5:F14"/>
-    <mergeCell ref="G5:H14"/>
+    <mergeCell ref="A5:B20"/>
+    <mergeCell ref="C5:D17"/>
+    <mergeCell ref="E5:F17"/>
+    <mergeCell ref="G5:H17"/>
     <mergeCell ref="I5:J7"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="M5:N5"/>
@@ -1524,30 +1601,28 @@
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="Q7:R7"/>
     <mergeCell ref="S7:T7"/>
-    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I8:J11"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="M8:N8"/>
     <mergeCell ref="O8:P8"/>
     <mergeCell ref="Q8:R8"/>
     <mergeCell ref="S8:T8"/>
-    <mergeCell ref="I9:J9"/>
     <mergeCell ref="K9:L9"/>
     <mergeCell ref="M9:N9"/>
     <mergeCell ref="O9:P9"/>
     <mergeCell ref="Q9:R9"/>
     <mergeCell ref="S9:T9"/>
-    <mergeCell ref="I10:J10"/>
     <mergeCell ref="K10:L10"/>
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="O10:P10"/>
     <mergeCell ref="Q10:R10"/>
     <mergeCell ref="S10:T10"/>
-    <mergeCell ref="I11:J12"/>
     <mergeCell ref="K11:L11"/>
     <mergeCell ref="M11:N11"/>
     <mergeCell ref="O11:P11"/>
     <mergeCell ref="Q11:R11"/>
     <mergeCell ref="S11:T11"/>
+    <mergeCell ref="I12:J12"/>
     <mergeCell ref="K12:L12"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="O12:P12"/>
@@ -1559,36 +1634,53 @@
     <mergeCell ref="O13:P13"/>
     <mergeCell ref="Q13:R13"/>
     <mergeCell ref="S13:T13"/>
-    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I14:J15"/>
     <mergeCell ref="K14:L14"/>
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="O14:P14"/>
     <mergeCell ref="Q14:R14"/>
     <mergeCell ref="S14:T14"/>
-    <mergeCell ref="C15:D17"/>
-    <mergeCell ref="E15:F17"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:J15"/>
     <mergeCell ref="K15:L15"/>
     <mergeCell ref="M15:N15"/>
     <mergeCell ref="O15:P15"/>
     <mergeCell ref="Q15:R15"/>
     <mergeCell ref="S15:T15"/>
-    <mergeCell ref="G16:H16"/>
     <mergeCell ref="I16:J16"/>
     <mergeCell ref="K16:L16"/>
     <mergeCell ref="M16:N16"/>
     <mergeCell ref="O16:P16"/>
     <mergeCell ref="Q16:R16"/>
     <mergeCell ref="S16:T16"/>
-    <mergeCell ref="G17:H17"/>
     <mergeCell ref="I17:J17"/>
     <mergeCell ref="K17:L17"/>
     <mergeCell ref="M17:N17"/>
     <mergeCell ref="O17:P17"/>
     <mergeCell ref="Q17:R17"/>
     <mergeCell ref="S17:T17"/>
-    <mergeCell ref="A18:U18"/>
+    <mergeCell ref="C18:D20"/>
+    <mergeCell ref="E18:F20"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:R18"/>
+    <mergeCell ref="S18:T18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="Q19:R19"/>
+    <mergeCell ref="S19:T19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="Q20:R20"/>
+    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="A21:U21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1610,7 +1702,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1658,7 +1750,7 @@
     </row>
     <row r="3" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1683,7 +1775,7 @@
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1708,19 +1800,19 @@
     </row>
     <row r="5" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
@@ -1730,12 +1822,12 @@
       <c r="M5" s="4"/>
       <c r="N5" s="4"/>
       <c r="O5" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
       <c r="R5" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
@@ -1746,16 +1838,16 @@
         <v>1</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
@@ -1777,16 +1869,16 @@
         <v>2</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
       <c r="E7" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
@@ -1808,16 +1900,16 @@
         <v>3</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="8"/>
@@ -1839,16 +1931,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
@@ -1858,7 +1950,7 @@
       <c r="M9" s="11"/>
       <c r="N9" s="11"/>
       <c r="O9" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
@@ -1872,16 +1964,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
@@ -1903,16 +1995,16 @@
         <v>6</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F11" s="11"/>
       <c r="G11" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H11" s="11"/>
       <c r="I11" s="11"/>
@@ -1934,16 +2026,16 @@
         <v>7</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F12" s="11"/>
       <c r="G12" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
@@ -1965,16 +2057,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H13" s="11"/>
       <c r="I13" s="11"/>
@@ -1996,16 +2088,16 @@
         <v>9</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F14" s="11"/>
       <c r="G14" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
@@ -2027,16 +2119,16 @@
         <v>10</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
       <c r="E15" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -2058,16 +2150,16 @@
         <v>11</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
@@ -2077,7 +2169,7 @@
       <c r="M16" s="13"/>
       <c r="N16" s="13"/>
       <c r="O16" s="13" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
@@ -2091,16 +2183,16 @@
         <v>12</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
       <c r="E17" s="13" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H17" s="13"/>
       <c r="I17" s="13"/>
@@ -2122,16 +2214,16 @@
         <v>13</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F18" s="13"/>
       <c r="G18" s="13" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
@@ -2153,16 +2245,16 @@
         <v>14</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
       <c r="E19" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F19" s="13"/>
       <c r="G19" s="13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H19" s="13"/>
       <c r="I19" s="13"/>
@@ -2184,16 +2276,16 @@
         <v>15</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F20" s="13"/>
       <c r="G20" s="13" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
@@ -2215,16 +2307,16 @@
         <v>16</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
       <c r="E21" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H21" s="13"/>
       <c r="I21" s="13"/>
@@ -2246,16 +2338,16 @@
         <v>17</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H22" s="13"/>
       <c r="I22" s="13"/>
@@ -2277,16 +2369,16 @@
         <v>18</v>
       </c>
       <c r="B23" s="13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H23" s="13"/>
       <c r="I23" s="13"/>
@@ -2328,7 +2420,7 @@
     </row>
     <row r="25" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -2353,19 +2445,19 @@
     </row>
     <row r="26" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
       <c r="E26" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
@@ -2375,7 +2467,7 @@
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
       <c r="O26" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
@@ -2385,16 +2477,16 @@
         <v>1</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
       <c r="E27" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F27" s="11"/>
       <c r="G27" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H27" s="11"/>
       <c r="I27" s="11"/>
@@ -2404,7 +2496,7 @@
       <c r="M27" s="11"/>
       <c r="N27" s="11"/>
       <c r="O27" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P27" s="11"/>
       <c r="Q27" s="11"/>
@@ -2434,7 +2526,7 @@
     </row>
     <row r="29" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -2459,19 +2551,19 @@
     </row>
     <row r="30" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H30" s="4"/>
       <c r="I30" s="4"/>
@@ -2481,7 +2573,7 @@
       <c r="M30" s="4"/>
       <c r="N30" s="4"/>
       <c r="O30" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
@@ -2491,16 +2583,16 @@
         <v>1</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
       <c r="E31" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F31" s="11"/>
       <c r="G31" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H31" s="11"/>
       <c r="I31" s="11"/>
@@ -2510,7 +2602,7 @@
       <c r="M31" s="11"/>
       <c r="N31" s="11"/>
       <c r="O31" s="11" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="P31" s="11"/>
       <c r="Q31" s="11"/>
@@ -2540,7 +2632,7 @@
     </row>
     <row r="33" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
@@ -2565,7 +2657,7 @@
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -2590,30 +2682,30 @@
     </row>
     <row r="35" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
       <c r="K35" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="4"/>
       <c r="N35" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="O35" s="4"/>
       <c r="P35" s="4"/>
@@ -2628,31 +2720,31 @@
         <v>1</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
       <c r="K36" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
       <c r="N36" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="O36" s="5"/>
       <c r="P36" s="5"/>
@@ -2671,12 +2763,12 @@
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="L37" s="5"/>
       <c r="M37" s="5"/>
@@ -2698,12 +2790,12 @@
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
@@ -2725,12 +2817,12 @@
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
       <c r="K39" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -2752,12 +2844,12 @@
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
@@ -2775,7 +2867,7 @@
         <v>2</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -2783,17 +2875,17 @@
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
       <c r="N41" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="O41" s="5"/>
       <c r="P41" s="5"/>
@@ -2812,12 +2904,12 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
@@ -2839,12 +2931,12 @@
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
@@ -2866,12 +2958,12 @@
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="L44" s="5"/>
       <c r="M44" s="5"/>
@@ -2893,12 +2985,12 @@
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
       <c r="H45" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
@@ -2920,12 +3012,12 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
@@ -2947,12 +3039,12 @@
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
       <c r="H47" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
@@ -2970,27 +3062,27 @@
         <v>3</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
       <c r="E48" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
       <c r="H48" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
       <c r="K48" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
       <c r="N48" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="O48" s="5"/>
       <c r="P48" s="5"/>
@@ -3009,12 +3101,12 @@
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
       <c r="H49" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L49" s="5"/>
       <c r="M49" s="5"/>
@@ -3036,12 +3128,12 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I50" s="5"/>
       <c r="J50" s="5"/>
       <c r="K50" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
@@ -3063,12 +3155,12 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I51" s="5"/>
       <c r="J51" s="5"/>
       <c r="K51" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
@@ -3086,13 +3178,13 @@
         <v>4</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E52" s="5" t="s">
         <v>18</v>
@@ -3100,25 +3192,25 @@
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
       <c r="H52" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J52" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K52" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="O52" s="5"/>
       <c r="P52" s="5"/>
@@ -3137,22 +3229,22 @@
       <c r="F53" s="5"/>
       <c r="G53" s="5"/>
       <c r="H53" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J53" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K53" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L53" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N53" s="5"/>
       <c r="O53" s="5"/>
@@ -3172,22 +3264,22 @@
       <c r="F54" s="5"/>
       <c r="G54" s="5"/>
       <c r="H54" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J54" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K54" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N54" s="5"/>
       <c r="O54" s="5"/>
@@ -3223,7 +3315,7 @@
     </row>
     <row r="56" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -3256,30 +3348,30 @@
     </row>
     <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
       <c r="H57" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
       <c r="K57" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L57" s="4"/>
       <c r="M57" s="4"/>
       <c r="N57" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="O57" s="4"/>
       <c r="P57" s="4"/>
@@ -3295,7 +3387,7 @@
       <c r="Z57" s="4"/>
       <c r="AA57" s="4"/>
       <c r="AB57" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AC57" s="4"/>
     </row>
@@ -3314,35 +3406,35 @@
       <c r="L58" s="4"/>
       <c r="M58" s="4"/>
       <c r="N58" s="15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="O58" s="15"/>
       <c r="P58" s="15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q58" s="15"/>
       <c r="R58" s="15" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="S58" s="15"/>
       <c r="T58" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="U58" s="15"/>
       <c r="V58" s="15" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="W58" s="15"/>
       <c r="X58" s="15" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="Y58" s="15"/>
       <c r="Z58" s="15" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="AA58" s="15"/>
       <c r="AB58" s="15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="AC58" s="15"/>
     </row>
@@ -3351,31 +3443,31 @@
         <v>1</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F59" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H59" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J59" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K59" s="5" t="n">
         <v>1</v>
@@ -3383,24 +3475,26 @@
       <c r="L59" s="5"/>
       <c r="M59" s="5"/>
       <c r="N59" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="O59" s="5"/>
-      <c r="P59" s="5" t="s">
-        <v>162</v>
-      </c>
+      <c r="P59" s="5"/>
       <c r="Q59" s="5"/>
-      <c r="R59" s="5" t="s">
-        <v>163</v>
-      </c>
+      <c r="R59" s="5"/>
       <c r="S59" s="5"/>
       <c r="T59" s="5"/>
       <c r="U59" s="5"/>
-      <c r="V59" s="5"/>
+      <c r="V59" s="5" t="s">
+        <v>164</v>
+      </c>
       <c r="W59" s="5"/>
-      <c r="X59" s="5"/>
+      <c r="X59" s="5" t="s">
+        <v>165</v>
+      </c>
       <c r="Y59" s="5"/>
-      <c r="Z59" s="5"/>
+      <c r="Z59" s="5" t="s">
+        <v>166</v>
+      </c>
       <c r="AA59" s="5"/>
       <c r="AB59" s="5"/>
       <c r="AC59" s="5"/>
@@ -3430,7 +3524,7 @@
     </row>
     <row r="61" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -3455,21 +3549,21 @@
     </row>
     <row r="62" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
       <c r="H62" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="I62" s="4"/>
       <c r="J62" s="4"/>
@@ -3482,21 +3576,21 @@
       <c r="B63" s="16"/>
       <c r="C63" s="9"/>
       <c r="D63" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
       <c r="H63" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J63" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K63" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3506,21 +3600,21 @@
       <c r="B64" s="16"/>
       <c r="C64" s="16"/>
       <c r="D64" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
       <c r="H64" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="J64" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="K64" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3530,7 +3624,7 @@
       <c r="B65" s="17"/>
       <c r="C65" s="9"/>
       <c r="D65" s="5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
@@ -3546,13 +3640,13 @@
       <c r="B66" s="17"/>
       <c r="C66" s="17"/>
       <c r="D66" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
       <c r="H66" s="18"/>
       <c r="I66" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="J66" s="5"/>
       <c r="K66" s="18"/>
@@ -3564,7 +3658,7 @@
       <c r="B67" s="19"/>
       <c r="C67" s="9"/>
       <c r="D67" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
@@ -3578,7 +3672,7 @@
       <c r="B68" s="19"/>
       <c r="C68" s="19"/>
       <c r="D68" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E68" s="5"/>
       <c r="F68" s="5"/>
@@ -3590,7 +3684,7 @@
       <c r="B69" s="20"/>
       <c r="C69" s="9"/>
       <c r="D69" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
@@ -3602,7 +3696,7 @@
       <c r="B70" s="20"/>
       <c r="C70" s="20"/>
       <c r="D70" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
@@ -3632,7 +3726,7 @@
     </row>
     <row r="72" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B72" s="14"/>
       <c r="C72" s="14"/>
@@ -3657,7 +3751,7 @@
     </row>
     <row r="73" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B73" s="6"/>
       <c r="C73" s="6"/>
@@ -3682,30 +3776,30 @@
     </row>
     <row r="74" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C74" s="4"/>
       <c r="D74" s="4"/>
       <c r="E74" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F74" s="4"/>
       <c r="G74" s="4"/>
       <c r="H74" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I74" s="4"/>
       <c r="J74" s="4"/>
       <c r="K74" s="4" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="L74" s="4"/>
       <c r="M74" s="4"/>
       <c r="N74" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="O74" s="4"/>
       <c r="P74" s="4"/>
@@ -3720,35 +3814,35 @@
         <v>1</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
       <c r="E75" s="5" t="s">
-        <v>176</v>
+        <v>22</v>
       </c>
       <c r="F75" s="5"/>
       <c r="G75" s="5"/>
       <c r="H75" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I75" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J75" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K75" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L75" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M75" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N75" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="O75" s="5"/>
       <c r="P75" s="5"/>
@@ -3767,22 +3861,22 @@
       <c r="F76" s="5"/>
       <c r="G76" s="5"/>
       <c r="H76" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I76" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J76" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K76" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L76" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N76" s="5"/>
       <c r="O76" s="5"/>
@@ -3802,22 +3896,22 @@
       <c r="F77" s="5"/>
       <c r="G77" s="5"/>
       <c r="H77" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I77" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J77" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="L77" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="M77" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="N77" s="5"/>
       <c r="O77" s="5"/>
@@ -3853,7 +3947,7 @@
     </row>
     <row r="79" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B79" s="6"/>
       <c r="C79" s="6"/>
@@ -3886,30 +3980,30 @@
     </row>
     <row r="80" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
       <c r="E80" s="4" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F80" s="4"/>
       <c r="G80" s="4"/>
       <c r="H80" s="4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I80" s="4"/>
       <c r="J80" s="4"/>
       <c r="K80" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L80" s="4"/>
       <c r="M80" s="4"/>
       <c r="N80" s="4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="O80" s="4"/>
       <c r="P80" s="4"/>
@@ -3925,7 +4019,7 @@
       <c r="Z80" s="4"/>
       <c r="AA80" s="4"/>
       <c r="AB80" s="4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AC80" s="4"/>
     </row>
@@ -3944,35 +4038,35 @@
       <c r="L81" s="4"/>
       <c r="M81" s="4"/>
       <c r="N81" s="15" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="O81" s="15"/>
       <c r="P81" s="15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="Q81" s="15"/>
       <c r="R81" s="15" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="S81" s="15"/>
       <c r="T81" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="U81" s="15"/>
       <c r="V81" s="15" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="W81" s="15"/>
       <c r="X81" s="15" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="Y81" s="15"/>
       <c r="Z81" s="15" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="AA81" s="15"/>
       <c r="AB81" s="15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="AC81" s="15"/>
     </row>
@@ -3981,31 +4075,31 @@
         <v>1</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F82" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G82" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H82" s="5" t="n">
         <v>1</v>
       </c>
       <c r="I82" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="J82" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K82" s="5" t="n">
         <v>1</v>
@@ -4013,24 +4107,24 @@
       <c r="L82" s="5"/>
       <c r="M82" s="5"/>
       <c r="N82" s="5" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="O82" s="5"/>
-      <c r="P82" s="5" t="s">
-        <v>179</v>
-      </c>
+      <c r="P82" s="5"/>
       <c r="Q82" s="5"/>
-      <c r="R82" s="5" t="s">
-        <v>163</v>
-      </c>
+      <c r="R82" s="5"/>
       <c r="S82" s="5"/>
       <c r="T82" s="5"/>
       <c r="U82" s="5"/>
       <c r="V82" s="5"/>
       <c r="W82" s="5"/>
-      <c r="X82" s="5"/>
+      <c r="X82" s="5" t="s">
+        <v>180</v>
+      </c>
       <c r="Y82" s="5"/>
-      <c r="Z82" s="5"/>
+      <c r="Z82" s="5" t="s">
+        <v>166</v>
+      </c>
       <c r="AA82" s="5"/>
       <c r="AB82" s="5"/>
       <c r="AC82" s="5"/>
@@ -4059,7 +4153,7 @@
       <c r="U83" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="232">
+  <mergeCells count="233">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -4232,9 +4326,10 @@
     <mergeCell ref="E59:G59"/>
     <mergeCell ref="H59:J59"/>
     <mergeCell ref="K59:M59"/>
-    <mergeCell ref="N59:O59"/>
-    <mergeCell ref="P59:Q59"/>
-    <mergeCell ref="R59:AC59"/>
+    <mergeCell ref="N59:U59"/>
+    <mergeCell ref="V59:W59"/>
+    <mergeCell ref="X59:Y59"/>
+    <mergeCell ref="Z59:AC59"/>
     <mergeCell ref="A60:U60"/>
     <mergeCell ref="A61:U61"/>
     <mergeCell ref="D62:F62"/>
@@ -4288,9 +4383,9 @@
     <mergeCell ref="E82:G82"/>
     <mergeCell ref="H82:J82"/>
     <mergeCell ref="K82:M82"/>
-    <mergeCell ref="N82:O82"/>
-    <mergeCell ref="P82:Q82"/>
-    <mergeCell ref="R82:AC82"/>
+    <mergeCell ref="N82:W82"/>
+    <mergeCell ref="X82:Y82"/>
+    <mergeCell ref="Z82:AC82"/>
     <mergeCell ref="A83:U83"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
[ Version 0.0.28.9 ] - roulette files was modified only for one roulette.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="172">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -254,15 +254,6 @@
     <t xml:space="preserve">ROULETTE</t>
   </si>
   <si>
-    <t xml:space="preserve">OUT_ROULETTE_EN2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO for roulette R2 motor driver enable pin – enable 2.</t>
-  </si>
-  <si>
     <t xml:space="preserve">OUT_ROULETTE_DIR1</t>
   </si>
   <si>
@@ -290,15 +281,6 @@
     <t xml:space="preserve">DI for roulette R1 open position end switches – end switch open 1.</t>
   </si>
   <si>
-    <t xml:space="preserve">IN_ROULETTE_ESO2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R2 open position end switches – end switch open 2.</t>
-  </si>
-  <si>
     <t xml:space="preserve">IN_ROULETTE_ESC1</t>
   </si>
   <si>
@@ -306,15 +288,6 @@
   </si>
   <si>
     <t xml:space="preserve">DI for roulette R1 close position end switches – end switch close 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IN_ROULETTE_ESC2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPIO26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DI for roulette R2 close position end switches – end switch close 2.</t>
   </si>
   <si>
     <t xml:space="preserve">ESP-IDF TIMERS</t>
@@ -1697,7 +1670,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC83"/>
+  <dimension ref="A1:AC80"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2180,7 +2153,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B17" s="13" t="s">
         <v>77</v>
@@ -2211,7 +2184,7 @@
     </row>
     <row r="18" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>80</v>
@@ -2242,7 +2215,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>83</v>
@@ -2273,7 +2246,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>86</v>
@@ -2302,450 +2275,438 @@
       <c r="T20" s="13"/>
       <c r="U20" s="13"/>
     </row>
-    <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="13" t="s">
+    <row r="21" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="2"/>
+      <c r="T21" s="2"/>
+      <c r="U21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13" t="s">
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6"/>
+      <c r="K22" s="6"/>
+      <c r="L22" s="6"/>
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6"/>
+      <c r="Q22" s="6"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="6"/>
+      <c r="T22" s="6"/>
+      <c r="U22" s="6"/>
+    </row>
+    <row r="23" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P23" s="4"/>
+      <c r="Q23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13" t="s">
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="13"/>
-      <c r="R21" s="13"/>
-      <c r="S21" s="13"/>
-      <c r="T21" s="13"/>
-      <c r="U21" s="13"/>
-    </row>
-    <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="13" t="s">
+      <c r="F24" s="11"/>
+      <c r="G24" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13" t="s">
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="P24" s="11"/>
+      <c r="Q24" s="11"/>
+    </row>
+    <row r="25" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
+      <c r="T25" s="2"/>
+      <c r="U25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13" t="s">
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="6"/>
+      <c r="P26" s="6"/>
+      <c r="Q26" s="6"/>
+      <c r="R26" s="6"/>
+      <c r="S26" s="6"/>
+      <c r="T26" s="6"/>
+      <c r="U26" s="6"/>
+    </row>
+    <row r="27" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P27" s="4"/>
+      <c r="Q27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="13"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="13"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
-      <c r="T22" s="13"/>
-      <c r="U22" s="13"/>
-    </row>
-    <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="13" t="s">
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13" t="s">
+      <c r="F28" s="11"/>
+      <c r="G28" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13" t="s">
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="11"/>
+      <c r="M28" s="11"/>
+      <c r="N28" s="11"/>
+      <c r="O28" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="P28" s="11"/>
+      <c r="Q28" s="11"/>
+    </row>
+    <row r="29" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
+      <c r="N29" s="2"/>
+      <c r="O29" s="2"/>
+      <c r="P29" s="2"/>
+      <c r="Q29" s="2"/>
+      <c r="R29" s="2"/>
+      <c r="S29" s="2"/>
+      <c r="T29" s="2"/>
+      <c r="U29" s="2"/>
+    </row>
+    <row r="30" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="13"/>
-      <c r="R23" s="13"/>
-      <c r="S23" s="13"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="13"/>
-    </row>
-    <row r="24" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-    </row>
-    <row r="25" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
+      <c r="O30" s="14"/>
+      <c r="P30" s="14"/>
+      <c r="Q30" s="14"/>
+      <c r="R30" s="14"/>
+      <c r="S30" s="14"/>
+      <c r="T30" s="14"/>
+      <c r="U30" s="14"/>
+    </row>
+    <row r="31" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
-      <c r="Q25" s="6"/>
-      <c r="R25" s="6"/>
-      <c r="S25" s="6"/>
-      <c r="T25" s="6"/>
-      <c r="U25" s="6"/>
-    </row>
-    <row r="26" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6"/>
+      <c r="M31" s="6"/>
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6"/>
+      <c r="R31" s="6"/>
+      <c r="S31" s="6"/>
+      <c r="T31" s="6"/>
+      <c r="U31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B32" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4" t="s">
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="P26" s="4"/>
-      <c r="Q26" s="4"/>
-    </row>
-    <row r="27" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="n">
+      <c r="O32" s="4"/>
+      <c r="P32" s="4"/>
+      <c r="Q32" s="4"/>
+      <c r="R32" s="4"/>
+      <c r="S32" s="4"/>
+      <c r="T32" s="4"/>
+      <c r="U32" s="4"/>
+    </row>
+    <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11" t="s">
-        <v>100</v>
-      </c>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-      <c r="N27" s="11"/>
-      <c r="O27" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="P27" s="11"/>
-      <c r="Q27" s="11"/>
-    </row>
-    <row r="28" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-      <c r="R28" s="2"/>
-      <c r="S28" s="2"/>
-      <c r="T28" s="2"/>
-      <c r="U28" s="2"/>
-    </row>
-    <row r="29" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
+      <c r="B33" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
-      <c r="M29" s="6"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="6"/>
-      <c r="Q29" s="6"/>
-      <c r="R29" s="6"/>
-      <c r="S29" s="6"/>
-      <c r="T29" s="6"/>
-      <c r="U29" s="6"/>
-    </row>
-    <row r="30" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="P30" s="4"/>
-      <c r="Q30" s="4"/>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" s="11" t="s">
+      <c r="C33" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11" t="s">
+      <c r="D33" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11" t="s">
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="H31" s="11"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="11"/>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11"/>
-      <c r="O31" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="P31" s="11"/>
-      <c r="Q31" s="11"/>
-    </row>
-    <row r="32" customFormat="false" ht="43.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-      <c r="R32" s="2"/>
-      <c r="S32" s="2"/>
-      <c r="T32" s="2"/>
-      <c r="U32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="14"/>
-      <c r="O33" s="14"/>
-      <c r="P33" s="14"/>
-      <c r="Q33" s="14"/>
-      <c r="R33" s="14"/>
-      <c r="S33" s="14"/>
-      <c r="T33" s="14"/>
-      <c r="U33" s="14"/>
-    </row>
-    <row r="34" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="6"/>
-      <c r="M34" s="6"/>
-      <c r="N34" s="6"/>
-      <c r="O34" s="6"/>
-      <c r="P34" s="6"/>
-      <c r="Q34" s="6"/>
-      <c r="R34" s="6"/>
-      <c r="S34" s="6"/>
-      <c r="T34" s="6"/>
-      <c r="U34" s="6"/>
-    </row>
-    <row r="35" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4" t="s">
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+    </row>
+    <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="9"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4" t="s">
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4" t="s">
+      <c r="L34" s="5"/>
+      <c r="M34" s="5"/>
+      <c r="N34" s="5"/>
+      <c r="O34" s="5"/>
+      <c r="P34" s="5"/>
+      <c r="Q34" s="5"/>
+      <c r="R34" s="5"/>
+      <c r="S34" s="5"/>
+      <c r="T34" s="5"/>
+      <c r="U34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="9"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="O35" s="4"/>
-      <c r="P35" s="4"/>
-      <c r="Q35" s="4"/>
-      <c r="R35" s="4"/>
-      <c r="S35" s="4"/>
-      <c r="T35" s="4"/>
-      <c r="U35" s="4"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="L35" s="5"/>
+      <c r="M35" s="5"/>
+      <c r="N35" s="5"/>
+      <c r="O35" s="5"/>
+      <c r="P35" s="5"/>
+      <c r="Q35" s="5"/>
+      <c r="R35" s="5"/>
+      <c r="S35" s="5"/>
+      <c r="T35" s="5"/>
+      <c r="U35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>113</v>
-      </c>
+      <c r="A36" s="9"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
       <c r="H36" s="5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
       <c r="K36" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
-      <c r="N36" s="5" t="s">
-        <v>116</v>
-      </c>
+      <c r="N36" s="5"/>
       <c r="O36" s="5"/>
       <c r="P36" s="5"/>
       <c r="Q36" s="5"/>
@@ -2763,12 +2724,12 @@
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
       <c r="H37" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
       <c r="K37" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="L37" s="5"/>
       <c r="M37" s="5"/>
@@ -2782,24 +2743,30 @@
       <c r="U37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9"/>
-      <c r="B38" s="5"/>
+      <c r="A38" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>116</v>
+      </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
       <c r="H38" s="5" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
       <c r="K38" s="5" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
-      <c r="N38" s="5"/>
+      <c r="N38" s="5" t="s">
+        <v>117</v>
+      </c>
       <c r="O38" s="5"/>
       <c r="P38" s="5"/>
       <c r="Q38" s="5"/>
@@ -2817,12 +2784,12 @@
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
       <c r="H39" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
       <c r="K39" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -2844,12 +2811,12 @@
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
       <c r="H40" s="5" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
       <c r="K40" s="5" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
@@ -2863,30 +2830,24 @@
       <c r="U40" s="5"/>
     </row>
     <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>125</v>
-      </c>
+      <c r="A41" s="9"/>
+      <c r="B41" s="5"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
       <c r="K41" s="5" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
-      <c r="N41" s="5" t="s">
-        <v>126</v>
-      </c>
+      <c r="N41" s="5"/>
       <c r="O41" s="5"/>
       <c r="P41" s="5"/>
       <c r="Q41" s="5"/>
@@ -2904,12 +2865,12 @@
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
       <c r="H42" s="5" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
       <c r="K42" s="5" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
@@ -2931,12 +2892,12 @@
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
       <c r="H43" s="5" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
       <c r="K43" s="5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
@@ -2958,12 +2919,12 @@
       <c r="F44" s="5"/>
       <c r="G44" s="5"/>
       <c r="H44" s="5" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
       <c r="K44" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="L44" s="5"/>
       <c r="M44" s="5"/>
@@ -2977,24 +2938,32 @@
       <c r="U44" s="5"/>
     </row>
     <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="9"/>
-      <c r="B45" s="5"/>
+      <c r="A45" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>127</v>
+      </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
+      <c r="E45" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
       <c r="H45" s="5" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
       <c r="K45" s="5" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
-      <c r="N45" s="5"/>
+      <c r="N45" s="5" t="s">
+        <v>129</v>
+      </c>
       <c r="O45" s="5"/>
       <c r="P45" s="5"/>
       <c r="Q45" s="5"/>
@@ -3012,12 +2981,12 @@
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
       <c r="H46" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
@@ -3039,12 +3008,12 @@
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
       <c r="H47" s="5" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
       <c r="K47" s="5" t="s">
-        <v>135</v>
+        <v>113</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
@@ -3058,32 +3027,24 @@
       <c r="U47" s="5"/>
     </row>
     <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>136</v>
-      </c>
+      <c r="A48" s="9"/>
+      <c r="B48" s="5"/>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
-      <c r="E48" s="5" t="s">
-        <v>33</v>
-      </c>
+      <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
       <c r="H48" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
       <c r="K48" s="5" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
-      <c r="N48" s="5" t="s">
-        <v>138</v>
-      </c>
+      <c r="N48" s="5"/>
       <c r="O48" s="5"/>
       <c r="P48" s="5"/>
       <c r="Q48" s="5"/>
@@ -3093,24 +3054,44 @@
       <c r="U48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="9"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
+      <c r="A49" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>18</v>
+      </c>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
       <c r="H49" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
+        <v>132</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="K49" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="L49" s="5"/>
-      <c r="M49" s="5"/>
-      <c r="N49" s="5"/>
+        <v>133</v>
+      </c>
+      <c r="L49" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M49" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="N49" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="O49" s="5"/>
       <c r="P49" s="5"/>
       <c r="Q49" s="5"/>
@@ -3128,15 +3109,23 @@
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
       <c r="H50" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="I50" s="5"/>
-      <c r="J50" s="5"/>
+        <v>135</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="K50" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="L50" s="5"/>
-      <c r="M50" s="5"/>
+        <v>136</v>
+      </c>
+      <c r="L50" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M50" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="N50" s="5"/>
       <c r="O50" s="5"/>
       <c r="P50" s="5"/>
@@ -3155,15 +3144,23 @@
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
       <c r="H51" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
+        <v>137</v>
+      </c>
+      <c r="I51" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="K51" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="L51" s="5"/>
-      <c r="M51" s="5"/>
+        <v>138</v>
+      </c>
+      <c r="L51" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M51" s="5" t="s">
+        <v>103</v>
+      </c>
       <c r="N51" s="5"/>
       <c r="O51" s="5"/>
       <c r="P51" s="5"/>
@@ -3173,987 +3170,870 @@
       <c r="T51" s="5"/>
       <c r="U51" s="5"/>
     </row>
-    <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="9" t="n">
+    <row r="52" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="2"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+      <c r="O52" s="2"/>
+      <c r="P52" s="2"/>
+      <c r="Q52" s="2"/>
+      <c r="R52" s="2"/>
+      <c r="S52" s="2"/>
+      <c r="T52" s="2"/>
+      <c r="U52" s="2"/>
+    </row>
+    <row r="53" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B53" s="6"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="6"/>
+      <c r="N53" s="6"/>
+      <c r="O53" s="6"/>
+      <c r="P53" s="6"/>
+      <c r="Q53" s="6"/>
+      <c r="R53" s="6"/>
+      <c r="S53" s="6"/>
+      <c r="T53" s="6"/>
+      <c r="U53" s="6"/>
+      <c r="V53" s="6"/>
+      <c r="W53" s="6"/>
+      <c r="X53" s="6"/>
+      <c r="Y53" s="6"/>
+      <c r="Z53" s="6"/>
+      <c r="AA53" s="6"/>
+      <c r="AB53" s="6"/>
+      <c r="AC53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="O54" s="4"/>
+      <c r="P54" s="4"/>
+      <c r="Q54" s="4"/>
+      <c r="R54" s="4"/>
+      <c r="S54" s="4"/>
+      <c r="T54" s="4"/>
+      <c r="U54" s="4"/>
+      <c r="V54" s="4"/>
+      <c r="W54" s="4"/>
+      <c r="X54" s="4"/>
+      <c r="Y54" s="4"/>
+      <c r="Z54" s="4"/>
+      <c r="AA54" s="4"/>
+      <c r="AB54" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="AC54" s="4"/>
+    </row>
+    <row r="55" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="4"/>
+      <c r="K55" s="4"/>
+      <c r="L55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="O55" s="15"/>
+      <c r="P55" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q55" s="15"/>
+      <c r="R55" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="S55" s="15"/>
+      <c r="T55" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="U55" s="15"/>
+      <c r="V55" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="W55" s="15"/>
+      <c r="X55" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y55" s="15"/>
+      <c r="Z55" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA55" s="15"/>
+      <c r="AB55" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="AC55" s="15"/>
+    </row>
+    <row r="56" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J56" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="K56" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L56" s="5"/>
+      <c r="M56" s="5"/>
+      <c r="N56" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="O56" s="5"/>
+      <c r="P56" s="5"/>
+      <c r="Q56" s="5"/>
+      <c r="R56" s="5"/>
+      <c r="S56" s="5"/>
+      <c r="T56" s="5"/>
+      <c r="U56" s="5"/>
+      <c r="V56" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="W56" s="5"/>
+      <c r="X56" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="Y56" s="5"/>
+      <c r="Z56" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="AA56" s="5"/>
+      <c r="AB56" s="5"/>
+      <c r="AC56" s="5"/>
+    </row>
+    <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
+      <c r="L57" s="2"/>
+      <c r="M57" s="2"/>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" s="2"/>
+      <c r="Q57" s="2"/>
+      <c r="R57" s="2"/>
+      <c r="S57" s="2"/>
+      <c r="T57" s="2"/>
+      <c r="U57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6"/>
+      <c r="K58" s="6"/>
+      <c r="L58" s="6"/>
+      <c r="M58" s="6"/>
+      <c r="N58" s="6"/>
+      <c r="O58" s="6"/>
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6"/>
+      <c r="R58" s="6"/>
+      <c r="S58" s="6"/>
+      <c r="T58" s="6"/>
+      <c r="U58" s="6"/>
+    </row>
+    <row r="59" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="H59" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="I59" s="4"/>
+      <c r="J59" s="4"/>
+      <c r="K59" s="4"/>
+    </row>
+    <row r="60" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B60" s="16"/>
+      <c r="C60" s="9"/>
+      <c r="D60" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="H60" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="J60" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="K60" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B61" s="16"/>
+      <c r="C61" s="16"/>
+      <c r="D61" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="H61" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I61" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="J61" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="K61" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B62" s="17"/>
+      <c r="C62" s="9"/>
+      <c r="D62" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E62" s="5"/>
+      <c r="F62" s="5"/>
+      <c r="H62" s="18"/>
+      <c r="I62" s="18"/>
+      <c r="J62" s="18"/>
+      <c r="K62" s="18"/>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B52" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E52" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="I52" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J52" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K52" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="L52" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="M52" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N52" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="O52" s="5"/>
-      <c r="P52" s="5"/>
-      <c r="Q52" s="5"/>
-      <c r="R52" s="5"/>
-      <c r="S52" s="5"/>
-      <c r="T52" s="5"/>
-      <c r="U52" s="5"/>
-    </row>
-    <row r="53" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="9"/>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="I53" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J53" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K53" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="L53" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="M53" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N53" s="5"/>
-      <c r="O53" s="5"/>
-      <c r="P53" s="5"/>
-      <c r="Q53" s="5"/>
-      <c r="R53" s="5"/>
-      <c r="S53" s="5"/>
-      <c r="T53" s="5"/>
-      <c r="U53" s="5"/>
-    </row>
-    <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="9"/>
-      <c r="B54" s="5"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="5"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I54" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J54" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K54" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="L54" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="M54" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N54" s="5"/>
-      <c r="O54" s="5"/>
-      <c r="P54" s="5"/>
-      <c r="Q54" s="5"/>
-      <c r="R54" s="5"/>
-      <c r="S54" s="5"/>
-      <c r="T54" s="5"/>
-      <c r="U54" s="5"/>
-    </row>
-    <row r="55" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
-      <c r="L55" s="2"/>
-      <c r="M55" s="2"/>
-      <c r="N55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="P55" s="2"/>
-      <c r="Q55" s="2"/>
-      <c r="R55" s="2"/>
-      <c r="S55" s="2"/>
-      <c r="T55" s="2"/>
-      <c r="U55" s="2"/>
-    </row>
-    <row r="56" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="B56" s="6"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="6"/>
-      <c r="F56" s="6"/>
-      <c r="G56" s="6"/>
-      <c r="H56" s="6"/>
-      <c r="I56" s="6"/>
-      <c r="J56" s="6"/>
-      <c r="K56" s="6"/>
-      <c r="L56" s="6"/>
-      <c r="M56" s="6"/>
-      <c r="N56" s="6"/>
-      <c r="O56" s="6"/>
-      <c r="P56" s="6"/>
-      <c r="Q56" s="6"/>
-      <c r="R56" s="6"/>
-      <c r="S56" s="6"/>
-      <c r="T56" s="6"/>
-      <c r="U56" s="6"/>
-      <c r="V56" s="6"/>
-      <c r="W56" s="6"/>
-      <c r="X56" s="6"/>
-      <c r="Y56" s="6"/>
-      <c r="Z56" s="6"/>
-      <c r="AA56" s="6"/>
-      <c r="AB56" s="6"/>
-      <c r="AC56" s="6"/>
-    </row>
-    <row r="57" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="L57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="O57" s="4"/>
-      <c r="P57" s="4"/>
-      <c r="Q57" s="4"/>
-      <c r="R57" s="4"/>
-      <c r="S57" s="4"/>
-      <c r="T57" s="4"/>
-      <c r="U57" s="4"/>
-      <c r="V57" s="4"/>
-      <c r="W57" s="4"/>
-      <c r="X57" s="4"/>
-      <c r="Y57" s="4"/>
-      <c r="Z57" s="4"/>
-      <c r="AA57" s="4"/>
-      <c r="AB57" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="AC57" s="4"/>
-    </row>
-    <row r="58" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="O58" s="15"/>
-      <c r="P58" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q58" s="15"/>
-      <c r="R58" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="S58" s="15"/>
-      <c r="T58" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="U58" s="15"/>
-      <c r="V58" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="W58" s="15"/>
-      <c r="X58" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="Y58" s="15"/>
-      <c r="Z58" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="AA58" s="15"/>
-      <c r="AB58" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="AC58" s="15"/>
-    </row>
-    <row r="59" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="F59" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="G59" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="H59" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I59" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J59" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K59" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L59" s="5"/>
-      <c r="M59" s="5"/>
-      <c r="N59" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="O59" s="5"/>
-      <c r="P59" s="5"/>
-      <c r="Q59" s="5"/>
-      <c r="R59" s="5"/>
-      <c r="S59" s="5"/>
-      <c r="T59" s="5"/>
-      <c r="U59" s="5"/>
-      <c r="V59" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="W59" s="5"/>
-      <c r="X59" s="5" t="s">
+      <c r="B63" s="17"/>
+      <c r="C63" s="17"/>
+      <c r="D63" s="5" t="s">
         <v>165</v>
-      </c>
-      <c r="Y59" s="5"/>
-      <c r="Z59" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA59" s="5"/>
-      <c r="AB59" s="5"/>
-      <c r="AC59" s="5"/>
-    </row>
-    <row r="60" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
-      <c r="I60" s="2"/>
-      <c r="J60" s="2"/>
-      <c r="K60" s="2"/>
-      <c r="L60" s="2"/>
-      <c r="M60" s="2"/>
-      <c r="N60" s="2"/>
-      <c r="O60" s="2"/>
-      <c r="P60" s="2"/>
-      <c r="Q60" s="2"/>
-      <c r="R60" s="2"/>
-      <c r="S60" s="2"/>
-      <c r="T60" s="2"/>
-      <c r="U60" s="2"/>
-    </row>
-    <row r="61" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="B61" s="6"/>
-      <c r="C61" s="6"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="6"/>
-      <c r="F61" s="6"/>
-      <c r="G61" s="6"/>
-      <c r="H61" s="6"/>
-      <c r="I61" s="6"/>
-      <c r="J61" s="6"/>
-      <c r="K61" s="6"/>
-      <c r="L61" s="6"/>
-      <c r="M61" s="6"/>
-      <c r="N61" s="6"/>
-      <c r="O61" s="6"/>
-      <c r="P61" s="6"/>
-      <c r="Q61" s="6"/>
-      <c r="R61" s="6"/>
-      <c r="S61" s="6"/>
-      <c r="T61" s="6"/>
-      <c r="U61" s="6"/>
-    </row>
-    <row r="62" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E62" s="4"/>
-      <c r="F62" s="4"/>
-      <c r="H62" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="I62" s="4"/>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B63" s="16"/>
-      <c r="C63" s="9"/>
-      <c r="D63" s="5" t="s">
-        <v>172</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
-      <c r="H63" s="5" t="s">
-        <v>173</v>
-      </c>
+      <c r="H63" s="18"/>
       <c r="I63" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="J63" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K63" s="5" t="s">
-        <v>49</v>
-      </c>
+        <v>168</v>
+      </c>
+      <c r="J63" s="5"/>
+      <c r="K63" s="18"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B64" s="16"/>
-      <c r="C64" s="16"/>
+        <v>5</v>
+      </c>
+      <c r="B64" s="19"/>
+      <c r="C64" s="9"/>
       <c r="D64" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
-      <c r="H64" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="I64" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="J64" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="K64" s="5" t="s">
-        <v>176</v>
-      </c>
+      <c r="I64" s="5"/>
+      <c r="J64" s="5"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B65" s="17"/>
-      <c r="C65" s="9"/>
+        <v>6</v>
+      </c>
+      <c r="B65" s="19"/>
+      <c r="C65" s="19"/>
       <c r="D65" s="5" t="s">
-        <v>172</v>
+        <v>49</v>
       </c>
       <c r="E65" s="5"/>
       <c r="F65" s="5"/>
-      <c r="H65" s="18"/>
-      <c r="I65" s="18"/>
-      <c r="J65" s="18"/>
-      <c r="K65" s="18"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
+        <v>7</v>
+      </c>
+      <c r="B66" s="20"/>
+      <c r="C66" s="9"/>
       <c r="D66" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
-      <c r="H66" s="18"/>
-      <c r="I66" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="J66" s="5"/>
-      <c r="K66" s="18"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B67" s="19"/>
-      <c r="C67" s="9"/>
+        <v>8</v>
+      </c>
+      <c r="B67" s="20"/>
+      <c r="C67" s="20"/>
       <c r="D67" s="5" t="s">
-        <v>175</v>
+        <v>49</v>
       </c>
       <c r="E67" s="5"/>
       <c r="F67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
-    </row>
-    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="B68" s="19"/>
-      <c r="C68" s="19"/>
-      <c r="D68" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-    </row>
-    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B69" s="20"/>
-      <c r="C69" s="9"/>
-      <c r="D69" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="E69" s="5"/>
-      <c r="F69" s="5"/>
-    </row>
-    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B70" s="20"/>
-      <c r="C70" s="20"/>
-      <c r="D70" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E70" s="5"/>
-      <c r="F70" s="5"/>
+    </row>
+    <row r="68" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2"/>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
+      <c r="F68" s="2"/>
+      <c r="G68" s="2"/>
+      <c r="H68" s="2"/>
+      <c r="I68" s="2"/>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
+      <c r="L68" s="2"/>
+      <c r="M68" s="2"/>
+      <c r="N68" s="2"/>
+      <c r="O68" s="2"/>
+      <c r="P68" s="2"/>
+      <c r="Q68" s="2"/>
+      <c r="R68" s="2"/>
+      <c r="S68" s="2"/>
+      <c r="T68" s="2"/>
+      <c r="U68" s="2"/>
+    </row>
+    <row r="69" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B69" s="14"/>
+      <c r="C69" s="14"/>
+      <c r="D69" s="14"/>
+      <c r="E69" s="14"/>
+      <c r="F69" s="14"/>
+      <c r="G69" s="14"/>
+      <c r="H69" s="14"/>
+      <c r="I69" s="14"/>
+      <c r="J69" s="14"/>
+      <c r="K69" s="14"/>
+      <c r="L69" s="14"/>
+      <c r="M69" s="14"/>
+      <c r="N69" s="14"/>
+      <c r="O69" s="14"/>
+      <c r="P69" s="14"/>
+      <c r="Q69" s="14"/>
+      <c r="R69" s="14"/>
+      <c r="S69" s="14"/>
+      <c r="T69" s="14"/>
+      <c r="U69" s="14"/>
+    </row>
+    <row r="70" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B70" s="6"/>
+      <c r="C70" s="6"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+      <c r="H70" s="6"/>
+      <c r="I70" s="6"/>
+      <c r="J70" s="6"/>
+      <c r="K70" s="6"/>
+      <c r="L70" s="6"/>
+      <c r="M70" s="6"/>
+      <c r="N70" s="6"/>
+      <c r="O70" s="6"/>
+      <c r="P70" s="6"/>
+      <c r="Q70" s="6"/>
+      <c r="R70" s="6"/>
+      <c r="S70" s="6"/>
+      <c r="T70" s="6"/>
+      <c r="U70" s="6"/>
     </row>
     <row r="71" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-      <c r="F71" s="2"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
-      <c r="I71" s="2"/>
-      <c r="J71" s="2"/>
-      <c r="K71" s="2"/>
-      <c r="L71" s="2"/>
-      <c r="M71" s="2"/>
-      <c r="N71" s="2"/>
-      <c r="O71" s="2"/>
-      <c r="P71" s="2"/>
-      <c r="Q71" s="2"/>
-      <c r="R71" s="2"/>
-      <c r="S71" s="2"/>
-      <c r="T71" s="2"/>
-      <c r="U71" s="2"/>
-    </row>
-    <row r="72" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B72" s="14"/>
-      <c r="C72" s="14"/>
-      <c r="D72" s="14"/>
-      <c r="E72" s="14"/>
-      <c r="F72" s="14"/>
-      <c r="G72" s="14"/>
-      <c r="H72" s="14"/>
-      <c r="I72" s="14"/>
-      <c r="J72" s="14"/>
-      <c r="K72" s="14"/>
-      <c r="L72" s="14"/>
-      <c r="M72" s="14"/>
-      <c r="N72" s="14"/>
-      <c r="O72" s="14"/>
-      <c r="P72" s="14"/>
-      <c r="Q72" s="14"/>
-      <c r="R72" s="14"/>
-      <c r="S72" s="14"/>
-      <c r="T72" s="14"/>
-      <c r="U72" s="14"/>
-    </row>
-    <row r="73" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B73" s="6"/>
-      <c r="C73" s="6"/>
-      <c r="D73" s="6"/>
-      <c r="E73" s="6"/>
-      <c r="F73" s="6"/>
-      <c r="G73" s="6"/>
-      <c r="H73" s="6"/>
-      <c r="I73" s="6"/>
-      <c r="J73" s="6"/>
-      <c r="K73" s="6"/>
-      <c r="L73" s="6"/>
-      <c r="M73" s="6"/>
-      <c r="N73" s="6"/>
-      <c r="O73" s="6"/>
-      <c r="P73" s="6"/>
-      <c r="Q73" s="6"/>
-      <c r="R73" s="6"/>
-      <c r="S73" s="6"/>
-      <c r="T73" s="6"/>
-      <c r="U73" s="6"/>
-    </row>
-    <row r="74" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="4" t="s">
+      <c r="A71" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="B71" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C74" s="4"/>
-      <c r="D74" s="4"/>
-      <c r="E74" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
-      <c r="H74" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I74" s="4"/>
-      <c r="J74" s="4"/>
-      <c r="K74" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="L74" s="4"/>
-      <c r="M74" s="4"/>
-      <c r="N74" s="4" t="s">
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+      <c r="H71" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I71" s="4"/>
+      <c r="J71" s="4"/>
+      <c r="K71" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="L71" s="4"/>
+      <c r="M71" s="4"/>
+      <c r="N71" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O74" s="4"/>
-      <c r="P74" s="4"/>
-      <c r="Q74" s="4"/>
-      <c r="R74" s="4"/>
-      <c r="S74" s="4"/>
-      <c r="T74" s="4"/>
-      <c r="U74" s="4"/>
-    </row>
-    <row r="75" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="9" t="n">
+      <c r="O71" s="4"/>
+      <c r="P71" s="4"/>
+      <c r="Q71" s="4"/>
+      <c r="R71" s="4"/>
+      <c r="S71" s="4"/>
+      <c r="T71" s="4"/>
+      <c r="U71" s="4"/>
+    </row>
+    <row r="72" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B75" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-      <c r="E75" s="5" t="s">
+      <c r="B72" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F75" s="5"/>
-      <c r="G75" s="5"/>
-      <c r="H75" s="5" t="s">
+      <c r="F72" s="5"/>
+      <c r="G72" s="5"/>
+      <c r="H72" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J72" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="K72" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="L72" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M72" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="N72" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="O72" s="5"/>
+      <c r="P72" s="5"/>
+      <c r="Q72" s="5"/>
+      <c r="R72" s="5"/>
+      <c r="S72" s="5"/>
+      <c r="T72" s="5"/>
+      <c r="U72" s="5"/>
+    </row>
+    <row r="73" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="9"/>
+      <c r="B73" s="5"/>
+      <c r="C73" s="5"/>
+      <c r="D73" s="5"/>
+      <c r="E73" s="5"/>
+      <c r="F73" s="5"/>
+      <c r="G73" s="5"/>
+      <c r="H73" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="I73" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J73" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="K73" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="L73" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M73" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="N73" s="5"/>
+      <c r="O73" s="5"/>
+      <c r="P73" s="5"/>
+      <c r="Q73" s="5"/>
+      <c r="R73" s="5"/>
+      <c r="S73" s="5"/>
+      <c r="T73" s="5"/>
+      <c r="U73" s="5"/>
+    </row>
+    <row r="74" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="9"/>
+      <c r="B74" s="5"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="I74" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J74" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="K74" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="L74" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M74" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="N74" s="5"/>
+      <c r="O74" s="5"/>
+      <c r="P74" s="5"/>
+      <c r="Q74" s="5"/>
+      <c r="R74" s="5"/>
+      <c r="S74" s="5"/>
+      <c r="T74" s="5"/>
+      <c r="U74" s="5"/>
+    </row>
+    <row r="75" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="2"/>
+      <c r="E75" s="2"/>
+      <c r="F75" s="2"/>
+      <c r="G75" s="2"/>
+      <c r="H75" s="2"/>
+      <c r="I75" s="2"/>
+      <c r="J75" s="2"/>
+      <c r="K75" s="2"/>
+      <c r="L75" s="2"/>
+      <c r="M75" s="2"/>
+      <c r="N75" s="2"/>
+      <c r="O75" s="2"/>
+      <c r="P75" s="2"/>
+      <c r="Q75" s="2"/>
+      <c r="R75" s="2"/>
+      <c r="S75" s="2"/>
+      <c r="T75" s="2"/>
+      <c r="U75" s="2"/>
+    </row>
+    <row r="76" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B76" s="6"/>
+      <c r="C76" s="6"/>
+      <c r="D76" s="6"/>
+      <c r="E76" s="6"/>
+      <c r="F76" s="6"/>
+      <c r="G76" s="6"/>
+      <c r="H76" s="6"/>
+      <c r="I76" s="6"/>
+      <c r="J76" s="6"/>
+      <c r="K76" s="6"/>
+      <c r="L76" s="6"/>
+      <c r="M76" s="6"/>
+      <c r="N76" s="6"/>
+      <c r="O76" s="6"/>
+      <c r="P76" s="6"/>
+      <c r="Q76" s="6"/>
+      <c r="R76" s="6"/>
+      <c r="S76" s="6"/>
+      <c r="T76" s="6"/>
+      <c r="U76" s="6"/>
+      <c r="V76" s="6"/>
+      <c r="W76" s="6"/>
+      <c r="X76" s="6"/>
+      <c r="Y76" s="6"/>
+      <c r="Z76" s="6"/>
+      <c r="AA76" s="6"/>
+      <c r="AB76" s="6"/>
+      <c r="AC76" s="6"/>
+    </row>
+    <row r="77" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="I75" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J75" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K75" s="5" t="s">
+      <c r="F77" s="4"/>
+      <c r="G77" s="4"/>
+      <c r="H77" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="L75" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="M75" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N75" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="O75" s="5"/>
-      <c r="P75" s="5"/>
-      <c r="Q75" s="5"/>
-      <c r="R75" s="5"/>
-      <c r="S75" s="5"/>
-      <c r="T75" s="5"/>
-      <c r="U75" s="5"/>
-    </row>
-    <row r="76" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="9"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-      <c r="G76" s="5"/>
-      <c r="H76" s="5" t="s">
+      <c r="I77" s="4"/>
+      <c r="J77" s="4"/>
+      <c r="K77" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="L77" s="4"/>
+      <c r="M77" s="4"/>
+      <c r="N77" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="I76" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J76" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K76" s="5" t="s">
+      <c r="O77" s="4"/>
+      <c r="P77" s="4"/>
+      <c r="Q77" s="4"/>
+      <c r="R77" s="4"/>
+      <c r="S77" s="4"/>
+      <c r="T77" s="4"/>
+      <c r="U77" s="4"/>
+      <c r="V77" s="4"/>
+      <c r="W77" s="4"/>
+      <c r="X77" s="4"/>
+      <c r="Y77" s="4"/>
+      <c r="Z77" s="4"/>
+      <c r="AA77" s="4"/>
+      <c r="AB77" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="L76" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="M76" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N76" s="5"/>
-      <c r="O76" s="5"/>
-      <c r="P76" s="5"/>
-      <c r="Q76" s="5"/>
-      <c r="R76" s="5"/>
-      <c r="S76" s="5"/>
-      <c r="T76" s="5"/>
-      <c r="U76" s="5"/>
-    </row>
-    <row r="77" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="9"/>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="5"/>
-      <c r="F77" s="5"/>
-      <c r="G77" s="5"/>
-      <c r="H77" s="5" t="s">
+      <c r="AC77" s="4"/>
+    </row>
+    <row r="78" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="4"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+      <c r="F78" s="4"/>
+      <c r="G78" s="4"/>
+      <c r="H78" s="4"/>
+      <c r="I78" s="4"/>
+      <c r="J78" s="4"/>
+      <c r="K78" s="4"/>
+      <c r="L78" s="4"/>
+      <c r="M78" s="4"/>
+      <c r="N78" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="I77" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J77" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K77" s="5" t="s">
+      <c r="O78" s="15"/>
+      <c r="P78" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="L77" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="M77" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="N77" s="5"/>
-      <c r="O77" s="5"/>
-      <c r="P77" s="5"/>
-      <c r="Q77" s="5"/>
-      <c r="R77" s="5"/>
-      <c r="S77" s="5"/>
-      <c r="T77" s="5"/>
-      <c r="U77" s="5"/>
-    </row>
-    <row r="78" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="2"/>
-      <c r="I78" s="2"/>
-      <c r="J78" s="2"/>
-      <c r="K78" s="2"/>
-      <c r="L78" s="2"/>
-      <c r="M78" s="2"/>
-      <c r="N78" s="2"/>
-      <c r="O78" s="2"/>
-      <c r="P78" s="2"/>
-      <c r="Q78" s="2"/>
-      <c r="R78" s="2"/>
-      <c r="S78" s="2"/>
-      <c r="T78" s="2"/>
-      <c r="U78" s="2"/>
-    </row>
-    <row r="79" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="6" t="s">
+      <c r="Q78" s="15"/>
+      <c r="R78" s="15" t="s">
         <v>148</v>
       </c>
-      <c r="B79" s="6"/>
-      <c r="C79" s="6"/>
-      <c r="D79" s="6"/>
-      <c r="E79" s="6"/>
-      <c r="F79" s="6"/>
-      <c r="G79" s="6"/>
-      <c r="H79" s="6"/>
-      <c r="I79" s="6"/>
-      <c r="J79" s="6"/>
-      <c r="K79" s="6"/>
-      <c r="L79" s="6"/>
-      <c r="M79" s="6"/>
-      <c r="N79" s="6"/>
-      <c r="O79" s="6"/>
-      <c r="P79" s="6"/>
-      <c r="Q79" s="6"/>
-      <c r="R79" s="6"/>
-      <c r="S79" s="6"/>
-      <c r="T79" s="6"/>
-      <c r="U79" s="6"/>
-      <c r="V79" s="6"/>
-      <c r="W79" s="6"/>
-      <c r="X79" s="6"/>
-      <c r="Y79" s="6"/>
-      <c r="Z79" s="6"/>
-      <c r="AA79" s="6"/>
-      <c r="AB79" s="6"/>
-      <c r="AC79" s="6"/>
+      <c r="S78" s="15"/>
+      <c r="T78" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="U78" s="15"/>
+      <c r="V78" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="W78" s="15"/>
+      <c r="X78" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y78" s="15"/>
+      <c r="Z78" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA78" s="15"/>
+      <c r="AB78" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="AC78" s="15"/>
+    </row>
+    <row r="79" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="G79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H79" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="J79" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="K79" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L79" s="5"/>
+      <c r="M79" s="5"/>
+      <c r="N79" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="O79" s="5"/>
+      <c r="P79" s="5"/>
+      <c r="Q79" s="5"/>
+      <c r="R79" s="5"/>
+      <c r="S79" s="5"/>
+      <c r="T79" s="5"/>
+      <c r="U79" s="5"/>
+      <c r="V79" s="5"/>
+      <c r="W79" s="5"/>
+      <c r="X79" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="Y79" s="5"/>
+      <c r="Z79" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="AA79" s="5"/>
+      <c r="AB79" s="5"/>
+      <c r="AC79" s="5"/>
     </row>
     <row r="80" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C80" s="4"/>
-      <c r="D80" s="4"/>
-      <c r="E80" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
-      <c r="H80" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I80" s="4"/>
-      <c r="J80" s="4"/>
-      <c r="K80" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="L80" s="4"/>
-      <c r="M80" s="4"/>
-      <c r="N80" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="O80" s="4"/>
-      <c r="P80" s="4"/>
-      <c r="Q80" s="4"/>
-      <c r="R80" s="4"/>
-      <c r="S80" s="4"/>
-      <c r="T80" s="4"/>
-      <c r="U80" s="4"/>
-      <c r="V80" s="4"/>
-      <c r="W80" s="4"/>
-      <c r="X80" s="4"/>
-      <c r="Y80" s="4"/>
-      <c r="Z80" s="4"/>
-      <c r="AA80" s="4"/>
-      <c r="AB80" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="AC80" s="4"/>
-    </row>
-    <row r="81" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="4"/>
-      <c r="B81" s="4"/>
-      <c r="C81" s="4"/>
-      <c r="D81" s="4"/>
-      <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
-      <c r="G81" s="4"/>
-      <c r="H81" s="4"/>
-      <c r="I81" s="4"/>
-      <c r="J81" s="4"/>
-      <c r="K81" s="4"/>
-      <c r="L81" s="4"/>
-      <c r="M81" s="4"/>
-      <c r="N81" s="15" t="s">
-        <v>155</v>
-      </c>
-      <c r="O81" s="15"/>
-      <c r="P81" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q81" s="15"/>
-      <c r="R81" s="15" t="s">
-        <v>157</v>
-      </c>
-      <c r="S81" s="15"/>
-      <c r="T81" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="U81" s="15"/>
-      <c r="V81" s="15" t="s">
-        <v>159</v>
-      </c>
-      <c r="W81" s="15"/>
-      <c r="X81" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="Y81" s="15"/>
-      <c r="Z81" s="15" t="s">
-        <v>161</v>
-      </c>
-      <c r="AA81" s="15"/>
-      <c r="AB81" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="AC81" s="15"/>
-    </row>
-    <row r="82" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C82" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="D82" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="F82" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="G82" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="H82" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I82" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="J82" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="K82" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L82" s="5"/>
-      <c r="M82" s="5"/>
-      <c r="N82" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="O82" s="5"/>
-      <c r="P82" s="5"/>
-      <c r="Q82" s="5"/>
-      <c r="R82" s="5"/>
-      <c r="S82" s="5"/>
-      <c r="T82" s="5"/>
-      <c r="U82" s="5"/>
-      <c r="V82" s="5"/>
-      <c r="W82" s="5"/>
-      <c r="X82" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="Y82" s="5"/>
-      <c r="Z82" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="AA82" s="5"/>
-      <c r="AB82" s="5"/>
-      <c r="AC82" s="5"/>
-    </row>
-    <row r="83" customFormat="false" ht="21.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
-      <c r="F83" s="2"/>
-      <c r="G83" s="2"/>
-      <c r="H83" s="2"/>
-      <c r="I83" s="2"/>
-      <c r="J83" s="2"/>
-      <c r="K83" s="2"/>
-      <c r="L83" s="2"/>
-      <c r="M83" s="2"/>
-      <c r="N83" s="2"/>
-      <c r="O83" s="2"/>
-      <c r="P83" s="2"/>
-      <c r="Q83" s="2"/>
-      <c r="R83" s="2"/>
-      <c r="S83" s="2"/>
-      <c r="T83" s="2"/>
-      <c r="U83" s="2"/>
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="E80" s="2"/>
+      <c r="F80" s="2"/>
+      <c r="G80" s="2"/>
+      <c r="H80" s="2"/>
+      <c r="I80" s="2"/>
+      <c r="J80" s="2"/>
+      <c r="K80" s="2"/>
+      <c r="L80" s="2"/>
+      <c r="M80" s="2"/>
+      <c r="N80" s="2"/>
+      <c r="O80" s="2"/>
+      <c r="P80" s="2"/>
+      <c r="Q80" s="2"/>
+      <c r="R80" s="2"/>
+      <c r="S80" s="2"/>
+      <c r="T80" s="2"/>
+      <c r="U80" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="233">
+  <mergeCells count="224">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -4200,8 +4080,8 @@
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:N16"/>
-    <mergeCell ref="O16:Q23"/>
-    <mergeCell ref="R16:U23"/>
+    <mergeCell ref="O16:Q20"/>
+    <mergeCell ref="R16:U20"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:N17"/>
@@ -4214,179 +4094,170 @@
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="G20:N20"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="G21:N21"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="G22:N22"/>
+    <mergeCell ref="A21:U21"/>
+    <mergeCell ref="A22:U22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="G23:N23"/>
-    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="O23:Q23"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="G24:N24"/>
+    <mergeCell ref="O24:Q24"/>
     <mergeCell ref="A25:U25"/>
-    <mergeCell ref="B26:D26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G26:N26"/>
-    <mergeCell ref="O26:Q26"/>
+    <mergeCell ref="A26:U26"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="G27:N27"/>
     <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="A28:U28"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="G28:N28"/>
+    <mergeCell ref="O28:Q28"/>
     <mergeCell ref="A29:U29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="G30:N30"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="G31:N31"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="A32:U32"/>
-    <mergeCell ref="A33:U33"/>
-    <mergeCell ref="A34:U34"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="A30:U30"/>
+    <mergeCell ref="A31:U31"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="N32:U32"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="B33:D37"/>
+    <mergeCell ref="E33:G44"/>
+    <mergeCell ref="H33:J33"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="N33:U37"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="K34:M34"/>
     <mergeCell ref="H35:J35"/>
     <mergeCell ref="K35:M35"/>
-    <mergeCell ref="N35:U35"/>
-    <mergeCell ref="A36:A40"/>
-    <mergeCell ref="B36:D40"/>
-    <mergeCell ref="E36:G47"/>
     <mergeCell ref="H36:J36"/>
     <mergeCell ref="K36:M36"/>
-    <mergeCell ref="N36:U40"/>
     <mergeCell ref="H37:J37"/>
     <mergeCell ref="K37:M37"/>
+    <mergeCell ref="A38:A44"/>
+    <mergeCell ref="B38:D44"/>
     <mergeCell ref="H38:J38"/>
     <mergeCell ref="K38:M38"/>
+    <mergeCell ref="N38:U44"/>
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="H40:J40"/>
     <mergeCell ref="K40:M40"/>
-    <mergeCell ref="A41:A47"/>
-    <mergeCell ref="B41:D47"/>
     <mergeCell ref="H41:J41"/>
     <mergeCell ref="K41:M41"/>
-    <mergeCell ref="N41:U47"/>
     <mergeCell ref="H42:J42"/>
     <mergeCell ref="K42:M42"/>
     <mergeCell ref="H43:J43"/>
     <mergeCell ref="K43:M43"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="K44:M44"/>
+    <mergeCell ref="A45:A48"/>
+    <mergeCell ref="B45:D48"/>
+    <mergeCell ref="E45:G48"/>
     <mergeCell ref="H45:J45"/>
     <mergeCell ref="K45:M45"/>
+    <mergeCell ref="N45:U48"/>
     <mergeCell ref="H46:J46"/>
     <mergeCell ref="K46:M46"/>
     <mergeCell ref="H47:J47"/>
     <mergeCell ref="K47:M47"/>
-    <mergeCell ref="A48:A51"/>
-    <mergeCell ref="B48:D51"/>
-    <mergeCell ref="E48:G51"/>
     <mergeCell ref="H48:J48"/>
     <mergeCell ref="K48:M48"/>
-    <mergeCell ref="N48:U51"/>
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B49:D51"/>
+    <mergeCell ref="E49:G51"/>
     <mergeCell ref="H49:J49"/>
     <mergeCell ref="K49:M49"/>
+    <mergeCell ref="N49:U51"/>
     <mergeCell ref="H50:J50"/>
     <mergeCell ref="K50:M50"/>
     <mergeCell ref="H51:J51"/>
     <mergeCell ref="K51:M51"/>
-    <mergeCell ref="A52:A54"/>
-    <mergeCell ref="B52:D54"/>
-    <mergeCell ref="E52:G54"/>
-    <mergeCell ref="H52:J52"/>
-    <mergeCell ref="K52:M52"/>
-    <mergeCell ref="N52:U54"/>
-    <mergeCell ref="H53:J53"/>
-    <mergeCell ref="K53:M53"/>
-    <mergeCell ref="H54:J54"/>
-    <mergeCell ref="K54:M54"/>
-    <mergeCell ref="A55:U55"/>
-    <mergeCell ref="A56:AC56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="B57:D58"/>
-    <mergeCell ref="E57:G58"/>
-    <mergeCell ref="H57:J58"/>
-    <mergeCell ref="K57:M58"/>
-    <mergeCell ref="N57:O57"/>
-    <mergeCell ref="P57:AA57"/>
-    <mergeCell ref="AB57:AC57"/>
-    <mergeCell ref="N58:O58"/>
-    <mergeCell ref="P58:Q58"/>
-    <mergeCell ref="R58:S58"/>
-    <mergeCell ref="T58:U58"/>
-    <mergeCell ref="V58:W58"/>
-    <mergeCell ref="X58:Y58"/>
-    <mergeCell ref="Z58:AA58"/>
-    <mergeCell ref="AB58:AC58"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="E59:G59"/>
-    <mergeCell ref="H59:J59"/>
-    <mergeCell ref="K59:M59"/>
-    <mergeCell ref="N59:U59"/>
-    <mergeCell ref="V59:W59"/>
-    <mergeCell ref="X59:Y59"/>
-    <mergeCell ref="Z59:AC59"/>
-    <mergeCell ref="A60:U60"/>
-    <mergeCell ref="A61:U61"/>
+    <mergeCell ref="A52:U52"/>
+    <mergeCell ref="A53:AC53"/>
+    <mergeCell ref="A54:A55"/>
+    <mergeCell ref="B54:D55"/>
+    <mergeCell ref="E54:G55"/>
+    <mergeCell ref="H54:J55"/>
+    <mergeCell ref="K54:M55"/>
+    <mergeCell ref="N54:O54"/>
+    <mergeCell ref="P54:AA54"/>
+    <mergeCell ref="AB54:AC54"/>
+    <mergeCell ref="N55:O55"/>
+    <mergeCell ref="P55:Q55"/>
+    <mergeCell ref="R55:S55"/>
+    <mergeCell ref="T55:U55"/>
+    <mergeCell ref="V55:W55"/>
+    <mergeCell ref="X55:Y55"/>
+    <mergeCell ref="Z55:AA55"/>
+    <mergeCell ref="AB55:AC55"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="H56:J56"/>
+    <mergeCell ref="K56:M56"/>
+    <mergeCell ref="N56:U56"/>
+    <mergeCell ref="V56:W56"/>
+    <mergeCell ref="X56:Y56"/>
+    <mergeCell ref="Z56:AC56"/>
+    <mergeCell ref="A57:U57"/>
+    <mergeCell ref="A58:U58"/>
+    <mergeCell ref="D59:F59"/>
+    <mergeCell ref="H59:K59"/>
+    <mergeCell ref="D60:F60"/>
+    <mergeCell ref="D61:F61"/>
     <mergeCell ref="D62:F62"/>
-    <mergeCell ref="H62:K62"/>
     <mergeCell ref="D63:F63"/>
+    <mergeCell ref="I63:J64"/>
     <mergeCell ref="D64:F64"/>
     <mergeCell ref="D65:F65"/>
     <mergeCell ref="D66:F66"/>
-    <mergeCell ref="I66:J67"/>
     <mergeCell ref="D67:F67"/>
-    <mergeCell ref="D68:F68"/>
-    <mergeCell ref="D69:F69"/>
-    <mergeCell ref="D70:F70"/>
-    <mergeCell ref="A71:U71"/>
-    <mergeCell ref="A72:U72"/>
-    <mergeCell ref="A73:U73"/>
-    <mergeCell ref="B74:D74"/>
-    <mergeCell ref="E74:G74"/>
+    <mergeCell ref="A68:U68"/>
+    <mergeCell ref="A69:U69"/>
+    <mergeCell ref="A70:U70"/>
+    <mergeCell ref="B71:D71"/>
+    <mergeCell ref="E71:G71"/>
+    <mergeCell ref="H71:J71"/>
+    <mergeCell ref="K71:M71"/>
+    <mergeCell ref="N71:U71"/>
+    <mergeCell ref="A72:A74"/>
+    <mergeCell ref="B72:D74"/>
+    <mergeCell ref="E72:G74"/>
+    <mergeCell ref="H72:J72"/>
+    <mergeCell ref="K72:M72"/>
+    <mergeCell ref="N72:U74"/>
+    <mergeCell ref="H73:J73"/>
+    <mergeCell ref="K73:M73"/>
     <mergeCell ref="H74:J74"/>
     <mergeCell ref="K74:M74"/>
-    <mergeCell ref="N74:U74"/>
-    <mergeCell ref="A75:A77"/>
-    <mergeCell ref="B75:D77"/>
-    <mergeCell ref="E75:G77"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="K75:M75"/>
-    <mergeCell ref="N75:U77"/>
-    <mergeCell ref="H76:J76"/>
-    <mergeCell ref="K76:M76"/>
-    <mergeCell ref="H77:J77"/>
-    <mergeCell ref="K77:M77"/>
-    <mergeCell ref="A78:U78"/>
-    <mergeCell ref="A79:AC79"/>
-    <mergeCell ref="A80:A81"/>
-    <mergeCell ref="B80:D81"/>
-    <mergeCell ref="E80:G81"/>
-    <mergeCell ref="H80:J81"/>
-    <mergeCell ref="K80:M81"/>
-    <mergeCell ref="N80:O80"/>
-    <mergeCell ref="P80:AA80"/>
-    <mergeCell ref="AB80:AC80"/>
-    <mergeCell ref="N81:O81"/>
-    <mergeCell ref="P81:Q81"/>
-    <mergeCell ref="R81:S81"/>
-    <mergeCell ref="T81:U81"/>
-    <mergeCell ref="V81:W81"/>
-    <mergeCell ref="X81:Y81"/>
-    <mergeCell ref="Z81:AA81"/>
-    <mergeCell ref="AB81:AC81"/>
-    <mergeCell ref="B82:D82"/>
-    <mergeCell ref="E82:G82"/>
-    <mergeCell ref="H82:J82"/>
-    <mergeCell ref="K82:M82"/>
-    <mergeCell ref="N82:W82"/>
-    <mergeCell ref="X82:Y82"/>
-    <mergeCell ref="Z82:AC82"/>
-    <mergeCell ref="A83:U83"/>
+    <mergeCell ref="A75:U75"/>
+    <mergeCell ref="A76:AC76"/>
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="B77:D78"/>
+    <mergeCell ref="E77:G78"/>
+    <mergeCell ref="H77:J78"/>
+    <mergeCell ref="K77:M78"/>
+    <mergeCell ref="N77:O77"/>
+    <mergeCell ref="P77:AA77"/>
+    <mergeCell ref="AB77:AC77"/>
+    <mergeCell ref="N78:O78"/>
+    <mergeCell ref="P78:Q78"/>
+    <mergeCell ref="R78:S78"/>
+    <mergeCell ref="T78:U78"/>
+    <mergeCell ref="V78:W78"/>
+    <mergeCell ref="X78:Y78"/>
+    <mergeCell ref="Z78:AA78"/>
+    <mergeCell ref="AB78:AC78"/>
+    <mergeCell ref="B79:D79"/>
+    <mergeCell ref="E79:G79"/>
+    <mergeCell ref="H79:J79"/>
+    <mergeCell ref="K79:M79"/>
+    <mergeCell ref="N79:W79"/>
+    <mergeCell ref="X79:Y79"/>
+    <mergeCell ref="Z79:AC79"/>
+    <mergeCell ref="A80:U80"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.29.18 ] - roulette driver circuit was tested. Future TODOs were added.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="DRIVERs" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="MOTION DIAGRAM" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="193">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -537,6 +538,69 @@
   </si>
   <si>
     <t xml:space="preserve">ROULETTE R1 ENABLE </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROULETTE DRIVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD4069UBE (NOT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR DRIVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!SLP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VDD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MHB4012 (NAND)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IN2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD4001BE (NOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOT 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOT 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOP 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOP 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10V</t>
   </si>
 </sst>
 </file>
@@ -546,7 +610,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -604,8 +668,23 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <u val="single"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -621,7 +700,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5D6A7"/>
-        <bgColor rgb="FF99CCFF"/>
+        <bgColor rgb="FFBDBDBD"/>
       </patternFill>
     </fill>
     <fill>
@@ -639,7 +718,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5F5F5"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
     <fill>
@@ -657,7 +736,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF9800"/>
-        <bgColor rgb="FFFF6600"/>
+        <bgColor rgb="FFFFCC00"/>
       </patternFill>
     </fill>
     <fill>
@@ -678,8 +757,32 @@
         <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFF5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF44336"/>
+        <bgColor rgb="FFFF8080"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDBDBD"/>
+        <bgColor rgb="FFE1BEE7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="15">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -689,6 +792,97 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
@@ -720,7 +914,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="73">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -802,6 +996,214 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -830,11 +1232,11 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFA5D6A7"/>
+      <rgbColor rgb="FFBDBDBD"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -852,7 +1254,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFA5D6A7"/>
       <rgbColor rgb="FFF8BBD0"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC80"/>
@@ -861,7 +1263,7 @@
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9800"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFF44336"/>
       <rgbColor rgb="FF795548"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
@@ -4267,4 +4669,364 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:W18"/>
+  <sheetFormatPr defaultColWidth="6.48828125" defaultRowHeight="36" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="21" width="6.49"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0"/>
+      <c r="B1" s="0"/>
+      <c r="C1" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+      <c r="I1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="L1" s="0"/>
+      <c r="M1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
+      <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+    </row>
+    <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
+      <c r="U2" s="24"/>
+      <c r="V2" s="25"/>
+      <c r="W2" s="26"/>
+    </row>
+    <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0"/>
+      <c r="C3" s="27"/>
+      <c r="L3" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="V3" s="0"/>
+      <c r="W3" s="29"/>
+    </row>
+    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0"/>
+      <c r="C4" s="27"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" s="31"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="32"/>
+      <c r="V4" s="0"/>
+      <c r="W4" s="29"/>
+    </row>
+    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0"/>
+      <c r="C5" s="27"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0"/>
+      <c r="L5" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="34"/>
+      <c r="P5" s="34"/>
+      <c r="Q5" s="35"/>
+      <c r="S5" s="0"/>
+      <c r="U5" s="36"/>
+      <c r="V5" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="W5" s="29"/>
+    </row>
+    <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0"/>
+      <c r="C6" s="27"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="K6" s="0"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="39"/>
+      <c r="O6" s="39"/>
+      <c r="P6" s="39"/>
+      <c r="Q6" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="S6" s="0"/>
+      <c r="U6" s="41"/>
+      <c r="V6" s="37"/>
+      <c r="W6" s="29"/>
+    </row>
+    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0"/>
+      <c r="C7" s="27"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="L7" s="28" t="s">
+        <v>175</v>
+      </c>
+      <c r="M7" s="28"/>
+      <c r="N7" s="28"/>
+      <c r="V7" s="0"/>
+      <c r="W7" s="29"/>
+    </row>
+    <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0"/>
+      <c r="C8" s="27"/>
+      <c r="G8" s="28" t="s">
+        <v>176</v>
+      </c>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="L8" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="M8" s="43"/>
+      <c r="N8" s="44"/>
+      <c r="V8" s="0"/>
+      <c r="W8" s="29"/>
+    </row>
+    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0"/>
+      <c r="C9" s="27"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="L9" s="48"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="V9" s="0"/>
+      <c r="W9" s="29"/>
+    </row>
+    <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0"/>
+      <c r="C10" s="27"/>
+      <c r="G10" s="51"/>
+      <c r="H10" s="52"/>
+      <c r="I10" s="53"/>
+      <c r="L10" s="28" t="s">
+        <v>179</v>
+      </c>
+      <c r="M10" s="28"/>
+      <c r="N10" s="28"/>
+      <c r="V10" s="0"/>
+      <c r="W10" s="29"/>
+    </row>
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="54" t="s">
+        <v>180</v>
+      </c>
+      <c r="E11" s="55"/>
+      <c r="G11" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="52"/>
+      <c r="I11" s="53" t="s">
+        <v>182</v>
+      </c>
+      <c r="L11" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="M11" s="43"/>
+      <c r="N11" s="44"/>
+      <c r="Q11" s="56"/>
+      <c r="V11" s="0"/>
+      <c r="W11" s="29"/>
+    </row>
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="54"/>
+      <c r="E12" s="57"/>
+      <c r="G12" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="H12" s="52"/>
+      <c r="I12" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="L12" s="48"/>
+      <c r="M12" s="49"/>
+      <c r="N12" s="50" t="s">
+        <v>178</v>
+      </c>
+      <c r="V12" s="0"/>
+      <c r="W12" s="29"/>
+    </row>
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0"/>
+      <c r="C13" s="27"/>
+      <c r="G13" s="51" t="s">
+        <v>49</v>
+      </c>
+      <c r="H13" s="52"/>
+      <c r="I13" s="53" t="s">
+        <v>49</v>
+      </c>
+      <c r="L13" s="28" t="s">
+        <v>185</v>
+      </c>
+      <c r="M13" s="28"/>
+      <c r="N13" s="28"/>
+      <c r="S13" s="58"/>
+      <c r="T13" s="59"/>
+      <c r="U13" s="60"/>
+      <c r="V13" s="61" t="s">
+        <v>186</v>
+      </c>
+      <c r="W13" s="29"/>
+    </row>
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0"/>
+      <c r="C14" s="27"/>
+      <c r="G14" s="62" t="s">
+        <v>187</v>
+      </c>
+      <c r="H14" s="63"/>
+      <c r="I14" s="64"/>
+      <c r="L14" s="42"/>
+      <c r="M14" s="44" t="s">
+        <v>178</v>
+      </c>
+      <c r="S14" s="58"/>
+      <c r="T14" s="59"/>
+      <c r="U14" s="60"/>
+      <c r="V14" s="61" t="s">
+        <v>188</v>
+      </c>
+      <c r="W14" s="29"/>
+    </row>
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0"/>
+      <c r="C15" s="27"/>
+      <c r="L15" s="65"/>
+      <c r="M15" s="66"/>
+      <c r="S15" s="58"/>
+      <c r="T15" s="59"/>
+      <c r="U15" s="60"/>
+      <c r="V15" s="61" t="s">
+        <v>189</v>
+      </c>
+      <c r="W15" s="29"/>
+    </row>
+    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0"/>
+      <c r="C16" s="27"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="60"/>
+      <c r="L16" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="M16" s="50"/>
+      <c r="P16" s="67"/>
+      <c r="Q16" s="60"/>
+      <c r="S16" s="58"/>
+      <c r="T16" s="59"/>
+      <c r="U16" s="60"/>
+      <c r="V16" s="61" t="s">
+        <v>190</v>
+      </c>
+      <c r="W16" s="29"/>
+    </row>
+    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C17" s="68"/>
+      <c r="E17" s="69" t="s">
+        <v>191</v>
+      </c>
+      <c r="F17" s="69"/>
+      <c r="P17" s="69" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q17" s="69"/>
+      <c r="V17" s="0"/>
+      <c r="W17" s="29"/>
+    </row>
+    <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C18" s="70"/>
+      <c r="D18" s="71"/>
+      <c r="E18" s="71"/>
+      <c r="F18" s="71"/>
+      <c r="G18" s="71"/>
+      <c r="H18" s="71"/>
+      <c r="I18" s="71"/>
+      <c r="J18" s="71"/>
+      <c r="K18" s="71"/>
+      <c r="L18" s="71"/>
+      <c r="M18" s="71"/>
+      <c r="N18" s="71"/>
+      <c r="O18" s="71"/>
+      <c r="P18" s="71"/>
+      <c r="Q18" s="71"/>
+      <c r="R18" s="71"/>
+      <c r="S18" s="71"/>
+      <c r="T18" s="71"/>
+      <c r="U18" s="71"/>
+      <c r="V18" s="71"/>
+      <c r="W18" s="72"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="V5:V6"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="P17:Q17"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[ Version 0.0.30.1 ] - vent driver UTP dupont cables were created.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="192">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -498,7 +498,7 @@
     <t xml:space="preserve">PROCESS CODE</t>
   </si>
   <si>
-    <t xml:space="preserve">RJ45 CONNECTION</t>
+    <t xml:space="preserve">DUPONT &amp; UTP CABLE CONNECTION</t>
   </si>
   <si>
     <t xml:space="preserve">CABLE</t>
@@ -510,25 +510,22 @@
     <t xml:space="preserve">COLOR 2</t>
   </si>
   <si>
-    <t xml:space="preserve">RJ45 socket schematics – BOTTOM VIEW</t>
+    <t xml:space="preserve">DUPONT terminal – TOP view</t>
   </si>
   <si>
     <t xml:space="preserve">+10V</t>
   </si>
   <si>
+    <t xml:space="preserve">+6V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PWM</t>
+  </si>
+  <si>
     <t xml:space="preserve">ESO</t>
   </si>
   <si>
     <t xml:space="preserve">ESC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+6V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PWM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CABLE INPUT</t>
   </si>
   <si>
     <t xml:space="preserve">roulette_dataset_t</t>
@@ -684,7 +681,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -694,7 +691,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC80"/>
-        <bgColor rgb="FFF8BBD0"/>
+        <bgColor rgb="FFFFCDD2"/>
       </patternFill>
     </fill>
     <fill>
@@ -730,13 +727,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF8BBD0"/>
-        <bgColor rgb="FFE1BEE7"/>
+        <bgColor rgb="FFFFCDD2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF9800"/>
         <bgColor rgb="FFFFCC00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCDD2"/>
+        <bgColor rgb="FFF8BBD0"/>
       </patternFill>
     </fill>
     <fill>
@@ -914,7 +917,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="75">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -983,7 +986,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -991,7 +998,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -999,211 +1006,215 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1253,7 +1264,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFCDD2"/>
       <rgbColor rgb="FFA5D6A7"/>
       <rgbColor rgb="FFF8BBD0"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -3863,16 +3874,16 @@
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
       <c r="H60" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="I60" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="J60" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I60" s="5" t="s">
+      <c r="K60" s="5" t="s">
         <v>165</v>
-      </c>
-      <c r="J60" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="K60" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3882,77 +3893,75 @@
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
       <c r="D61" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
       <c r="H61" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J61" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="K61" s="5" t="s">
-        <v>167</v>
+        <v>49</v>
+      </c>
+      <c r="K61" s="17" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B62" s="17"/>
+      <c r="B62" s="18"/>
       <c r="C62" s="9"/>
       <c r="D62" s="5" t="s">
         <v>163</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
-      <c r="H62" s="18"/>
-      <c r="I62" s="18"/>
-      <c r="J62" s="18"/>
-      <c r="K62" s="18"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="19"/>
+      <c r="J62" s="19"/>
+      <c r="K62" s="19"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="17"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
       <c r="D63" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
-      <c r="H63" s="18"/>
-      <c r="I63" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="J63" s="5"/>
-      <c r="K63" s="18"/>
+      <c r="H63" s="19"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
+      <c r="K63" s="19"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B64" s="19"/>
+      <c r="B64" s="21"/>
       <c r="C64" s="9"/>
       <c r="D64" s="5" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
-      <c r="I64" s="5"/>
-      <c r="J64" s="5"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B65" s="19"/>
-      <c r="C65" s="19"/>
+      <c r="B65" s="21"/>
+      <c r="C65" s="21"/>
       <c r="D65" s="5" t="s">
         <v>49</v>
       </c>
@@ -3963,10 +3972,10 @@
       <c r="A66" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B66" s="20"/>
+      <c r="B66" s="22"/>
       <c r="C66" s="9"/>
       <c r="D66" s="5" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E66" s="5"/>
       <c r="F66" s="5"/>
@@ -3975,8 +3984,8 @@
       <c r="A67" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B67" s="20"/>
-      <c r="C67" s="20"/>
+      <c r="B67" s="22"/>
+      <c r="C67" s="22"/>
       <c r="D67" s="5" t="s">
         <v>49</v>
       </c>
@@ -4096,7 +4105,7 @@
         <v>1</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
@@ -4124,7 +4133,7 @@
         <v>103</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="O72" s="5"/>
       <c r="P72" s="5"/>
@@ -4357,7 +4366,7 @@
         <v>1</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>103</v>
@@ -4401,7 +4410,7 @@
       <c r="V79" s="5"/>
       <c r="W79" s="5"/>
       <c r="X79" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="Y79" s="5"/>
       <c r="Z79" s="5" t="s">
@@ -4435,7 +4444,7 @@
       <c r="U80" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="224">
+  <mergeCells count="223">
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="A3:U3"/>
@@ -4611,7 +4620,6 @@
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="D62:F62"/>
     <mergeCell ref="D63:F63"/>
-    <mergeCell ref="I63:J64"/>
     <mergeCell ref="D64:F64"/>
     <mergeCell ref="D65:F65"/>
     <mergeCell ref="D66:F66"/>
@@ -4679,335 +4687,334 @@
   <dimension ref="A1:W18"/>
   <sheetFormatPr defaultColWidth="6.48828125" defaultRowHeight="36" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="21" width="6.49"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="19" width="6.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0"/>
-      <c r="B1" s="0"/>
-      <c r="C1" s="22" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="24" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
+      <c r="S1" s="23"/>
+    </row>
+    <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
+      <c r="V2" s="27"/>
+      <c r="W2" s="28"/>
+    </row>
+    <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="23"/>
+      <c r="C3" s="29"/>
+      <c r="L3" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="0"/>
-      <c r="G1" s="0"/>
-      <c r="H1" s="0"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
-      <c r="K1" s="0"/>
-      <c r="L1" s="0"/>
-      <c r="M1" s="0"/>
-      <c r="N1" s="0"/>
-      <c r="O1" s="0"/>
-      <c r="P1" s="0"/>
-      <c r="Q1" s="0"/>
-      <c r="R1" s="0"/>
-      <c r="S1" s="0"/>
-    </row>
-    <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="24"/>
-      <c r="R2" s="24"/>
-      <c r="S2" s="24"/>
-      <c r="T2" s="24"/>
-      <c r="U2" s="24"/>
-      <c r="V2" s="25"/>
-      <c r="W2" s="26"/>
-    </row>
-    <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0"/>
-      <c r="C3" s="27"/>
-      <c r="L3" s="28" t="s">
+      <c r="V3" s="23"/>
+      <c r="W3" s="31"/>
+    </row>
+    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23"/>
+      <c r="C4" s="29"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="M4" s="33"/>
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="33"/>
+      <c r="Q4" s="34"/>
+      <c r="V4" s="23"/>
+      <c r="W4" s="31"/>
+    </row>
+    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23"/>
+      <c r="C5" s="29"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="35" t="s">
         <v>173</v>
       </c>
-      <c r="V3" s="0"/>
-      <c r="W3" s="29"/>
-    </row>
-    <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0"/>
-      <c r="C4" s="27"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
-      <c r="K4" s="0"/>
-      <c r="L4" s="30" t="s">
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="37"/>
+      <c r="S5" s="23"/>
+      <c r="U5" s="38"/>
+      <c r="V5" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="31"/>
-      <c r="N4" s="31"/>
-      <c r="O4" s="31"/>
-      <c r="P4" s="31"/>
-      <c r="Q4" s="32"/>
-      <c r="V4" s="0"/>
-      <c r="W4" s="29"/>
-    </row>
-    <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0"/>
-      <c r="C5" s="27"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="K5" s="0"/>
-      <c r="L5" s="33" t="s">
+      <c r="W5" s="31"/>
+    </row>
+    <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23"/>
+      <c r="C6" s="29"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="40"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="S6" s="23"/>
+      <c r="U6" s="43"/>
+      <c r="V6" s="39"/>
+      <c r="W6" s="31"/>
+    </row>
+    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23"/>
+      <c r="C7" s="29"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="L7" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="34"/>
-      <c r="Q5" s="35"/>
-      <c r="S5" s="0"/>
-      <c r="U5" s="36"/>
-      <c r="V5" s="37" t="s">
-        <v>44</v>
-      </c>
-      <c r="W5" s="29"/>
-    </row>
-    <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0"/>
-      <c r="C6" s="27"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="38"/>
-      <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
-      <c r="O6" s="39"/>
-      <c r="P6" s="39"/>
-      <c r="Q6" s="40" t="s">
+      <c r="M7" s="44"/>
+      <c r="N7" s="44"/>
+      <c r="V7" s="23"/>
+      <c r="W7" s="31"/>
+    </row>
+    <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23"/>
+      <c r="C8" s="29"/>
+      <c r="G8" s="44" t="s">
+        <v>175</v>
+      </c>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="L8" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="S6" s="0"/>
-      <c r="U6" s="41"/>
-      <c r="V6" s="37"/>
-      <c r="W6" s="29"/>
-    </row>
-    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0"/>
-      <c r="C7" s="27"/>
-      <c r="G7" s="0"/>
-      <c r="H7" s="0"/>
-      <c r="I7" s="0"/>
-      <c r="L7" s="28" t="s">
-        <v>175</v>
-      </c>
-      <c r="M7" s="28"/>
-      <c r="N7" s="28"/>
-      <c r="V7" s="0"/>
-      <c r="W7" s="29"/>
-    </row>
-    <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0"/>
-      <c r="C8" s="27"/>
-      <c r="G8" s="28" t="s">
+      <c r="M8" s="46"/>
+      <c r="N8" s="47"/>
+      <c r="V8" s="23"/>
+      <c r="W8" s="31"/>
+    </row>
+    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23"/>
+      <c r="C9" s="29"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="50" t="s">
         <v>176</v>
       </c>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="L8" s="42" t="s">
+      <c r="L9" s="51"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="53" t="s">
+        <v>177</v>
+      </c>
+      <c r="V9" s="23"/>
+      <c r="W9" s="31"/>
+    </row>
+    <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23"/>
+      <c r="C10" s="29"/>
+      <c r="G10" s="54"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="56"/>
+      <c r="L10" s="44" t="s">
+        <v>178</v>
+      </c>
+      <c r="M10" s="44"/>
+      <c r="N10" s="44"/>
+      <c r="V10" s="23"/>
+      <c r="W10" s="31"/>
+    </row>
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="57" t="s">
+        <v>179</v>
+      </c>
+      <c r="E11" s="58"/>
+      <c r="G11" s="54" t="s">
+        <v>180</v>
+      </c>
+      <c r="H11" s="55"/>
+      <c r="I11" s="56" t="s">
+        <v>181</v>
+      </c>
+      <c r="L11" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="M8" s="43"/>
-      <c r="N8" s="44"/>
-      <c r="V8" s="0"/>
-      <c r="W8" s="29"/>
-    </row>
-    <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0"/>
-      <c r="C9" s="27"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="46"/>
-      <c r="I9" s="47" t="s">
+      <c r="M11" s="46"/>
+      <c r="N11" s="47"/>
+      <c r="V11" s="23"/>
+      <c r="W11" s="31"/>
+    </row>
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="57"/>
+      <c r="E12" s="59"/>
+      <c r="G12" s="54" t="s">
+        <v>182</v>
+      </c>
+      <c r="H12" s="55"/>
+      <c r="I12" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="L12" s="51"/>
+      <c r="M12" s="52"/>
+      <c r="N12" s="53" t="s">
         <v>177</v>
       </c>
-      <c r="L9" s="48"/>
-      <c r="M9" s="49"/>
-      <c r="N9" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="V9" s="0"/>
-      <c r="W9" s="29"/>
-    </row>
-    <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0"/>
-      <c r="C10" s="27"/>
-      <c r="G10" s="51"/>
-      <c r="H10" s="52"/>
-      <c r="I10" s="53"/>
-      <c r="L10" s="28" t="s">
-        <v>179</v>
-      </c>
-      <c r="M10" s="28"/>
-      <c r="N10" s="28"/>
-      <c r="V10" s="0"/>
-      <c r="W10" s="29"/>
-    </row>
-    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="54" t="s">
-        <v>180</v>
-      </c>
-      <c r="E11" s="55"/>
-      <c r="G11" s="51" t="s">
-        <v>181</v>
-      </c>
-      <c r="H11" s="52"/>
-      <c r="I11" s="53" t="s">
-        <v>182</v>
-      </c>
-      <c r="L11" s="42" t="s">
+      <c r="V12" s="23"/>
+      <c r="W12" s="31"/>
+    </row>
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23"/>
+      <c r="C13" s="29"/>
+      <c r="G13" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="M11" s="43"/>
-      <c r="N11" s="44"/>
-      <c r="Q11" s="56"/>
-      <c r="V11" s="0"/>
-      <c r="W11" s="29"/>
-    </row>
-    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="54"/>
-      <c r="E12" s="57"/>
-      <c r="G12" s="51" t="s">
-        <v>183</v>
-      </c>
-      <c r="H12" s="52"/>
-      <c r="I12" s="53" t="s">
+      <c r="H13" s="55"/>
+      <c r="I13" s="56" t="s">
+        <v>49</v>
+      </c>
+      <c r="L13" s="44" t="s">
         <v>184</v>
       </c>
-      <c r="L12" s="48"/>
-      <c r="M12" s="49"/>
-      <c r="N12" s="50" t="s">
-        <v>178</v>
-      </c>
-      <c r="V12" s="0"/>
-      <c r="W12" s="29"/>
-    </row>
-    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0"/>
-      <c r="C13" s="27"/>
-      <c r="G13" s="51" t="s">
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="S13" s="60"/>
+      <c r="T13" s="61"/>
+      <c r="U13" s="62"/>
+      <c r="V13" s="63" t="s">
+        <v>185</v>
+      </c>
+      <c r="W13" s="31"/>
+    </row>
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23"/>
+      <c r="C14" s="29"/>
+      <c r="G14" s="64" t="s">
+        <v>186</v>
+      </c>
+      <c r="H14" s="65"/>
+      <c r="I14" s="66"/>
+      <c r="L14" s="45"/>
+      <c r="M14" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="S14" s="60"/>
+      <c r="T14" s="61"/>
+      <c r="U14" s="62"/>
+      <c r="V14" s="63" t="s">
+        <v>187</v>
+      </c>
+      <c r="W14" s="31"/>
+    </row>
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23"/>
+      <c r="C15" s="29"/>
+      <c r="L15" s="67"/>
+      <c r="M15" s="68"/>
+      <c r="S15" s="60"/>
+      <c r="T15" s="61"/>
+      <c r="U15" s="62"/>
+      <c r="V15" s="63" t="s">
+        <v>188</v>
+      </c>
+      <c r="W15" s="31"/>
+    </row>
+    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23"/>
+      <c r="C16" s="29"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="62"/>
+      <c r="L16" s="51" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="52"/>
-      <c r="I13" s="53" t="s">
-        <v>49</v>
-      </c>
-      <c r="L13" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="M13" s="28"/>
-      <c r="N13" s="28"/>
-      <c r="S13" s="58"/>
-      <c r="T13" s="59"/>
-      <c r="U13" s="60"/>
-      <c r="V13" s="61" t="s">
-        <v>186</v>
-      </c>
-      <c r="W13" s="29"/>
-    </row>
-    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0"/>
-      <c r="C14" s="27"/>
-      <c r="G14" s="62" t="s">
-        <v>187</v>
-      </c>
-      <c r="H14" s="63"/>
-      <c r="I14" s="64"/>
-      <c r="L14" s="42"/>
-      <c r="M14" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S14" s="58"/>
-      <c r="T14" s="59"/>
-      <c r="U14" s="60"/>
-      <c r="V14" s="61" t="s">
-        <v>188</v>
-      </c>
-      <c r="W14" s="29"/>
-    </row>
-    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0"/>
-      <c r="C15" s="27"/>
-      <c r="L15" s="65"/>
-      <c r="M15" s="66"/>
-      <c r="S15" s="58"/>
-      <c r="T15" s="59"/>
-      <c r="U15" s="60"/>
-      <c r="V15" s="61" t="s">
+      <c r="M16" s="53"/>
+      <c r="P16" s="69"/>
+      <c r="Q16" s="62"/>
+      <c r="S16" s="60"/>
+      <c r="T16" s="61"/>
+      <c r="U16" s="62"/>
+      <c r="V16" s="63" t="s">
         <v>189</v>
       </c>
-      <c r="W15" s="29"/>
-    </row>
-    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0"/>
-      <c r="C16" s="27"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="60"/>
-      <c r="L16" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="M16" s="50"/>
-      <c r="P16" s="67"/>
-      <c r="Q16" s="60"/>
-      <c r="S16" s="58"/>
-      <c r="T16" s="59"/>
-      <c r="U16" s="60"/>
-      <c r="V16" s="61" t="s">
+      <c r="W16" s="31"/>
+    </row>
+    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C17" s="70"/>
+      <c r="E17" s="71" t="s">
         <v>190</v>
       </c>
-      <c r="W16" s="29"/>
-    </row>
-    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="68"/>
-      <c r="E17" s="69" t="s">
+      <c r="F17" s="71"/>
+      <c r="P17" s="71" t="s">
         <v>191</v>
       </c>
-      <c r="F17" s="69"/>
-      <c r="P17" s="69" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q17" s="69"/>
-      <c r="V17" s="0"/>
-      <c r="W17" s="29"/>
+      <c r="Q17" s="71"/>
+      <c r="V17" s="23"/>
+      <c r="W17" s="31"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="70"/>
-      <c r="D18" s="71"/>
-      <c r="E18" s="71"/>
-      <c r="F18" s="71"/>
-      <c r="G18" s="71"/>
-      <c r="H18" s="71"/>
-      <c r="I18" s="71"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="71"/>
-      <c r="L18" s="71"/>
-      <c r="M18" s="71"/>
-      <c r="N18" s="71"/>
-      <c r="O18" s="71"/>
-      <c r="P18" s="71"/>
-      <c r="Q18" s="71"/>
-      <c r="R18" s="71"/>
-      <c r="S18" s="71"/>
-      <c r="T18" s="71"/>
-      <c r="U18" s="71"/>
-      <c r="V18" s="71"/>
-      <c r="W18" s="72"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="73"/>
+      <c r="E18" s="73"/>
+      <c r="F18" s="73"/>
+      <c r="G18" s="73"/>
+      <c r="H18" s="73"/>
+      <c r="I18" s="73"/>
+      <c r="J18" s="73"/>
+      <c r="K18" s="73"/>
+      <c r="L18" s="73"/>
+      <c r="M18" s="73"/>
+      <c r="N18" s="73"/>
+      <c r="O18" s="73"/>
+      <c r="P18" s="73"/>
+      <c r="Q18" s="73"/>
+      <c r="R18" s="73"/>
+      <c r="S18" s="73"/>
+      <c r="T18" s="73"/>
+      <c r="U18" s="73"/>
+      <c r="V18" s="73"/>
+      <c r="W18" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
[ Version 0.0.30.3 ] - new servo driver was build on breadboard.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="193">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -526,6 +526,9 @@
   </si>
   <si>
     <t xml:space="preserve">ESC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARROW</t>
   </si>
   <si>
     <t xml:space="preserve">roulette_dataset_t</t>
@@ -607,7 +610,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -661,6 +664,21 @@
       <b val="true"/>
       <i val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -738,12 +756,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCDD2"/>
-        <bgColor rgb="FFF8BBD0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF4CAF50"/>
         <bgColor rgb="FF808080"/>
       </patternFill>
@@ -758,6 +770,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF795548"/>
         <bgColor rgb="FF993366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCDD2"/>
+        <bgColor rgb="FFF8BBD0"/>
       </patternFill>
     </fill>
     <fill>
@@ -795,6 +813,20 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
@@ -871,22 +903,8 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
       <diagonal/>
@@ -917,7 +935,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="84">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -986,7 +1004,55 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="12" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -994,19 +1060,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1018,27 +1072,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1046,19 +1088,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1066,7 +1120,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1074,19 +1128,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1094,43 +1148,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1138,11 +1172,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1150,15 +1204,7 @@
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1166,7 +1212,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1174,35 +1228,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="17" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="17" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1210,11 +1256,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1230,7 +1284,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFF5F5F5"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -1247,8 +1301,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFF5F5F5"/>
       <rgbColor rgb="FFEEEEEE"/>
-      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -3861,6 +3915,10 @@
       <c r="I59" s="4"/>
       <c r="J59" s="4"/>
       <c r="K59" s="4"/>
+      <c r="L59" s="4"/>
+      <c r="M59" s="4"/>
+      <c r="N59" s="4"/>
+      <c r="O59" s="4"/>
     </row>
     <row r="60" customFormat="false" ht="14.4" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="n">
@@ -3873,18 +3931,22 @@
       </c>
       <c r="E60" s="5"/>
       <c r="F60" s="5"/>
-      <c r="H60" s="5" t="s">
+      <c r="H60" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="I60" s="5" t="s">
+      <c r="I60" s="18"/>
+      <c r="J60" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="J60" s="5" t="s">
+      <c r="K60" s="18"/>
+      <c r="L60" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="K60" s="5" t="s">
+      <c r="M60" s="18"/>
+      <c r="N60" s="21" t="s">
         <v>165</v>
       </c>
+      <c r="O60" s="18"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="9" t="n">
@@ -3897,71 +3959,74 @@
       </c>
       <c r="E61" s="5"/>
       <c r="F61" s="5"/>
-      <c r="H61" s="5" t="s">
+      <c r="H61" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="I61" s="5" t="s">
+      <c r="I61" s="22"/>
+      <c r="J61" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="J61" s="5" t="s">
+      <c r="K61" s="23"/>
+      <c r="L61" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="K61" s="17" t="s">
+      <c r="M61" s="24"/>
+      <c r="N61" s="21" t="s">
         <v>49</v>
       </c>
+      <c r="O61" s="25"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B62" s="18"/>
+      <c r="B62" s="26"/>
       <c r="C62" s="9"/>
       <c r="D62" s="5" t="s">
         <v>163</v>
       </c>
       <c r="E62" s="5"/>
       <c r="F62" s="5"/>
-      <c r="H62" s="19"/>
-      <c r="I62" s="19"/>
-      <c r="J62" s="19"/>
-      <c r="K62" s="19"/>
+      <c r="O62" s="27" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B63" s="18"/>
-      <c r="C63" s="18"/>
+      <c r="B63" s="26"/>
+      <c r="C63" s="26"/>
       <c r="D63" s="5" t="s">
         <v>167</v>
       </c>
       <c r="E63" s="5"/>
       <c r="F63" s="5"/>
-      <c r="H63" s="19"/>
-      <c r="I63" s="20"/>
-      <c r="J63" s="20"/>
-      <c r="K63" s="19"/>
+      <c r="H63" s="28"/>
+      <c r="I63" s="29"/>
+      <c r="J63" s="29"/>
+      <c r="K63" s="28"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B64" s="21"/>
+      <c r="B64" s="30"/>
       <c r="C64" s="9"/>
       <c r="D64" s="5" t="s">
         <v>164</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
-      <c r="I64" s="20"/>
-      <c r="J64" s="20"/>
+      <c r="I64" s="29"/>
+      <c r="J64" s="29"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B65" s="21"/>
-      <c r="C65" s="21"/>
+      <c r="B65" s="30"/>
+      <c r="C65" s="30"/>
       <c r="D65" s="5" t="s">
         <v>49</v>
       </c>
@@ -3972,7 +4037,7 @@
       <c r="A66" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B66" s="22"/>
+      <c r="B66" s="31"/>
       <c r="C66" s="9"/>
       <c r="D66" s="5" t="s">
         <v>165</v>
@@ -3984,8 +4049,8 @@
       <c r="A67" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B67" s="22"/>
-      <c r="C67" s="22"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="31"/>
       <c r="D67" s="5" t="s">
         <v>49</v>
       </c>
@@ -4105,7 +4170,7 @@
         <v>1</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
@@ -4133,7 +4198,7 @@
         <v>103</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O72" s="5"/>
       <c r="P72" s="5"/>
@@ -4366,7 +4431,7 @@
         <v>1</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>103</v>
@@ -4410,7 +4475,7 @@
       <c r="V79" s="5"/>
       <c r="W79" s="5"/>
       <c r="X79" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="Y79" s="5"/>
       <c r="Z79" s="5" t="s">
@@ -4615,7 +4680,7 @@
     <mergeCell ref="A57:U57"/>
     <mergeCell ref="A58:U58"/>
     <mergeCell ref="D59:F59"/>
-    <mergeCell ref="H59:K59"/>
+    <mergeCell ref="H59:O59"/>
     <mergeCell ref="D60:F60"/>
     <mergeCell ref="D61:F61"/>
     <mergeCell ref="D62:F62"/>
@@ -4687,334 +4752,334 @@
   <dimension ref="A1:W18"/>
   <sheetFormatPr defaultColWidth="6.48828125" defaultRowHeight="36" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="19" width="6.49"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="28" width="6.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="23"/>
-      <c r="B1" s="23"/>
-      <c r="C1" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
+      <c r="A1" s="32"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
-      <c r="Q2" s="26"/>
-      <c r="R2" s="26"/>
-      <c r="S2" s="26"/>
-      <c r="T2" s="26"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="27"/>
-      <c r="W2" s="28"/>
+      <c r="A2" s="32"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="35"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
+      <c r="Q2" s="35"/>
+      <c r="R2" s="35"/>
+      <c r="S2" s="35"/>
+      <c r="T2" s="35"/>
+      <c r="U2" s="35"/>
+      <c r="V2" s="36"/>
+      <c r="W2" s="37"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23"/>
-      <c r="C3" s="29"/>
-      <c r="L3" s="30" t="s">
-        <v>172</v>
-      </c>
-      <c r="V3" s="23"/>
-      <c r="W3" s="31"/>
+      <c r="A3" s="32"/>
+      <c r="C3" s="38"/>
+      <c r="L3" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="V3" s="32"/>
+      <c r="W3" s="40"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23"/>
-      <c r="C4" s="29"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="32" t="s">
+      <c r="A4" s="32"/>
+      <c r="C4" s="38"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="33"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="33"/>
-      <c r="P4" s="33"/>
-      <c r="Q4" s="34"/>
-      <c r="V4" s="23"/>
-      <c r="W4" s="31"/>
+      <c r="M4" s="42"/>
+      <c r="N4" s="42"/>
+      <c r="O4" s="42"/>
+      <c r="P4" s="42"/>
+      <c r="Q4" s="43"/>
+      <c r="V4" s="32"/>
+      <c r="W4" s="40"/>
     </row>
     <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23"/>
-      <c r="C5" s="29"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="35" t="s">
-        <v>173</v>
-      </c>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="37"/>
-      <c r="S5" s="23"/>
-      <c r="U5" s="38"/>
-      <c r="V5" s="39" t="s">
+      <c r="A5" s="32"/>
+      <c r="C5" s="38"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="45"/>
+      <c r="Q5" s="46"/>
+      <c r="S5" s="32"/>
+      <c r="U5" s="47"/>
+      <c r="V5" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="W5" s="31"/>
+      <c r="W5" s="40"/>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23"/>
-      <c r="C6" s="29"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-      <c r="P6" s="41"/>
-      <c r="Q6" s="42" t="s">
+      <c r="A6" s="32"/>
+      <c r="C6" s="38"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="50"/>
+      <c r="N6" s="50"/>
+      <c r="O6" s="50"/>
+      <c r="P6" s="50"/>
+      <c r="Q6" s="51" t="s">
         <v>49</v>
       </c>
-      <c r="S6" s="23"/>
-      <c r="U6" s="43"/>
-      <c r="V6" s="39"/>
-      <c r="W6" s="31"/>
+      <c r="S6" s="32"/>
+      <c r="U6" s="52"/>
+      <c r="V6" s="48"/>
+      <c r="W6" s="40"/>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23"/>
-      <c r="C7" s="29"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="L7" s="44" t="s">
-        <v>174</v>
-      </c>
-      <c r="M7" s="44"/>
-      <c r="N7" s="44"/>
-      <c r="V7" s="23"/>
-      <c r="W7" s="31"/>
+      <c r="A7" s="32"/>
+      <c r="C7" s="38"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="L7" s="53" t="s">
+        <v>175</v>
+      </c>
+      <c r="M7" s="53"/>
+      <c r="N7" s="53"/>
+      <c r="V7" s="32"/>
+      <c r="W7" s="40"/>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23"/>
-      <c r="C8" s="29"/>
-      <c r="G8" s="44" t="s">
-        <v>175</v>
-      </c>
-      <c r="H8" s="44"/>
-      <c r="I8" s="44"/>
-      <c r="L8" s="45" t="s">
+      <c r="A8" s="32"/>
+      <c r="C8" s="38"/>
+      <c r="G8" s="53" t="s">
+        <v>176</v>
+      </c>
+      <c r="H8" s="53"/>
+      <c r="I8" s="53"/>
+      <c r="L8" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="M8" s="46"/>
-      <c r="N8" s="47"/>
-      <c r="V8" s="23"/>
-      <c r="W8" s="31"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="56"/>
+      <c r="V8" s="32"/>
+      <c r="W8" s="40"/>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23"/>
-      <c r="C9" s="29"/>
-      <c r="G9" s="48"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="50" t="s">
-        <v>176</v>
-      </c>
-      <c r="L9" s="51"/>
-      <c r="M9" s="52"/>
-      <c r="N9" s="53" t="s">
+      <c r="A9" s="32"/>
+      <c r="C9" s="38"/>
+      <c r="G9" s="57"/>
+      <c r="H9" s="58"/>
+      <c r="I9" s="59" t="s">
         <v>177</v>
       </c>
-      <c r="V9" s="23"/>
-      <c r="W9" s="31"/>
+      <c r="L9" s="60"/>
+      <c r="M9" s="61"/>
+      <c r="N9" s="62" t="s">
+        <v>178</v>
+      </c>
+      <c r="V9" s="32"/>
+      <c r="W9" s="40"/>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23"/>
-      <c r="C10" s="29"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="56"/>
-      <c r="L10" s="44" t="s">
+      <c r="A10" s="32"/>
+      <c r="C10" s="38"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="64"/>
+      <c r="I10" s="65"/>
+      <c r="L10" s="53" t="s">
+        <v>179</v>
+      </c>
+      <c r="M10" s="53"/>
+      <c r="N10" s="53"/>
+      <c r="V10" s="32"/>
+      <c r="W10" s="40"/>
+    </row>
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="32"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="66" t="s">
+        <v>180</v>
+      </c>
+      <c r="E11" s="67"/>
+      <c r="G11" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="H11" s="64"/>
+      <c r="I11" s="65" t="s">
+        <v>182</v>
+      </c>
+      <c r="L11" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="M11" s="55"/>
+      <c r="N11" s="56"/>
+      <c r="V11" s="32"/>
+      <c r="W11" s="40"/>
+    </row>
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="66"/>
+      <c r="E12" s="68"/>
+      <c r="G12" s="63" t="s">
+        <v>183</v>
+      </c>
+      <c r="H12" s="64"/>
+      <c r="I12" s="65" t="s">
+        <v>184</v>
+      </c>
+      <c r="L12" s="60"/>
+      <c r="M12" s="61"/>
+      <c r="N12" s="62" t="s">
         <v>178</v>
       </c>
-      <c r="M10" s="44"/>
-      <c r="N10" s="44"/>
-      <c r="V10" s="23"/>
-      <c r="W10" s="31"/>
-    </row>
-    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="57" t="s">
-        <v>179</v>
-      </c>
-      <c r="E11" s="58"/>
-      <c r="G11" s="54" t="s">
-        <v>180</v>
-      </c>
-      <c r="H11" s="55"/>
-      <c r="I11" s="56" t="s">
-        <v>181</v>
-      </c>
-      <c r="L11" s="45" t="s">
+      <c r="V12" s="32"/>
+      <c r="W12" s="40"/>
+    </row>
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="32"/>
+      <c r="C13" s="38"/>
+      <c r="G13" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="M11" s="46"/>
-      <c r="N11" s="47"/>
-      <c r="V11" s="23"/>
-      <c r="W11" s="31"/>
-    </row>
-    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="57"/>
-      <c r="E12" s="59"/>
-      <c r="G12" s="54" t="s">
-        <v>182</v>
-      </c>
-      <c r="H12" s="55"/>
-      <c r="I12" s="56" t="s">
-        <v>183</v>
-      </c>
-      <c r="L12" s="51"/>
-      <c r="M12" s="52"/>
-      <c r="N12" s="53" t="s">
-        <v>177</v>
-      </c>
-      <c r="V12" s="23"/>
-      <c r="W12" s="31"/>
-    </row>
-    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23"/>
-      <c r="C13" s="29"/>
-      <c r="G13" s="54" t="s">
+      <c r="H13" s="64"/>
+      <c r="I13" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="55"/>
-      <c r="I13" s="56" t="s">
+      <c r="L13" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="M13" s="53"/>
+      <c r="N13" s="53"/>
+      <c r="S13" s="69"/>
+      <c r="T13" s="70"/>
+      <c r="U13" s="71"/>
+      <c r="V13" s="72" t="s">
+        <v>186</v>
+      </c>
+      <c r="W13" s="40"/>
+    </row>
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32"/>
+      <c r="C14" s="38"/>
+      <c r="G14" s="73" t="s">
+        <v>187</v>
+      </c>
+      <c r="H14" s="74"/>
+      <c r="I14" s="75"/>
+      <c r="L14" s="54"/>
+      <c r="M14" s="56" t="s">
+        <v>178</v>
+      </c>
+      <c r="S14" s="69"/>
+      <c r="T14" s="70"/>
+      <c r="U14" s="71"/>
+      <c r="V14" s="72" t="s">
+        <v>188</v>
+      </c>
+      <c r="W14" s="40"/>
+    </row>
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32"/>
+      <c r="C15" s="38"/>
+      <c r="L15" s="76"/>
+      <c r="M15" s="77"/>
+      <c r="S15" s="69"/>
+      <c r="T15" s="70"/>
+      <c r="U15" s="71"/>
+      <c r="V15" s="72" t="s">
+        <v>189</v>
+      </c>
+      <c r="W15" s="40"/>
+    </row>
+    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32"/>
+      <c r="C16" s="38"/>
+      <c r="E16" s="78"/>
+      <c r="F16" s="71"/>
+      <c r="L16" s="60" t="s">
         <v>49</v>
       </c>
-      <c r="L13" s="44" t="s">
-        <v>184</v>
-      </c>
-      <c r="M13" s="44"/>
-      <c r="N13" s="44"/>
-      <c r="S13" s="60"/>
-      <c r="T13" s="61"/>
-      <c r="U13" s="62"/>
-      <c r="V13" s="63" t="s">
-        <v>185</v>
-      </c>
-      <c r="W13" s="31"/>
-    </row>
-    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23"/>
-      <c r="C14" s="29"/>
-      <c r="G14" s="64" t="s">
-        <v>186</v>
-      </c>
-      <c r="H14" s="65"/>
-      <c r="I14" s="66"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="47" t="s">
-        <v>177</v>
-      </c>
-      <c r="S14" s="60"/>
-      <c r="T14" s="61"/>
-      <c r="U14" s="62"/>
-      <c r="V14" s="63" t="s">
-        <v>187</v>
-      </c>
-      <c r="W14" s="31"/>
-    </row>
-    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23"/>
-      <c r="C15" s="29"/>
-      <c r="L15" s="67"/>
-      <c r="M15" s="68"/>
-      <c r="S15" s="60"/>
-      <c r="T15" s="61"/>
-      <c r="U15" s="62"/>
-      <c r="V15" s="63" t="s">
-        <v>188</v>
-      </c>
-      <c r="W15" s="31"/>
-    </row>
-    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23"/>
-      <c r="C16" s="29"/>
-      <c r="E16" s="69"/>
-      <c r="F16" s="62"/>
-      <c r="L16" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="M16" s="53"/>
-      <c r="P16" s="69"/>
-      <c r="Q16" s="62"/>
-      <c r="S16" s="60"/>
-      <c r="T16" s="61"/>
-      <c r="U16" s="62"/>
-      <c r="V16" s="63" t="s">
-        <v>189</v>
-      </c>
-      <c r="W16" s="31"/>
+      <c r="M16" s="62"/>
+      <c r="P16" s="78"/>
+      <c r="Q16" s="71"/>
+      <c r="S16" s="69"/>
+      <c r="T16" s="70"/>
+      <c r="U16" s="71"/>
+      <c r="V16" s="72" t="s">
+        <v>190</v>
+      </c>
+      <c r="W16" s="40"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="70"/>
-      <c r="E17" s="71" t="s">
-        <v>190</v>
-      </c>
-      <c r="F17" s="71"/>
-      <c r="P17" s="71" t="s">
+      <c r="C17" s="79"/>
+      <c r="E17" s="80" t="s">
         <v>191</v>
       </c>
-      <c r="Q17" s="71"/>
-      <c r="V17" s="23"/>
-      <c r="W17" s="31"/>
+      <c r="F17" s="80"/>
+      <c r="P17" s="80" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q17" s="80"/>
+      <c r="V17" s="32"/>
+      <c r="W17" s="40"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="72"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="73"/>
-      <c r="F18" s="73"/>
-      <c r="G18" s="73"/>
-      <c r="H18" s="73"/>
-      <c r="I18" s="73"/>
-      <c r="J18" s="73"/>
-      <c r="K18" s="73"/>
-      <c r="L18" s="73"/>
-      <c r="M18" s="73"/>
-      <c r="N18" s="73"/>
-      <c r="O18" s="73"/>
-      <c r="P18" s="73"/>
-      <c r="Q18" s="73"/>
-      <c r="R18" s="73"/>
-      <c r="S18" s="73"/>
-      <c r="T18" s="73"/>
-      <c r="U18" s="73"/>
-      <c r="V18" s="73"/>
-      <c r="W18" s="74"/>
+      <c r="C18" s="81"/>
+      <c r="D18" s="82"/>
+      <c r="E18" s="82"/>
+      <c r="F18" s="82"/>
+      <c r="G18" s="82"/>
+      <c r="H18" s="82"/>
+      <c r="I18" s="82"/>
+      <c r="J18" s="82"/>
+      <c r="K18" s="82"/>
+      <c r="L18" s="82"/>
+      <c r="M18" s="82"/>
+      <c r="N18" s="82"/>
+      <c r="O18" s="82"/>
+      <c r="P18" s="82"/>
+      <c r="Q18" s="82"/>
+      <c r="R18" s="82"/>
+      <c r="S18" s="82"/>
+      <c r="T18" s="82"/>
+      <c r="U18" s="82"/>
+      <c r="V18" s="82"/>
+      <c r="W18" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
[ Version 0.0.30.14 ] - drainage vent schematic and Excel diagram were updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="198">
   <si>
     <t xml:space="preserve">MAIN</t>
   </si>
@@ -540,28 +540,43 @@
     <t xml:space="preserve">ROULETTE R1 ENABLE </t>
   </si>
   <si>
+    <t xml:space="preserve">6V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENT 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRAINAGE VENT DRIVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENT 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CD4069UBE (NOT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOTOR DRIVER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">!SLP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VDD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MHB4012 (NAND)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ROULETTE DRIVER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESP32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CD4069UBE (NOT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR DRIVER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">!SLP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VDD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MHB4012 (NAND)</t>
   </si>
   <si>
     <t xml:space="preserve">MOTOR</t>
@@ -610,7 +625,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="18">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -698,6 +713,46 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="28"/>
+      <color rgb="FFFF9800"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="28"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="28"/>
+      <color rgb="FF4CAF50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="28"/>
+      <color rgb="FF2196F3"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="28"/>
+      <color rgb="FF795548"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="18">
     <fill>
@@ -780,8 +835,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEEEEEE"/>
-        <bgColor rgb="FFF5F5F5"/>
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF003300"/>
       </patternFill>
     </fill>
     <fill>
@@ -792,8 +847,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF000000"/>
-        <bgColor rgb="FF003300"/>
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFF5F5F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -935,7 +990,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="95">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1068,51 +1123,143 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1120,34 +1267,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1200,15 +1319,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="15" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1216,11 +1331,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1245,18 +1356,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="17" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="16" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4749,7 +4848,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:AH39"/>
   <sheetFormatPr defaultColWidth="6.48828125" defaultRowHeight="36" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="28" width="6.49"/>
@@ -4757,341 +4856,882 @@
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="32"/>
-      <c r="B1" s="32"/>
-      <c r="C1" s="33" t="s">
-        <v>172</v>
-      </c>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
-      <c r="R1" s="32"/>
-      <c r="S1" s="32"/>
+      <c r="B1" s="0"/>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+      <c r="I1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="L1" s="0"/>
+      <c r="M1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
+      <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+      <c r="T1" s="0"/>
+      <c r="U1" s="0"/>
+      <c r="V1" s="0"/>
+      <c r="W1" s="0"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
-      <c r="S2" s="35"/>
-      <c r="T2" s="35"/>
-      <c r="U2" s="35"/>
-      <c r="V2" s="36"/>
-      <c r="W2" s="37"/>
+      <c r="B2" s="0"/>
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0"/>
+      <c r="J2" s="0"/>
+      <c r="K2" s="0"/>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0"/>
+      <c r="N2" s="0"/>
+      <c r="O2" s="0"/>
+      <c r="P2" s="0"/>
+      <c r="Q2" s="0"/>
+      <c r="R2" s="0"/>
+      <c r="S2" s="0"/>
+      <c r="T2" s="0"/>
+      <c r="U2" s="0"/>
+      <c r="V2" s="0"/>
+      <c r="W2" s="0"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32"/>
-      <c r="C3" s="38"/>
-      <c r="L3" s="39" t="s">
-        <v>173</v>
-      </c>
-      <c r="V3" s="32"/>
-      <c r="W3" s="40"/>
+      <c r="B3" s="0"/>
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
+      <c r="K3" s="0"/>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0"/>
+      <c r="N3" s="0"/>
+      <c r="O3" s="0"/>
+      <c r="P3" s="0"/>
+      <c r="Q3" s="0"/>
+      <c r="R3" s="0"/>
+      <c r="S3" s="0"/>
+      <c r="T3" s="0"/>
+      <c r="U3" s="0"/>
+      <c r="V3" s="0"/>
+      <c r="W3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32"/>
-      <c r="C4" s="38"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="41" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4" s="42"/>
-      <c r="N4" s="42"/>
-      <c r="O4" s="42"/>
-      <c r="P4" s="42"/>
-      <c r="Q4" s="43"/>
-      <c r="V4" s="32"/>
-      <c r="W4" s="40"/>
+      <c r="B4" s="0"/>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
+      <c r="O4" s="0"/>
+      <c r="P4" s="0"/>
+      <c r="Q4" s="0"/>
+      <c r="R4" s="0"/>
+      <c r="S4" s="0"/>
+      <c r="T4" s="0"/>
+      <c r="U4" s="0"/>
+      <c r="V4" s="0"/>
+      <c r="W4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32"/>
-      <c r="C5" s="38"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
-      <c r="K5" s="32"/>
-      <c r="L5" s="44" t="s">
-        <v>174</v>
-      </c>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="46"/>
-      <c r="S5" s="32"/>
-      <c r="U5" s="47"/>
-      <c r="V5" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="W5" s="40"/>
+      <c r="B5" s="0"/>
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0"/>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0"/>
+      <c r="N5" s="0"/>
+      <c r="O5" s="0"/>
+      <c r="P5" s="0"/>
+      <c r="Q5" s="0"/>
+      <c r="R5" s="0"/>
+      <c r="S5" s="0"/>
+      <c r="T5" s="0"/>
+      <c r="U5" s="0"/>
+      <c r="V5" s="0"/>
+      <c r="W5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32"/>
-      <c r="C6" s="38"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="49"/>
-      <c r="M6" s="50"/>
-      <c r="N6" s="50"/>
-      <c r="O6" s="50"/>
-      <c r="P6" s="50"/>
-      <c r="Q6" s="51" t="s">
-        <v>49</v>
-      </c>
-      <c r="S6" s="32"/>
-      <c r="U6" s="52"/>
-      <c r="V6" s="48"/>
-      <c r="W6" s="40"/>
+      <c r="B6" s="0"/>
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="K6" s="0"/>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0"/>
+      <c r="N6" s="0"/>
+      <c r="O6" s="0"/>
+      <c r="P6" s="0"/>
+      <c r="Q6" s="0"/>
+      <c r="R6" s="0"/>
+      <c r="S6" s="0"/>
+      <c r="T6" s="0"/>
+      <c r="U6" s="0"/>
+      <c r="V6" s="0"/>
+      <c r="W6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32"/>
-      <c r="C7" s="38"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="L7" s="53" t="s">
-        <v>175</v>
-      </c>
-      <c r="M7" s="53"/>
-      <c r="N7" s="53"/>
-      <c r="V7" s="32"/>
-      <c r="W7" s="40"/>
+      <c r="B7" s="0"/>
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+      <c r="K7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="0"/>
+      <c r="P7" s="0"/>
+      <c r="Q7" s="0"/>
+      <c r="R7" s="0"/>
+      <c r="S7" s="0"/>
+      <c r="T7" s="0"/>
+      <c r="U7" s="0"/>
+      <c r="V7" s="0"/>
+      <c r="W7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32"/>
-      <c r="C8" s="38"/>
-      <c r="G8" s="53" t="s">
-        <v>176</v>
-      </c>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="L8" s="54" t="s">
-        <v>49</v>
-      </c>
-      <c r="M8" s="55"/>
-      <c r="N8" s="56"/>
-      <c r="V8" s="32"/>
-      <c r="W8" s="40"/>
+      <c r="B8" s="0"/>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+      <c r="K8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+      <c r="Q8" s="0"/>
+      <c r="R8" s="0"/>
+      <c r="S8" s="0"/>
+      <c r="T8" s="0"/>
+      <c r="U8" s="0"/>
+      <c r="V8" s="0"/>
+      <c r="W8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32"/>
-      <c r="C9" s="38"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="58"/>
-      <c r="I9" s="59" t="s">
-        <v>177</v>
-      </c>
-      <c r="L9" s="60"/>
-      <c r="M9" s="61"/>
-      <c r="N9" s="62" t="s">
-        <v>178</v>
-      </c>
-      <c r="V9" s="32"/>
-      <c r="W9" s="40"/>
+      <c r="B9" s="0"/>
+      <c r="C9" s="0"/>
+      <c r="D9" s="0"/>
+      <c r="E9" s="0"/>
+      <c r="F9" s="0"/>
+      <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
+      <c r="I9" s="0"/>
+      <c r="J9" s="0"/>
+      <c r="K9" s="0"/>
+      <c r="L9" s="0"/>
+      <c r="M9" s="0"/>
+      <c r="N9" s="0"/>
+      <c r="O9" s="0"/>
+      <c r="P9" s="0"/>
+      <c r="Q9" s="0"/>
+      <c r="R9" s="0"/>
+      <c r="S9" s="0"/>
+      <c r="T9" s="0"/>
+      <c r="U9" s="0"/>
+      <c r="V9" s="0"/>
+      <c r="W9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32"/>
-      <c r="C10" s="38"/>
-      <c r="G10" s="63"/>
-      <c r="H10" s="64"/>
-      <c r="I10" s="65"/>
-      <c r="L10" s="53" t="s">
-        <v>179</v>
-      </c>
-      <c r="M10" s="53"/>
-      <c r="N10" s="53"/>
-      <c r="V10" s="32"/>
-      <c r="W10" s="40"/>
+      <c r="B10" s="0"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="34"/>
+      <c r="U10" s="34"/>
+      <c r="V10" s="34"/>
+      <c r="W10" s="35"/>
     </row>
     <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="66" t="s">
-        <v>180</v>
-      </c>
-      <c r="E11" s="67"/>
-      <c r="G11" s="63" t="s">
-        <v>181</v>
-      </c>
-      <c r="H11" s="64"/>
-      <c r="I11" s="65" t="s">
-        <v>182</v>
-      </c>
-      <c r="L11" s="54" t="s">
-        <v>49</v>
-      </c>
-      <c r="M11" s="55"/>
-      <c r="N11" s="56"/>
-      <c r="V11" s="32"/>
-      <c r="W11" s="40"/>
+      <c r="B11" s="0"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="0"/>
+      <c r="E11" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="F11" s="37"/>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
+      <c r="I11" s="0"/>
+      <c r="J11" s="0"/>
+      <c r="K11" s="0"/>
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="0"/>
+      <c r="P11" s="0"/>
+      <c r="Q11" s="0"/>
+      <c r="R11" s="0"/>
+      <c r="S11" s="0"/>
+      <c r="T11" s="0"/>
+      <c r="U11" s="0"/>
+      <c r="V11" s="0"/>
+      <c r="W11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="66"/>
-      <c r="E12" s="68"/>
-      <c r="G12" s="63" t="s">
-        <v>183</v>
-      </c>
-      <c r="H12" s="64"/>
-      <c r="I12" s="65" t="s">
-        <v>184</v>
-      </c>
-      <c r="L12" s="60"/>
-      <c r="M12" s="61"/>
-      <c r="N12" s="62" t="s">
-        <v>178</v>
-      </c>
-      <c r="V12" s="32"/>
-      <c r="W12" s="40"/>
+      <c r="B12" s="0"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="0"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="40"/>
+      <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
+      <c r="I12" s="0"/>
+      <c r="J12" s="0"/>
+      <c r="K12" s="0"/>
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="0"/>
+      <c r="P12" s="0"/>
+      <c r="Q12" s="0"/>
+      <c r="R12" s="0"/>
+      <c r="S12" s="0"/>
+      <c r="T12" s="0"/>
+      <c r="U12" s="0"/>
+      <c r="V12" s="0"/>
+      <c r="W12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32"/>
-      <c r="C13" s="38"/>
-      <c r="G13" s="63" t="s">
-        <v>49</v>
-      </c>
-      <c r="H13" s="64"/>
-      <c r="I13" s="65" t="s">
-        <v>49</v>
-      </c>
-      <c r="L13" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="M13" s="53"/>
-      <c r="N13" s="53"/>
-      <c r="S13" s="69"/>
-      <c r="T13" s="70"/>
-      <c r="U13" s="71"/>
-      <c r="V13" s="72" t="s">
-        <v>186</v>
-      </c>
-      <c r="W13" s="40"/>
+      <c r="B13" s="0"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="0"/>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
+      <c r="K13" s="0"/>
+      <c r="L13" s="0"/>
+      <c r="M13" s="0"/>
+      <c r="N13" s="0"/>
+      <c r="O13" s="0"/>
+      <c r="P13" s="0"/>
+      <c r="Q13" s="0"/>
+      <c r="R13" s="0"/>
+      <c r="S13" s="0"/>
+      <c r="T13" s="0"/>
+      <c r="U13" s="0"/>
+      <c r="V13" s="0"/>
+      <c r="W13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32"/>
-      <c r="C14" s="38"/>
-      <c r="G14" s="73" t="s">
-        <v>187</v>
-      </c>
-      <c r="H14" s="74"/>
-      <c r="I14" s="75"/>
-      <c r="L14" s="54"/>
-      <c r="M14" s="56" t="s">
-        <v>178</v>
-      </c>
-      <c r="S14" s="69"/>
-      <c r="T14" s="70"/>
-      <c r="U14" s="71"/>
-      <c r="V14" s="72" t="s">
-        <v>188</v>
-      </c>
-      <c r="W14" s="40"/>
+      <c r="B14" s="0"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="41" t="s">
+        <v>173</v>
+      </c>
+      <c r="E14" s="42" t="s">
+        <v>174</v>
+      </c>
+      <c r="F14" s="43" t="s">
+        <v>174</v>
+      </c>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
+      <c r="K14" s="0"/>
+      <c r="L14" s="0"/>
+      <c r="M14" s="0"/>
+      <c r="N14" s="0"/>
+      <c r="O14" s="0"/>
+      <c r="P14" s="0"/>
+      <c r="Q14" s="0"/>
+      <c r="R14" s="0"/>
+      <c r="S14" s="0"/>
+      <c r="T14" s="0"/>
+      <c r="U14" s="0"/>
+      <c r="V14" s="0"/>
+      <c r="W14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32"/>
-      <c r="C15" s="38"/>
-      <c r="L15" s="76"/>
-      <c r="M15" s="77"/>
-      <c r="S15" s="69"/>
-      <c r="T15" s="70"/>
-      <c r="U15" s="71"/>
-      <c r="V15" s="72" t="s">
-        <v>189</v>
-      </c>
-      <c r="W15" s="40"/>
+      <c r="B15" s="0"/>
+      <c r="C15" s="36"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" s="45" t="s">
+        <v>174</v>
+      </c>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="K15" s="0"/>
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="0"/>
+      <c r="P15" s="0"/>
+      <c r="Q15" s="0"/>
+      <c r="R15" s="0"/>
+      <c r="S15" s="0"/>
+      <c r="T15" s="0"/>
+      <c r="U15" s="0"/>
+      <c r="V15" s="0"/>
+      <c r="W15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32"/>
-      <c r="C16" s="38"/>
-      <c r="E16" s="78"/>
-      <c r="F16" s="71"/>
-      <c r="L16" s="60" t="s">
+      <c r="B16" s="0"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="46" t="s">
+        <v>174</v>
+      </c>
+      <c r="F16" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="K16" s="0"/>
+      <c r="L16" s="0"/>
+      <c r="M16" s="0"/>
+      <c r="N16" s="0"/>
+      <c r="O16" s="0"/>
+      <c r="P16" s="0"/>
+      <c r="Q16" s="0"/>
+      <c r="R16" s="48" t="s">
+        <v>175</v>
+      </c>
+      <c r="S16" s="48"/>
+      <c r="T16" s="48"/>
+      <c r="U16" s="48"/>
+      <c r="V16" s="0"/>
+      <c r="W16" s="38"/>
+    </row>
+    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0"/>
+      <c r="C17" s="36"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="49" t="s">
+        <v>174</v>
+      </c>
+      <c r="F17" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
+      <c r="J17" s="0"/>
+      <c r="K17" s="0"/>
+      <c r="L17" s="0"/>
+      <c r="M17" s="0"/>
+      <c r="N17" s="0"/>
+      <c r="O17" s="0"/>
+      <c r="P17" s="0"/>
+      <c r="Q17" s="0"/>
+      <c r="R17" s="0"/>
+      <c r="S17" s="0"/>
+      <c r="T17" s="0"/>
+      <c r="U17" s="0"/>
+      <c r="V17" s="0"/>
+      <c r="W17" s="38"/>
+    </row>
+    <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0"/>
+      <c r="C18" s="36"/>
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
+      <c r="J18" s="0"/>
+      <c r="K18" s="0"/>
+      <c r="L18" s="0"/>
+      <c r="M18" s="0"/>
+      <c r="N18" s="0"/>
+      <c r="O18" s="0"/>
+      <c r="P18" s="0"/>
+      <c r="Q18" s="0"/>
+      <c r="R18" s="0"/>
+      <c r="S18" s="0"/>
+      <c r="T18" s="0"/>
+      <c r="U18" s="0"/>
+      <c r="V18" s="0"/>
+      <c r="W18" s="38"/>
+    </row>
+    <row r="19" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="0"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="41" t="s">
+        <v>176</v>
+      </c>
+      <c r="E19" s="49" t="s">
+        <v>174</v>
+      </c>
+      <c r="F19" s="50" t="s">
+        <v>174</v>
+      </c>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
+      <c r="K19" s="0"/>
+      <c r="L19" s="0"/>
+      <c r="M19" s="0"/>
+      <c r="N19" s="0"/>
+      <c r="O19" s="0"/>
+      <c r="P19" s="0"/>
+      <c r="Q19" s="0"/>
+      <c r="R19" s="0"/>
+      <c r="S19" s="0"/>
+      <c r="T19" s="0"/>
+      <c r="U19" s="0"/>
+      <c r="V19" s="0"/>
+      <c r="W19" s="38"/>
+    </row>
+    <row r="20" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="51"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="46" t="s">
+        <v>174</v>
+      </c>
+      <c r="F20" s="47" t="s">
+        <v>174</v>
+      </c>
+      <c r="W20" s="52"/>
+    </row>
+    <row r="21" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="32"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="44" t="s">
+        <v>174</v>
+      </c>
+      <c r="F21" s="45" t="s">
+        <v>174</v>
+      </c>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="32"/>
+      <c r="N21" s="32"/>
+      <c r="O21" s="32"/>
+      <c r="P21" s="32"/>
+      <c r="Q21" s="32"/>
+      <c r="R21" s="32"/>
+      <c r="S21" s="32"/>
+      <c r="U21" s="53"/>
+      <c r="V21" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="W21" s="52"/>
+      <c r="X21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C22" s="55"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="42" t="s">
+        <v>174</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>174</v>
+      </c>
+      <c r="G22" s="56"/>
+      <c r="H22" s="56"/>
+      <c r="I22" s="56"/>
+      <c r="J22" s="56"/>
+      <c r="K22" s="56"/>
+      <c r="L22" s="56"/>
+      <c r="M22" s="56"/>
+      <c r="N22" s="56"/>
+      <c r="O22" s="56"/>
+      <c r="P22" s="56"/>
+      <c r="Q22" s="56"/>
+      <c r="R22" s="56"/>
+      <c r="S22" s="56"/>
+      <c r="T22" s="56"/>
+      <c r="U22" s="57"/>
+      <c r="V22" s="54"/>
+      <c r="W22" s="52"/>
+      <c r="X22" s="0"/>
+    </row>
+    <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C23" s="55"/>
+      <c r="L23" s="58" t="s">
+        <v>177</v>
+      </c>
+      <c r="U23" s="0"/>
+      <c r="V23" s="0"/>
+      <c r="W23" s="52"/>
+      <c r="X23" s="0"/>
+    </row>
+    <row r="24" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C24" s="55"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+      <c r="L24" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="M24" s="60"/>
+      <c r="N24" s="60"/>
+      <c r="O24" s="60"/>
+      <c r="P24" s="60"/>
+      <c r="Q24" s="61"/>
+      <c r="V24" s="32"/>
+      <c r="W24" s="52"/>
+      <c r="X24" s="0"/>
+    </row>
+    <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C25" s="55"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="62" t="s">
+        <v>178</v>
+      </c>
+      <c r="M25" s="63"/>
+      <c r="N25" s="63"/>
+      <c r="O25" s="63"/>
+      <c r="P25" s="63"/>
+      <c r="Q25" s="64"/>
+      <c r="S25" s="32"/>
+      <c r="U25" s="53"/>
+      <c r="V25" s="54" t="s">
+        <v>44</v>
+      </c>
+      <c r="W25" s="52"/>
+      <c r="X25" s="0"/>
+    </row>
+    <row r="26" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C26" s="55"/>
+      <c r="I26" s="32"/>
+      <c r="J26" s="32"/>
+      <c r="K26" s="32"/>
+      <c r="L26" s="65"/>
+      <c r="M26" s="66"/>
+      <c r="N26" s="66"/>
+      <c r="O26" s="66"/>
+      <c r="P26" s="66"/>
+      <c r="Q26" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="M16" s="62"/>
-      <c r="P16" s="78"/>
-      <c r="Q16" s="71"/>
-      <c r="S16" s="69"/>
-      <c r="T16" s="70"/>
-      <c r="U16" s="71"/>
-      <c r="V16" s="72" t="s">
+      <c r="S26" s="32"/>
+      <c r="U26" s="68"/>
+      <c r="V26" s="54"/>
+      <c r="W26" s="52"/>
+      <c r="X26" s="0"/>
+    </row>
+    <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C27" s="55"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="L27" s="69" t="s">
+        <v>179</v>
+      </c>
+      <c r="M27" s="69"/>
+      <c r="N27" s="69"/>
+      <c r="V27" s="32"/>
+      <c r="W27" s="52"/>
+      <c r="X27" s="0"/>
+    </row>
+    <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="55"/>
+      <c r="G28" s="69" t="s">
+        <v>180</v>
+      </c>
+      <c r="H28" s="69"/>
+      <c r="I28" s="69"/>
+      <c r="L28" s="70" t="s">
+        <v>49</v>
+      </c>
+      <c r="M28" s="71"/>
+      <c r="N28" s="72"/>
+      <c r="V28" s="32"/>
+      <c r="W28" s="52"/>
+      <c r="X28" s="0"/>
+      <c r="AF28" s="0"/>
+      <c r="AG28" s="0"/>
+      <c r="AH28" s="0"/>
+    </row>
+    <row r="29" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C29" s="55"/>
+      <c r="G29" s="73"/>
+      <c r="H29" s="74"/>
+      <c r="I29" s="75" t="s">
+        <v>181</v>
+      </c>
+      <c r="L29" s="76"/>
+      <c r="M29" s="77"/>
+      <c r="N29" s="78" t="s">
+        <v>182</v>
+      </c>
+      <c r="V29" s="32"/>
+      <c r="W29" s="52"/>
+      <c r="X29" s="0"/>
+    </row>
+    <row r="30" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C30" s="55"/>
+      <c r="G30" s="79"/>
+      <c r="H30" s="80"/>
+      <c r="I30" s="81"/>
+      <c r="L30" s="69" t="s">
+        <v>183</v>
+      </c>
+      <c r="M30" s="69"/>
+      <c r="N30" s="69"/>
+      <c r="R30" s="48" t="s">
+        <v>184</v>
+      </c>
+      <c r="S30" s="48"/>
+      <c r="T30" s="48"/>
+      <c r="V30" s="32"/>
+      <c r="W30" s="52"/>
+      <c r="X30" s="0"/>
+    </row>
+    <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C31" s="55"/>
+      <c r="D31" s="41" t="s">
+        <v>185</v>
+      </c>
+      <c r="E31" s="82"/>
+      <c r="G31" s="79" t="s">
+        <v>186</v>
+      </c>
+      <c r="H31" s="80"/>
+      <c r="I31" s="81" t="s">
+        <v>187</v>
+      </c>
+      <c r="L31" s="70" t="s">
+        <v>49</v>
+      </c>
+      <c r="M31" s="71"/>
+      <c r="N31" s="72"/>
+      <c r="V31" s="32"/>
+      <c r="W31" s="52"/>
+      <c r="X31" s="0"/>
+    </row>
+    <row r="32" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="55"/>
+      <c r="D32" s="41"/>
+      <c r="E32" s="83"/>
+      <c r="G32" s="79" t="s">
+        <v>188</v>
+      </c>
+      <c r="H32" s="80"/>
+      <c r="I32" s="81" t="s">
+        <v>189</v>
+      </c>
+      <c r="L32" s="76"/>
+      <c r="M32" s="77"/>
+      <c r="N32" s="78" t="s">
+        <v>182</v>
+      </c>
+      <c r="V32" s="32"/>
+      <c r="W32" s="52"/>
+      <c r="X32" s="0"/>
+    </row>
+    <row r="33" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="55"/>
+      <c r="G33" s="79" t="s">
+        <v>49</v>
+      </c>
+      <c r="H33" s="80"/>
+      <c r="I33" s="81" t="s">
+        <v>49</v>
+      </c>
+      <c r="L33" s="69" t="s">
         <v>190</v>
       </c>
-      <c r="W16" s="40"/>
-    </row>
-    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="79"/>
-      <c r="E17" s="80" t="s">
+      <c r="M33" s="69"/>
+      <c r="N33" s="69"/>
+      <c r="S33" s="84"/>
+      <c r="T33" s="85"/>
+      <c r="U33" s="40"/>
+      <c r="V33" s="86" t="s">
         <v>191</v>
       </c>
-      <c r="F17" s="80"/>
-      <c r="P17" s="80" t="s">
+      <c r="W33" s="52"/>
+      <c r="X33" s="0"/>
+    </row>
+    <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C34" s="55"/>
+      <c r="G34" s="87" t="s">
         <v>192</v>
       </c>
-      <c r="Q17" s="80"/>
-      <c r="V17" s="32"/>
-      <c r="W17" s="40"/>
-    </row>
-    <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="81"/>
-      <c r="D18" s="82"/>
-      <c r="E18" s="82"/>
-      <c r="F18" s="82"/>
-      <c r="G18" s="82"/>
-      <c r="H18" s="82"/>
-      <c r="I18" s="82"/>
-      <c r="J18" s="82"/>
-      <c r="K18" s="82"/>
-      <c r="L18" s="82"/>
-      <c r="M18" s="82"/>
-      <c r="N18" s="82"/>
-      <c r="O18" s="82"/>
-      <c r="P18" s="82"/>
-      <c r="Q18" s="82"/>
-      <c r="R18" s="82"/>
-      <c r="S18" s="82"/>
-      <c r="T18" s="82"/>
-      <c r="U18" s="82"/>
-      <c r="V18" s="82"/>
-      <c r="W18" s="83"/>
+      <c r="H34" s="88"/>
+      <c r="I34" s="89"/>
+      <c r="L34" s="70"/>
+      <c r="M34" s="72" t="s">
+        <v>182</v>
+      </c>
+      <c r="S34" s="84"/>
+      <c r="T34" s="85"/>
+      <c r="U34" s="40"/>
+      <c r="V34" s="86" t="s">
+        <v>193</v>
+      </c>
+      <c r="W34" s="52"/>
+      <c r="X34" s="0"/>
+    </row>
+    <row r="35" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C35" s="55"/>
+      <c r="L35" s="90"/>
+      <c r="M35" s="91"/>
+      <c r="S35" s="84"/>
+      <c r="T35" s="85"/>
+      <c r="U35" s="40"/>
+      <c r="V35" s="86" t="s">
+        <v>194</v>
+      </c>
+      <c r="W35" s="52"/>
+      <c r="X35" s="0"/>
+    </row>
+    <row r="36" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C36" s="55"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="40"/>
+      <c r="L36" s="76" t="s">
+        <v>49</v>
+      </c>
+      <c r="M36" s="78"/>
+      <c r="P36" s="39"/>
+      <c r="Q36" s="40"/>
+      <c r="S36" s="84"/>
+      <c r="T36" s="85"/>
+      <c r="U36" s="40"/>
+      <c r="V36" s="86" t="s">
+        <v>195</v>
+      </c>
+      <c r="W36" s="52"/>
+      <c r="X36" s="0"/>
+    </row>
+    <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C37" s="51"/>
+      <c r="E37" s="37" t="s">
+        <v>196</v>
+      </c>
+      <c r="F37" s="37"/>
+      <c r="P37" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q37" s="37"/>
+      <c r="V37" s="32"/>
+      <c r="W37" s="52"/>
+      <c r="X37" s="0"/>
+    </row>
+    <row r="38" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C38" s="92"/>
+      <c r="D38" s="93"/>
+      <c r="E38" s="93"/>
+      <c r="F38" s="93"/>
+      <c r="G38" s="93"/>
+      <c r="H38" s="93"/>
+      <c r="I38" s="93"/>
+      <c r="J38" s="93"/>
+      <c r="K38" s="93"/>
+      <c r="L38" s="93"/>
+      <c r="M38" s="93"/>
+      <c r="N38" s="93"/>
+      <c r="O38" s="93"/>
+      <c r="P38" s="93"/>
+      <c r="Q38" s="93"/>
+      <c r="R38" s="93"/>
+      <c r="S38" s="93"/>
+      <c r="T38" s="93"/>
+      <c r="U38" s="93"/>
+      <c r="V38" s="93"/>
+      <c r="W38" s="94"/>
+      <c r="X38" s="0"/>
+    </row>
+    <row r="39" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="X39" s="0"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="V5:V6"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="L13:N13"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="P17:Q17"/>
+  <mergeCells count="14">
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="R16:U16"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="V21:V22"/>
+    <mergeCell ref="V25:V26"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="G28:I28"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="R30:T30"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="P37:Q37"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
[ Version 0.0.30.18 ] - schematics were updated.
</commit_message>
<xml_diff>
--- a/docs/smartflowerpot_tech_db.xlsx
+++ b/docs/smartflowerpot_tech_db.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="1" state="visible" r:id="rId3"/>
@@ -764,7 +764,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC80"/>
-        <bgColor rgb="FFFFCDD2"/>
+        <bgColor rgb="FFFDD835"/>
       </patternFill>
     </fill>
     <fill>
@@ -806,7 +806,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF9800"/>
-        <bgColor rgb="FFFFCC00"/>
+        <bgColor rgb="FFFB8C00"/>
       </patternFill>
     </fill>
     <fill>
@@ -842,7 +842,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF44336"/>
-        <bgColor rgb="FFFF8080"/>
+        <bgColor rgb="FF993366"/>
       </patternFill>
     </fill>
     <fill>
@@ -990,7 +990,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="94">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1123,19 +1123,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1143,7 +1143,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1159,27 +1159,27 @@
       <alignment horizontal="center" vertical="center" textRotation="180" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1187,11 +1187,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1209,10 +1209,6 @@
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1400,10 +1396,10 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF5F5F5"/>
+      <rgbColor rgb="FFFFF9C4"/>
       <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFF44336"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFE1BEE7"/>
       <rgbColor rgb="FF000080"/>
@@ -1415,7 +1411,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF5F5F5"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFCDD2"/>
       <rgbColor rgb="FFA5D6A7"/>
@@ -1425,9 +1421,9 @@
       <rgbColor rgb="FF2196F3"/>
       <rgbColor rgb="FF29B6F6"/>
       <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFDD835"/>
       <rgbColor rgb="FFFF9800"/>
-      <rgbColor rgb="FFF44336"/>
+      <rgbColor rgb="FFFB8C00"/>
       <rgbColor rgb="FF795548"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
@@ -1552,6 +1548,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <tabColor rgb="FFFB8C00"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U21"/>
@@ -2234,6 +2231,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <tabColor rgb="FFFDD835"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC80"/>
@@ -4846,6 +4844,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
+    <tabColor rgb="FFFFF9C4"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AH39"/>
@@ -4856,232 +4855,232 @@
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="32"/>
-      <c r="B1" s="0"/>
-      <c r="C1" s="0"/>
-      <c r="D1" s="0"/>
-      <c r="E1" s="0"/>
-      <c r="F1" s="0"/>
-      <c r="G1" s="0"/>
-      <c r="H1" s="0"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
-      <c r="K1" s="0"/>
-      <c r="L1" s="0"/>
-      <c r="M1" s="0"/>
-      <c r="N1" s="0"/>
-      <c r="O1" s="0"/>
-      <c r="P1" s="0"/>
-      <c r="Q1" s="0"/>
-      <c r="R1" s="0"/>
-      <c r="S1" s="0"/>
-      <c r="T1" s="0"/>
-      <c r="U1" s="0"/>
-      <c r="V1" s="0"/>
-      <c r="W1" s="0"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+      <c r="O1" s="32"/>
+      <c r="P1" s="32"/>
+      <c r="Q1" s="32"/>
+      <c r="R1" s="32"/>
+      <c r="S1" s="32"/>
+      <c r="T1" s="32"/>
+      <c r="U1" s="32"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32"/>
-      <c r="B2" s="0"/>
-      <c r="C2" s="0"/>
-      <c r="D2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
-      <c r="G2" s="0"/>
-      <c r="H2" s="0"/>
-      <c r="I2" s="0"/>
-      <c r="J2" s="0"/>
-      <c r="K2" s="0"/>
-      <c r="L2" s="0"/>
-      <c r="M2" s="0"/>
-      <c r="N2" s="0"/>
-      <c r="O2" s="0"/>
-      <c r="P2" s="0"/>
-      <c r="Q2" s="0"/>
-      <c r="R2" s="0"/>
-      <c r="S2" s="0"/>
-      <c r="T2" s="0"/>
-      <c r="U2" s="0"/>
-      <c r="V2" s="0"/>
-      <c r="W2" s="0"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="32"/>
+      <c r="Q2" s="32"/>
+      <c r="R2" s="32"/>
+      <c r="S2" s="32"/>
+      <c r="T2" s="32"/>
+      <c r="U2" s="32"/>
+      <c r="V2" s="32"/>
+      <c r="W2" s="32"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="32"/>
-      <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0"/>
-      <c r="K3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
-      <c r="N3" s="0"/>
-      <c r="O3" s="0"/>
-      <c r="P3" s="0"/>
-      <c r="Q3" s="0"/>
-      <c r="R3" s="0"/>
-      <c r="S3" s="0"/>
-      <c r="T3" s="0"/>
-      <c r="U3" s="0"/>
-      <c r="V3" s="0"/>
-      <c r="W3" s="0"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
+      <c r="L3" s="32"/>
+      <c r="M3" s="32"/>
+      <c r="N3" s="32"/>
+      <c r="O3" s="32"/>
+      <c r="P3" s="32"/>
+      <c r="Q3" s="32"/>
+      <c r="R3" s="32"/>
+      <c r="S3" s="32"/>
+      <c r="T3" s="32"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="32"/>
+      <c r="W3" s="32"/>
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="32"/>
-      <c r="B4" s="0"/>
-      <c r="C4" s="0"/>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
-      <c r="K4" s="0"/>
-      <c r="L4" s="0"/>
-      <c r="M4" s="0"/>
-      <c r="N4" s="0"/>
-      <c r="O4" s="0"/>
-      <c r="P4" s="0"/>
-      <c r="Q4" s="0"/>
-      <c r="R4" s="0"/>
-      <c r="S4" s="0"/>
-      <c r="T4" s="0"/>
-      <c r="U4" s="0"/>
-      <c r="V4" s="0"/>
-      <c r="W4" s="0"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
+      <c r="K4" s="32"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="32"/>
+      <c r="N4" s="32"/>
+      <c r="O4" s="32"/>
+      <c r="P4" s="32"/>
+      <c r="Q4" s="32"/>
+      <c r="R4" s="32"/>
+      <c r="S4" s="32"/>
+      <c r="T4" s="32"/>
+      <c r="U4" s="32"/>
+      <c r="V4" s="32"/>
+      <c r="W4" s="32"/>
     </row>
     <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32"/>
-      <c r="B5" s="0"/>
-      <c r="C5" s="0"/>
-      <c r="D5" s="0"/>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="K5" s="0"/>
-      <c r="L5" s="0"/>
-      <c r="M5" s="0"/>
-      <c r="N5" s="0"/>
-      <c r="O5" s="0"/>
-      <c r="P5" s="0"/>
-      <c r="Q5" s="0"/>
-      <c r="R5" s="0"/>
-      <c r="S5" s="0"/>
-      <c r="T5" s="0"/>
-      <c r="U5" s="0"/>
-      <c r="V5" s="0"/>
-      <c r="W5" s="0"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="32"/>
+      <c r="N5" s="32"/>
+      <c r="O5" s="32"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="32"/>
+      <c r="R5" s="32"/>
+      <c r="S5" s="32"/>
+      <c r="T5" s="32"/>
+      <c r="U5" s="32"/>
+      <c r="V5" s="32"/>
+      <c r="W5" s="32"/>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="32"/>
-      <c r="B6" s="0"/>
-      <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
-      <c r="E6" s="0"/>
-      <c r="F6" s="0"/>
-      <c r="G6" s="0"/>
-      <c r="H6" s="0"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="0"/>
-      <c r="M6" s="0"/>
-      <c r="N6" s="0"/>
-      <c r="O6" s="0"/>
-      <c r="P6" s="0"/>
-      <c r="Q6" s="0"/>
-      <c r="R6" s="0"/>
-      <c r="S6" s="0"/>
-      <c r="T6" s="0"/>
-      <c r="U6" s="0"/>
-      <c r="V6" s="0"/>
-      <c r="W6" s="0"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32"/>
+      <c r="R6" s="32"/>
+      <c r="S6" s="32"/>
+      <c r="T6" s="32"/>
+      <c r="U6" s="32"/>
+      <c r="V6" s="32"/>
+      <c r="W6" s="32"/>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="32"/>
-      <c r="B7" s="0"/>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
-      <c r="E7" s="0"/>
-      <c r="F7" s="0"/>
-      <c r="G7" s="0"/>
-      <c r="H7" s="0"/>
-      <c r="I7" s="0"/>
-      <c r="J7" s="0"/>
-      <c r="K7" s="0"/>
-      <c r="L7" s="0"/>
-      <c r="M7" s="0"/>
-      <c r="N7" s="0"/>
-      <c r="O7" s="0"/>
-      <c r="P7" s="0"/>
-      <c r="Q7" s="0"/>
-      <c r="R7" s="0"/>
-      <c r="S7" s="0"/>
-      <c r="T7" s="0"/>
-      <c r="U7" s="0"/>
-      <c r="V7" s="0"/>
-      <c r="W7" s="0"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="32"/>
+      <c r="P7" s="32"/>
+      <c r="Q7" s="32"/>
+      <c r="R7" s="32"/>
+      <c r="S7" s="32"/>
+      <c r="T7" s="32"/>
+      <c r="U7" s="32"/>
+      <c r="V7" s="32"/>
+      <c r="W7" s="32"/>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="32"/>
-      <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
-      <c r="F8" s="0"/>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0"/>
-      <c r="K8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="0"/>
-      <c r="O8" s="0"/>
-      <c r="P8" s="0"/>
-      <c r="Q8" s="0"/>
-      <c r="R8" s="0"/>
-      <c r="S8" s="0"/>
-      <c r="T8" s="0"/>
-      <c r="U8" s="0"/>
-      <c r="V8" s="0"/>
-      <c r="W8" s="0"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="32"/>
+      <c r="N8" s="32"/>
+      <c r="O8" s="32"/>
+      <c r="P8" s="32"/>
+      <c r="Q8" s="32"/>
+      <c r="R8" s="32"/>
+      <c r="S8" s="32"/>
+      <c r="T8" s="32"/>
+      <c r="U8" s="32"/>
+      <c r="V8" s="32"/>
+      <c r="W8" s="32"/>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="32"/>
-      <c r="B9" s="0"/>
-      <c r="C9" s="0"/>
-      <c r="D9" s="0"/>
-      <c r="E9" s="0"/>
-      <c r="F9" s="0"/>
-      <c r="G9" s="0"/>
-      <c r="H9" s="0"/>
-      <c r="I9" s="0"/>
-      <c r="J9" s="0"/>
-      <c r="K9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
-      <c r="N9" s="0"/>
-      <c r="O9" s="0"/>
-      <c r="P9" s="0"/>
-      <c r="Q9" s="0"/>
-      <c r="R9" s="0"/>
-      <c r="S9" s="0"/>
-      <c r="T9" s="0"/>
-      <c r="U9" s="0"/>
-      <c r="V9" s="0"/>
-      <c r="W9" s="0"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="32"/>
+      <c r="K9" s="32"/>
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="32"/>
+      <c r="P9" s="32"/>
+      <c r="Q9" s="32"/>
+      <c r="R9" s="32"/>
+      <c r="S9" s="32"/>
+      <c r="T9" s="32"/>
+      <c r="U9" s="32"/>
+      <c r="V9" s="32"/>
+      <c r="W9" s="32"/>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32"/>
-      <c r="B10" s="0"/>
+      <c r="B10" s="32"/>
       <c r="C10" s="33"/>
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
@@ -5106,84 +5105,84 @@
     </row>
     <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="32"/>
-      <c r="B11" s="0"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="36"/>
-      <c r="D11" s="0"/>
+      <c r="D11" s="32"/>
       <c r="E11" s="37" t="s">
         <v>172</v>
       </c>
       <c r="F11" s="37"/>
-      <c r="G11" s="0"/>
-      <c r="H11" s="0"/>
-      <c r="I11" s="0"/>
-      <c r="J11" s="0"/>
-      <c r="K11" s="0"/>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="0"/>
-      <c r="O11" s="0"/>
-      <c r="P11" s="0"/>
-      <c r="Q11" s="0"/>
-      <c r="R11" s="0"/>
-      <c r="S11" s="0"/>
-      <c r="T11" s="0"/>
-      <c r="U11" s="0"/>
-      <c r="V11" s="0"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="32"/>
+      <c r="K11" s="32"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="32"/>
+      <c r="N11" s="32"/>
+      <c r="O11" s="32"/>
+      <c r="P11" s="32"/>
+      <c r="Q11" s="32"/>
+      <c r="R11" s="32"/>
+      <c r="S11" s="32"/>
+      <c r="T11" s="32"/>
+      <c r="U11" s="32"/>
+      <c r="V11" s="32"/>
       <c r="W11" s="38"/>
     </row>
     <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="32"/>
-      <c r="B12" s="0"/>
+      <c r="B12" s="32"/>
       <c r="C12" s="36"/>
-      <c r="D12" s="0"/>
+      <c r="D12" s="32"/>
       <c r="E12" s="39"/>
       <c r="F12" s="40"/>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
-      <c r="I12" s="0"/>
-      <c r="J12" s="0"/>
-      <c r="K12" s="0"/>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="0"/>
-      <c r="O12" s="0"/>
-      <c r="P12" s="0"/>
-      <c r="Q12" s="0"/>
-      <c r="R12" s="0"/>
-      <c r="S12" s="0"/>
-      <c r="T12" s="0"/>
-      <c r="U12" s="0"/>
-      <c r="V12" s="0"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="32"/>
+      <c r="N12" s="32"/>
+      <c r="O12" s="32"/>
+      <c r="P12" s="32"/>
+      <c r="Q12" s="32"/>
+      <c r="R12" s="32"/>
+      <c r="S12" s="32"/>
+      <c r="T12" s="32"/>
+      <c r="U12" s="32"/>
+      <c r="V12" s="32"/>
       <c r="W12" s="38"/>
     </row>
     <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32"/>
-      <c r="B13" s="0"/>
+      <c r="B13" s="32"/>
       <c r="C13" s="36"/>
-      <c r="D13" s="0"/>
-      <c r="E13" s="0"/>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="K13" s="0"/>
-      <c r="L13" s="0"/>
-      <c r="M13" s="0"/>
-      <c r="N13" s="0"/>
-      <c r="O13" s="0"/>
-      <c r="P13" s="0"/>
-      <c r="Q13" s="0"/>
-      <c r="R13" s="0"/>
-      <c r="S13" s="0"/>
-      <c r="T13" s="0"/>
-      <c r="U13" s="0"/>
-      <c r="V13" s="0"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
+      <c r="T13" s="32"/>
+      <c r="U13" s="32"/>
+      <c r="V13" s="32"/>
       <c r="W13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="32"/>
-      <c r="B14" s="0"/>
+      <c r="B14" s="32"/>
       <c r="C14" s="36"/>
       <c r="D14" s="41" t="s">
         <v>173</v>
@@ -5194,27 +5193,27 @@
       <c r="F14" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="K14" s="0"/>
-      <c r="L14" s="0"/>
-      <c r="M14" s="0"/>
-      <c r="N14" s="0"/>
-      <c r="O14" s="0"/>
-      <c r="P14" s="0"/>
-      <c r="Q14" s="0"/>
-      <c r="R14" s="0"/>
-      <c r="S14" s="0"/>
-      <c r="T14" s="0"/>
-      <c r="U14" s="0"/>
-      <c r="V14" s="0"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="32"/>
+      <c r="K14" s="32"/>
+      <c r="L14" s="32"/>
+      <c r="M14" s="32"/>
+      <c r="N14" s="32"/>
+      <c r="O14" s="32"/>
+      <c r="P14" s="32"/>
+      <c r="Q14" s="32"/>
+      <c r="R14" s="32"/>
+      <c r="S14" s="32"/>
+      <c r="T14" s="32"/>
+      <c r="U14" s="32"/>
+      <c r="V14" s="32"/>
       <c r="W14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="32"/>
-      <c r="B15" s="0"/>
+      <c r="B15" s="32"/>
       <c r="C15" s="36"/>
       <c r="D15" s="41"/>
       <c r="E15" s="44" t="s">
@@ -5223,27 +5222,27 @@
       <c r="F15" s="45" t="s">
         <v>174</v>
       </c>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="K15" s="0"/>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="0"/>
-      <c r="O15" s="0"/>
-      <c r="P15" s="0"/>
-      <c r="Q15" s="0"/>
-      <c r="R15" s="0"/>
-      <c r="S15" s="0"/>
-      <c r="T15" s="0"/>
-      <c r="U15" s="0"/>
-      <c r="V15" s="0"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="32"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="32"/>
+      <c r="N15" s="32"/>
+      <c r="O15" s="32"/>
+      <c r="P15" s="32"/>
+      <c r="Q15" s="32"/>
+      <c r="R15" s="32"/>
+      <c r="S15" s="32"/>
+      <c r="T15" s="32"/>
+      <c r="U15" s="32"/>
+      <c r="V15" s="32"/>
       <c r="W15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="32"/>
-      <c r="B16" s="0"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="36"/>
       <c r="D16" s="41"/>
       <c r="E16" s="46" t="s">
@@ -5252,28 +5251,28 @@
       <c r="F16" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0"/>
-      <c r="K16" s="0"/>
-      <c r="L16" s="0"/>
-      <c r="M16" s="0"/>
-      <c r="N16" s="0"/>
-      <c r="O16" s="0"/>
-      <c r="P16" s="0"/>
-      <c r="Q16" s="0"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="32"/>
+      <c r="M16" s="32"/>
+      <c r="N16" s="32"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="32"/>
+      <c r="Q16" s="32"/>
       <c r="R16" s="48" t="s">
         <v>175</v>
       </c>
       <c r="S16" s="48"/>
       <c r="T16" s="48"/>
       <c r="U16" s="48"/>
-      <c r="V16" s="0"/>
+      <c r="V16" s="32"/>
       <c r="W16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="0"/>
+      <c r="B17" s="32"/>
       <c r="C17" s="36"/>
       <c r="D17" s="41"/>
       <c r="E17" s="49" t="s">
@@ -5282,50 +5281,50 @@
       <c r="F17" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
-      <c r="I17" s="0"/>
-      <c r="J17" s="0"/>
-      <c r="K17" s="0"/>
-      <c r="L17" s="0"/>
-      <c r="M17" s="0"/>
-      <c r="N17" s="0"/>
-      <c r="O17" s="0"/>
-      <c r="P17" s="0"/>
-      <c r="Q17" s="0"/>
-      <c r="R17" s="0"/>
-      <c r="S17" s="0"/>
-      <c r="T17" s="0"/>
-      <c r="U17" s="0"/>
-      <c r="V17" s="0"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="32"/>
+      <c r="N17" s="32"/>
+      <c r="O17" s="32"/>
+      <c r="P17" s="32"/>
+      <c r="Q17" s="32"/>
+      <c r="R17" s="32"/>
+      <c r="S17" s="32"/>
+      <c r="T17" s="32"/>
+      <c r="U17" s="32"/>
+      <c r="V17" s="32"/>
       <c r="W17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0"/>
+      <c r="B18" s="32"/>
       <c r="C18" s="36"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
-      <c r="J18" s="0"/>
-      <c r="K18" s="0"/>
-      <c r="L18" s="0"/>
-      <c r="M18" s="0"/>
-      <c r="N18" s="0"/>
-      <c r="O18" s="0"/>
-      <c r="P18" s="0"/>
-      <c r="Q18" s="0"/>
-      <c r="R18" s="0"/>
-      <c r="S18" s="0"/>
-      <c r="T18" s="0"/>
-      <c r="U18" s="0"/>
-      <c r="V18" s="0"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="32"/>
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="32"/>
+      <c r="L18" s="32"/>
+      <c r="M18" s="32"/>
+      <c r="N18" s="32"/>
+      <c r="O18" s="32"/>
+      <c r="P18" s="32"/>
+      <c r="Q18" s="32"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
       <c r="W18" s="38"/>
     </row>
     <row r="19" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0"/>
+      <c r="B19" s="32"/>
       <c r="C19" s="36"/>
       <c r="D19" s="41" t="s">
         <v>176</v>
@@ -5336,22 +5335,22 @@
       <c r="F19" s="50" t="s">
         <v>174</v>
       </c>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
-      <c r="J19" s="0"/>
-      <c r="K19" s="0"/>
-      <c r="L19" s="0"/>
-      <c r="M19" s="0"/>
-      <c r="N19" s="0"/>
-      <c r="O19" s="0"/>
-      <c r="P19" s="0"/>
-      <c r="Q19" s="0"/>
-      <c r="R19" s="0"/>
-      <c r="S19" s="0"/>
-      <c r="T19" s="0"/>
-      <c r="U19" s="0"/>
-      <c r="V19" s="0"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
+      <c r="N19" s="32"/>
+      <c r="O19" s="32"/>
+      <c r="P19" s="32"/>
+      <c r="Q19" s="32"/>
+      <c r="R19" s="32"/>
+      <c r="S19" s="32"/>
+      <c r="T19" s="32"/>
+      <c r="U19" s="32"/>
+      <c r="V19" s="32"/>
       <c r="W19" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5393,10 +5392,10 @@
         <v>47</v>
       </c>
       <c r="W21" s="52"/>
-      <c r="X21" s="0"/>
+      <c r="X21" s="32"/>
     </row>
     <row r="22" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="55"/>
+      <c r="C22" s="36"/>
       <c r="D22" s="41"/>
       <c r="E22" s="42" t="s">
         <v>174</v>
@@ -5404,151 +5403,151 @@
       <c r="F22" s="43" t="s">
         <v>174</v>
       </c>
-      <c r="G22" s="56"/>
-      <c r="H22" s="56"/>
-      <c r="I22" s="56"/>
-      <c r="J22" s="56"/>
-      <c r="K22" s="56"/>
-      <c r="L22" s="56"/>
-      <c r="M22" s="56"/>
-      <c r="N22" s="56"/>
-      <c r="O22" s="56"/>
-      <c r="P22" s="56"/>
-      <c r="Q22" s="56"/>
-      <c r="R22" s="56"/>
-      <c r="S22" s="56"/>
-      <c r="T22" s="56"/>
-      <c r="U22" s="57"/>
+      <c r="G22" s="55"/>
+      <c r="H22" s="55"/>
+      <c r="I22" s="55"/>
+      <c r="J22" s="55"/>
+      <c r="K22" s="55"/>
+      <c r="L22" s="55"/>
+      <c r="M22" s="55"/>
+      <c r="N22" s="55"/>
+      <c r="O22" s="55"/>
+      <c r="P22" s="55"/>
+      <c r="Q22" s="55"/>
+      <c r="R22" s="55"/>
+      <c r="S22" s="55"/>
+      <c r="T22" s="55"/>
+      <c r="U22" s="56"/>
       <c r="V22" s="54"/>
       <c r="W22" s="52"/>
-      <c r="X22" s="0"/>
+      <c r="X22" s="32"/>
     </row>
     <row r="23" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="55"/>
-      <c r="L23" s="58" t="s">
+      <c r="C23" s="36"/>
+      <c r="L23" s="57" t="s">
         <v>177</v>
       </c>
-      <c r="U23" s="0"/>
-      <c r="V23" s="0"/>
+      <c r="U23" s="32"/>
+      <c r="V23" s="32"/>
       <c r="W23" s="52"/>
-      <c r="X23" s="0"/>
+      <c r="X23" s="32"/>
     </row>
     <row r="24" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C24" s="55"/>
+      <c r="C24" s="36"/>
       <c r="I24" s="32"/>
       <c r="J24" s="32"/>
       <c r="K24" s="32"/>
-      <c r="L24" s="59" t="s">
+      <c r="L24" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="M24" s="60"/>
-      <c r="N24" s="60"/>
-      <c r="O24" s="60"/>
-      <c r="P24" s="60"/>
-      <c r="Q24" s="61"/>
+      <c r="M24" s="59"/>
+      <c r="N24" s="59"/>
+      <c r="O24" s="59"/>
+      <c r="P24" s="59"/>
+      <c r="Q24" s="60"/>
       <c r="V24" s="32"/>
       <c r="W24" s="52"/>
-      <c r="X24" s="0"/>
+      <c r="X24" s="32"/>
     </row>
     <row r="25" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="55"/>
+      <c r="C25" s="36"/>
       <c r="I25" s="32"/>
       <c r="J25" s="32"/>
       <c r="K25" s="32"/>
-      <c r="L25" s="62" t="s">
+      <c r="L25" s="61" t="s">
         <v>178</v>
       </c>
-      <c r="M25" s="63"/>
-      <c r="N25" s="63"/>
-      <c r="O25" s="63"/>
-      <c r="P25" s="63"/>
-      <c r="Q25" s="64"/>
+      <c r="M25" s="62"/>
+      <c r="N25" s="62"/>
+      <c r="O25" s="62"/>
+      <c r="P25" s="62"/>
+      <c r="Q25" s="63"/>
       <c r="S25" s="32"/>
       <c r="U25" s="53"/>
       <c r="V25" s="54" t="s">
         <v>44</v>
       </c>
       <c r="W25" s="52"/>
-      <c r="X25" s="0"/>
+      <c r="X25" s="32"/>
     </row>
     <row r="26" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="55"/>
+      <c r="C26" s="36"/>
       <c r="I26" s="32"/>
       <c r="J26" s="32"/>
       <c r="K26" s="32"/>
-      <c r="L26" s="65"/>
-      <c r="M26" s="66"/>
-      <c r="N26" s="66"/>
-      <c r="O26" s="66"/>
-      <c r="P26" s="66"/>
-      <c r="Q26" s="67" t="s">
+      <c r="L26" s="64"/>
+      <c r="M26" s="65"/>
+      <c r="N26" s="65"/>
+      <c r="O26" s="65"/>
+      <c r="P26" s="65"/>
+      <c r="Q26" s="66" t="s">
         <v>49</v>
       </c>
       <c r="S26" s="32"/>
-      <c r="U26" s="68"/>
+      <c r="U26" s="67"/>
       <c r="V26" s="54"/>
       <c r="W26" s="52"/>
-      <c r="X26" s="0"/>
+      <c r="X26" s="32"/>
     </row>
     <row r="27" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="55"/>
+      <c r="C27" s="36"/>
       <c r="G27" s="32"/>
       <c r="H27" s="32"/>
       <c r="I27" s="32"/>
-      <c r="L27" s="69" t="s">
+      <c r="L27" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="M27" s="69"/>
-      <c r="N27" s="69"/>
+      <c r="M27" s="68"/>
+      <c r="N27" s="68"/>
       <c r="V27" s="32"/>
       <c r="W27" s="52"/>
-      <c r="X27" s="0"/>
+      <c r="X27" s="32"/>
     </row>
     <row r="28" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="55"/>
-      <c r="G28" s="69" t="s">
+      <c r="C28" s="36"/>
+      <c r="G28" s="68" t="s">
         <v>180</v>
       </c>
-      <c r="H28" s="69"/>
-      <c r="I28" s="69"/>
-      <c r="L28" s="70" t="s">
+      <c r="H28" s="68"/>
+      <c r="I28" s="68"/>
+      <c r="L28" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="M28" s="71"/>
-      <c r="N28" s="72"/>
+      <c r="M28" s="70"/>
+      <c r="N28" s="71"/>
       <c r="V28" s="32"/>
       <c r="W28" s="52"/>
-      <c r="X28" s="0"/>
-      <c r="AF28" s="0"/>
-      <c r="AG28" s="0"/>
-      <c r="AH28" s="0"/>
+      <c r="X28" s="32"/>
+      <c r="AF28" s="32"/>
+      <c r="AG28" s="32"/>
+      <c r="AH28" s="32"/>
     </row>
     <row r="29" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C29" s="55"/>
-      <c r="G29" s="73"/>
-      <c r="H29" s="74"/>
-      <c r="I29" s="75" t="s">
+      <c r="C29" s="36"/>
+      <c r="G29" s="72"/>
+      <c r="H29" s="73"/>
+      <c r="I29" s="74" t="s">
         <v>181</v>
       </c>
-      <c r="L29" s="76"/>
-      <c r="M29" s="77"/>
-      <c r="N29" s="78" t="s">
+      <c r="L29" s="75"/>
+      <c r="M29" s="76"/>
+      <c r="N29" s="77" t="s">
         <v>182</v>
       </c>
       <c r="V29" s="32"/>
       <c r="W29" s="52"/>
-      <c r="X29" s="0"/>
+      <c r="X29" s="32"/>
     </row>
     <row r="30" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="55"/>
-      <c r="G30" s="79"/>
-      <c r="H30" s="80"/>
-      <c r="I30" s="81"/>
-      <c r="L30" s="69" t="s">
+      <c r="C30" s="36"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="79"/>
+      <c r="I30" s="80"/>
+      <c r="L30" s="68" t="s">
         <v>183</v>
       </c>
-      <c r="M30" s="69"/>
-      <c r="N30" s="69"/>
+      <c r="M30" s="68"/>
+      <c r="N30" s="68"/>
       <c r="R30" s="48" t="s">
         <v>184</v>
       </c>
@@ -5556,124 +5555,124 @@
       <c r="T30" s="48"/>
       <c r="V30" s="32"/>
       <c r="W30" s="52"/>
-      <c r="X30" s="0"/>
+      <c r="X30" s="32"/>
     </row>
     <row r="31" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="55"/>
+      <c r="C31" s="36"/>
       <c r="D31" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="E31" s="82"/>
-      <c r="G31" s="79" t="s">
+      <c r="E31" s="81"/>
+      <c r="G31" s="78" t="s">
         <v>186</v>
       </c>
-      <c r="H31" s="80"/>
-      <c r="I31" s="81" t="s">
+      <c r="H31" s="79"/>
+      <c r="I31" s="80" t="s">
         <v>187</v>
       </c>
-      <c r="L31" s="70" t="s">
+      <c r="L31" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="M31" s="71"/>
-      <c r="N31" s="72"/>
+      <c r="M31" s="70"/>
+      <c r="N31" s="71"/>
       <c r="V31" s="32"/>
       <c r="W31" s="52"/>
-      <c r="X31" s="0"/>
+      <c r="X31" s="32"/>
     </row>
     <row r="32" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="55"/>
+      <c r="C32" s="36"/>
       <c r="D32" s="41"/>
-      <c r="E32" s="83"/>
-      <c r="G32" s="79" t="s">
+      <c r="E32" s="82"/>
+      <c r="G32" s="78" t="s">
         <v>188</v>
       </c>
-      <c r="H32" s="80"/>
-      <c r="I32" s="81" t="s">
+      <c r="H32" s="79"/>
+      <c r="I32" s="80" t="s">
         <v>189</v>
       </c>
-      <c r="L32" s="76"/>
-      <c r="M32" s="77"/>
-      <c r="N32" s="78" t="s">
+      <c r="L32" s="75"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="77" t="s">
         <v>182</v>
       </c>
       <c r="V32" s="32"/>
       <c r="W32" s="52"/>
-      <c r="X32" s="0"/>
+      <c r="X32" s="32"/>
     </row>
     <row r="33" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="55"/>
-      <c r="G33" s="79" t="s">
+      <c r="C33" s="36"/>
+      <c r="G33" s="78" t="s">
         <v>49</v>
       </c>
-      <c r="H33" s="80"/>
-      <c r="I33" s="81" t="s">
+      <c r="H33" s="79"/>
+      <c r="I33" s="80" t="s">
         <v>49</v>
       </c>
-      <c r="L33" s="69" t="s">
+      <c r="L33" s="68" t="s">
         <v>190</v>
       </c>
-      <c r="M33" s="69"/>
-      <c r="N33" s="69"/>
-      <c r="S33" s="84"/>
-      <c r="T33" s="85"/>
+      <c r="M33" s="68"/>
+      <c r="N33" s="68"/>
+      <c r="S33" s="83"/>
+      <c r="T33" s="84"/>
       <c r="U33" s="40"/>
-      <c r="V33" s="86" t="s">
+      <c r="V33" s="85" t="s">
         <v>191</v>
       </c>
       <c r="W33" s="52"/>
-      <c r="X33" s="0"/>
+      <c r="X33" s="32"/>
     </row>
     <row r="34" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="55"/>
-      <c r="G34" s="87" t="s">
+      <c r="C34" s="36"/>
+      <c r="G34" s="86" t="s">
         <v>192</v>
       </c>
-      <c r="H34" s="88"/>
-      <c r="I34" s="89"/>
-      <c r="L34" s="70"/>
-      <c r="M34" s="72" t="s">
+      <c r="H34" s="87"/>
+      <c r="I34" s="88"/>
+      <c r="L34" s="69"/>
+      <c r="M34" s="71" t="s">
         <v>182</v>
       </c>
-      <c r="S34" s="84"/>
-      <c r="T34" s="85"/>
+      <c r="S34" s="83"/>
+      <c r="T34" s="84"/>
       <c r="U34" s="40"/>
-      <c r="V34" s="86" t="s">
+      <c r="V34" s="85" t="s">
         <v>193</v>
       </c>
       <c r="W34" s="52"/>
-      <c r="X34" s="0"/>
+      <c r="X34" s="32"/>
     </row>
     <row r="35" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C35" s="55"/>
-      <c r="L35" s="90"/>
-      <c r="M35" s="91"/>
-      <c r="S35" s="84"/>
-      <c r="T35" s="85"/>
+      <c r="C35" s="36"/>
+      <c r="L35" s="89"/>
+      <c r="M35" s="90"/>
+      <c r="S35" s="83"/>
+      <c r="T35" s="84"/>
       <c r="U35" s="40"/>
-      <c r="V35" s="86" t="s">
+      <c r="V35" s="85" t="s">
         <v>194</v>
       </c>
       <c r="W35" s="52"/>
-      <c r="X35" s="0"/>
+      <c r="X35" s="32"/>
     </row>
     <row r="36" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="55"/>
+      <c r="C36" s="36"/>
       <c r="E36" s="39"/>
       <c r="F36" s="40"/>
-      <c r="L36" s="76" t="s">
+      <c r="L36" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="M36" s="78"/>
+      <c r="M36" s="77"/>
       <c r="P36" s="39"/>
       <c r="Q36" s="40"/>
-      <c r="S36" s="84"/>
-      <c r="T36" s="85"/>
+      <c r="S36" s="83"/>
+      <c r="T36" s="84"/>
       <c r="U36" s="40"/>
-      <c r="V36" s="86" t="s">
+      <c r="V36" s="85" t="s">
         <v>195</v>
       </c>
       <c r="W36" s="52"/>
-      <c r="X36" s="0"/>
+      <c r="X36" s="32"/>
     </row>
     <row r="37" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C37" s="51"/>
@@ -5687,34 +5686,34 @@
       <c r="Q37" s="37"/>
       <c r="V37" s="32"/>
       <c r="W37" s="52"/>
-      <c r="X37" s="0"/>
+      <c r="X37" s="32"/>
     </row>
     <row r="38" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="92"/>
-      <c r="D38" s="93"/>
-      <c r="E38" s="93"/>
-      <c r="F38" s="93"/>
-      <c r="G38" s="93"/>
-      <c r="H38" s="93"/>
-      <c r="I38" s="93"/>
-      <c r="J38" s="93"/>
-      <c r="K38" s="93"/>
-      <c r="L38" s="93"/>
-      <c r="M38" s="93"/>
-      <c r="N38" s="93"/>
-      <c r="O38" s="93"/>
-      <c r="P38" s="93"/>
-      <c r="Q38" s="93"/>
-      <c r="R38" s="93"/>
-      <c r="S38" s="93"/>
-      <c r="T38" s="93"/>
-      <c r="U38" s="93"/>
-      <c r="V38" s="93"/>
-      <c r="W38" s="94"/>
-      <c r="X38" s="0"/>
+      <c r="C38" s="91"/>
+      <c r="D38" s="92"/>
+      <c r="E38" s="92"/>
+      <c r="F38" s="92"/>
+      <c r="G38" s="92"/>
+      <c r="H38" s="92"/>
+      <c r="I38" s="92"/>
+      <c r="J38" s="92"/>
+      <c r="K38" s="92"/>
+      <c r="L38" s="92"/>
+      <c r="M38" s="92"/>
+      <c r="N38" s="92"/>
+      <c r="O38" s="92"/>
+      <c r="P38" s="92"/>
+      <c r="Q38" s="92"/>
+      <c r="R38" s="92"/>
+      <c r="S38" s="92"/>
+      <c r="T38" s="92"/>
+      <c r="U38" s="92"/>
+      <c r="V38" s="92"/>
+      <c r="W38" s="93"/>
+      <c r="X38" s="32"/>
     </row>
     <row r="39" customFormat="false" ht="36" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="X39" s="0"/>
+      <c r="X39" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>